<commit_message>
implementacion funcion si error
</commit_message>
<xml_diff>
--- a/examples/DB_Supermercado.xlsx
+++ b/examples/DB_Supermercado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EducacionIT\Documents\office\Excel\xls-mj15\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBFB6C6-6254-479A-9441-8A016063E92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF55D92-8FFC-40C6-98B9-EBAB1C7FC01B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7173,7 +7173,7 @@
         <v>3230017545</v>
       </c>
       <c r="AI14" s="95">
-        <f t="shared" ref="AI14:AN14" si="23">SUM(AI10:AI13)</f>
+        <f t="shared" ref="AI14:AM14" si="23">SUM(AI10:AI13)</f>
         <v>9072</v>
       </c>
       <c r="AJ14" s="51">
@@ -7332,23 +7332,23 @@
         <v>645115066</v>
       </c>
       <c r="E17" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,E$16)</f>
+        <f t="shared" ref="E17:I22" si="27">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,E$16)</f>
         <v>23075</v>
       </c>
       <c r="F17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,F$16)</f>
+        <f t="shared" si="27"/>
         <v>14026</v>
       </c>
       <c r="G17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,G$16)</f>
+        <f t="shared" si="27"/>
         <v>37242</v>
       </c>
       <c r="H17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,H$16)</f>
+        <f t="shared" si="27"/>
         <v>34352</v>
       </c>
       <c r="I17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,I$16)</f>
+        <f t="shared" si="27"/>
         <v>12970</v>
       </c>
       <c r="J17" s="17">
@@ -7356,23 +7356,23 @@
         <v>121665</v>
       </c>
       <c r="L17" s="97">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,L$16)</f>
+        <f t="shared" ref="L17:P22" si="28">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,L$16)</f>
         <v>109144041</v>
       </c>
       <c r="M17" s="59">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,M$16)</f>
+        <f t="shared" si="28"/>
         <v>53223672</v>
       </c>
       <c r="N17" s="59">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,N$16)</f>
+        <f t="shared" si="28"/>
         <v>240818885</v>
       </c>
       <c r="O17" s="59">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,O$16)</f>
+        <f t="shared" si="28"/>
         <v>169977929</v>
       </c>
       <c r="P17" s="59">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,P$16)</f>
+        <f t="shared" si="28"/>
         <v>71950539</v>
       </c>
       <c r="Q17" s="59">
@@ -7394,23 +7394,23 @@
       <c r="AF17" s="68"/>
       <c r="AG17" s="68"/>
       <c r="AI17" s="82">
-        <f t="shared" ref="AI17:AM22" si="27">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_region,AI$16)</f>
+        <f t="shared" ref="AI17:AM22" si="29">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_region,AI$16)</f>
         <v>23075</v>
       </c>
       <c r="AJ17" s="17">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>7195</v>
       </c>
       <c r="AK17" s="17">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>39170</v>
       </c>
       <c r="AL17" s="17">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>39255</v>
       </c>
       <c r="AM17" s="17">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>12970</v>
       </c>
       <c r="AN17" s="17">
@@ -7418,23 +7418,23 @@
         <v>121665</v>
       </c>
       <c r="AP17" s="97">
-        <f t="shared" ref="AP17:AT22" si="28">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_region,AP$16)</f>
+        <f t="shared" ref="AP17:AT22" si="30">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_region,AP$16)</f>
         <v>109144041</v>
       </c>
       <c r="AQ17" s="59">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>52631529</v>
       </c>
       <c r="AR17" s="59">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>240927099</v>
       </c>
       <c r="AS17" s="59">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>170461858</v>
       </c>
       <c r="AT17" s="59">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>71950539</v>
       </c>
       <c r="AU17" s="59">
@@ -7455,51 +7455,51 @@
         <v>761464717</v>
       </c>
       <c r="E18" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_producto,E$16)</f>
+        <f t="shared" si="27"/>
         <v>27346</v>
       </c>
       <c r="F18" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_producto,F$16)</f>
+        <f t="shared" si="27"/>
         <v>51553</v>
       </c>
       <c r="G18" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_producto,G$16)</f>
+        <f t="shared" si="27"/>
         <v>19565</v>
       </c>
       <c r="H18" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_producto,H$16)</f>
+        <f t="shared" si="27"/>
         <v>12991</v>
       </c>
       <c r="I18" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_producto,I$16)</f>
+        <f t="shared" si="27"/>
         <v>14165</v>
       </c>
       <c r="J18" s="18">
-        <f t="shared" ref="J18:J22" si="29">SUM(E18:I18)</f>
+        <f t="shared" ref="J18:J22" si="31">SUM(E18:I18)</f>
         <v>125620</v>
       </c>
       <c r="L18" s="98">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_producto,L$16)</f>
+        <f t="shared" si="28"/>
         <v>193222871</v>
       </c>
       <c r="M18" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_producto,M$16)</f>
+        <f t="shared" si="28"/>
         <v>271532147</v>
       </c>
       <c r="N18" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_producto,N$16)</f>
+        <f t="shared" si="28"/>
         <v>131950052</v>
       </c>
       <c r="O18" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_producto,O$16)</f>
+        <f t="shared" si="28"/>
         <v>75839132</v>
       </c>
       <c r="P18" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_producto,P$16)</f>
+        <f t="shared" si="28"/>
         <v>88920515</v>
       </c>
       <c r="Q18" s="60">
-        <f t="shared" ref="Q18:Q22" si="30">SUM(L18:P18)</f>
+        <f t="shared" ref="Q18:Q22" si="32">SUM(L18:P18)</f>
         <v>761464717</v>
       </c>
       <c r="S18" s="94"/>
@@ -7517,51 +7517,51 @@
       <c r="AF18" s="68"/>
       <c r="AG18" s="68"/>
       <c r="AI18" s="83">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>27346</v>
       </c>
       <c r="AJ18" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>51553</v>
       </c>
       <c r="AK18" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>19565</v>
       </c>
       <c r="AL18" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>12991</v>
       </c>
       <c r="AM18" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>14165</v>
       </c>
       <c r="AN18" s="18">
-        <f t="shared" ref="AN18:AN22" si="31">SUM(AI18:AM18)</f>
+        <f t="shared" ref="AN18:AN22" si="33">SUM(AI18:AM18)</f>
         <v>125620</v>
       </c>
       <c r="AP18" s="98">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>193222871</v>
       </c>
       <c r="AQ18" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>271532147</v>
       </c>
       <c r="AR18" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>131950052</v>
       </c>
       <c r="AS18" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>75839132</v>
       </c>
       <c r="AT18" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>88920515</v>
       </c>
       <c r="AU18" s="60">
-        <f t="shared" ref="AU18:AU22" si="32">SUM(AP18:AT18)</f>
+        <f t="shared" ref="AU18:AU22" si="34">SUM(AP18:AT18)</f>
         <v>761464717</v>
       </c>
     </row>
@@ -7578,51 +7578,51 @@
         <v>226722785</v>
       </c>
       <c r="E19" s="84">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_producto,E$16)</f>
+        <f t="shared" si="27"/>
         <v>9125</v>
       </c>
       <c r="F19" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_producto,F$16)</f>
+        <f t="shared" si="27"/>
         <v>9023</v>
       </c>
       <c r="G19" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_producto,G$16)</f>
+        <f t="shared" si="27"/>
         <v>6969</v>
       </c>
       <c r="H19" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_producto,H$16)</f>
+        <f t="shared" si="27"/>
         <v>2096</v>
       </c>
       <c r="I19" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_producto,I$16)</f>
+        <f t="shared" si="27"/>
         <v>5143</v>
       </c>
       <c r="J19" s="19">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>32356</v>
       </c>
       <c r="L19" s="99">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_producto,L$16)</f>
+        <f t="shared" si="28"/>
         <v>59797810</v>
       </c>
       <c r="M19" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_producto,M$16)</f>
+        <f t="shared" si="28"/>
         <v>63246530</v>
       </c>
       <c r="N19" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_producto,N$16)</f>
+        <f t="shared" si="28"/>
         <v>40433106</v>
       </c>
       <c r="O19" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_producto,O$16)</f>
+        <f t="shared" si="28"/>
         <v>31378227</v>
       </c>
       <c r="P19" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_producto,P$16)</f>
+        <f t="shared" si="28"/>
         <v>31867112</v>
       </c>
       <c r="Q19" s="61">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>226722785</v>
       </c>
       <c r="S19" s="94"/>
@@ -7640,51 +7640,51 @@
       <c r="AF19" s="68"/>
       <c r="AG19" s="68"/>
       <c r="AI19" s="84">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>9125</v>
       </c>
       <c r="AJ19" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>9023</v>
       </c>
       <c r="AK19" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>6969</v>
       </c>
       <c r="AL19" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>2096</v>
       </c>
       <c r="AM19" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>5143</v>
       </c>
       <c r="AN19" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>32356</v>
       </c>
       <c r="AP19" s="99">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>59797810</v>
       </c>
       <c r="AQ19" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>63246530</v>
       </c>
       <c r="AR19" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>40433106</v>
       </c>
       <c r="AS19" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>31378227</v>
       </c>
       <c r="AT19" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>31867112</v>
       </c>
       <c r="AU19" s="61">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>226722785</v>
       </c>
     </row>
@@ -7701,51 +7701,51 @@
         <v>312257691</v>
       </c>
       <c r="E20" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_producto,E$16)</f>
+        <f t="shared" si="27"/>
         <v>21722</v>
       </c>
       <c r="F20" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_producto,F$16)</f>
+        <f t="shared" si="27"/>
         <v>197836</v>
       </c>
       <c r="G20" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_producto,G$16)</f>
+        <f t="shared" si="27"/>
         <v>18868</v>
       </c>
       <c r="H20" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_producto,H$16)</f>
+        <f t="shared" si="27"/>
         <v>5457</v>
       </c>
       <c r="I20" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_producto,I$16)</f>
+        <f t="shared" si="27"/>
         <v>112414</v>
       </c>
       <c r="J20" s="18">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>356297</v>
       </c>
       <c r="L20" s="98">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_producto,L$16)</f>
+        <f t="shared" si="28"/>
         <v>135280108</v>
       </c>
       <c r="M20" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_producto,M$16)</f>
+        <f t="shared" si="28"/>
         <v>45710704</v>
       </c>
       <c r="N20" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_producto,N$16)</f>
+        <f t="shared" si="28"/>
         <v>31481567</v>
       </c>
       <c r="O20" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_producto,O$16)</f>
+        <f t="shared" si="28"/>
         <v>23001252</v>
       </c>
       <c r="P20" s="60">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_producto,P$16)</f>
+        <f t="shared" si="28"/>
         <v>76784060</v>
       </c>
       <c r="Q20" s="60">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>312257691</v>
       </c>
       <c r="S20" s="94"/>
@@ -7763,51 +7763,51 @@
       <c r="AF20" s="68"/>
       <c r="AG20" s="68"/>
       <c r="AI20" s="83">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>30665</v>
       </c>
       <c r="AJ20" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>103585</v>
       </c>
       <c r="AK20" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>9925</v>
       </c>
       <c r="AL20" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>197831</v>
       </c>
       <c r="AM20" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>14291</v>
       </c>
       <c r="AN20" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>356297</v>
       </c>
       <c r="AP20" s="98">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>139608342</v>
       </c>
       <c r="AQ20" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>44964557</v>
       </c>
       <c r="AR20" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>27153333</v>
       </c>
       <c r="AS20" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>23830600</v>
       </c>
       <c r="AT20" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>76700859</v>
       </c>
       <c r="AU20" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>312257691</v>
       </c>
     </row>
@@ -7824,51 +7824,51 @@
         <v>722503562</v>
       </c>
       <c r="E21" s="84">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_producto,E$16)</f>
+        <f t="shared" si="27"/>
         <v>18175</v>
       </c>
       <c r="F21" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_producto,F$16)</f>
+        <f t="shared" si="27"/>
         <v>15576</v>
       </c>
       <c r="G21" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_producto,G$16)</f>
+        <f t="shared" si="27"/>
         <v>10706</v>
       </c>
       <c r="H21" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_producto,H$16)</f>
+        <f t="shared" si="27"/>
         <v>55164</v>
       </c>
       <c r="I21" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_producto,I$16)</f>
+        <f t="shared" si="27"/>
         <v>22674</v>
       </c>
       <c r="J21" s="19">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>122295</v>
       </c>
       <c r="L21" s="99">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_producto,L$16)</f>
+        <f t="shared" si="28"/>
         <v>103659911</v>
       </c>
       <c r="M21" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_producto,M$16)</f>
+        <f t="shared" si="28"/>
         <v>93604609</v>
       </c>
       <c r="N21" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_producto,N$16)</f>
+        <f t="shared" si="28"/>
         <v>77744662</v>
       </c>
       <c r="O21" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_producto,O$16)</f>
+        <f t="shared" si="28"/>
         <v>336958448</v>
       </c>
       <c r="P21" s="61">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_producto,P$16)</f>
+        <f t="shared" si="28"/>
         <v>110535932</v>
       </c>
       <c r="Q21" s="61">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>722503562</v>
       </c>
       <c r="S21" s="94"/>
@@ -7886,51 +7886,51 @@
       <c r="AF21" s="68"/>
       <c r="AG21" s="68"/>
       <c r="AI21" s="84">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>11047</v>
       </c>
       <c r="AJ21" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>25399</v>
       </c>
       <c r="AK21" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>12633</v>
       </c>
       <c r="AL21" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>53237</v>
       </c>
       <c r="AM21" s="19">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>19979</v>
       </c>
       <c r="AN21" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>122295</v>
       </c>
       <c r="AP21" s="99">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>94535993</v>
       </c>
       <c r="AQ21" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>93622843</v>
       </c>
       <c r="AR21" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>78668644</v>
       </c>
       <c r="AS21" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>336034466</v>
       </c>
       <c r="AT21" s="61">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>119641616</v>
       </c>
       <c r="AU21" s="61">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>722503562</v>
       </c>
     </row>
@@ -7947,51 +7947,51 @@
         <v>561953724</v>
       </c>
       <c r="E22" s="88">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_producto,E$16)</f>
+        <f t="shared" si="27"/>
         <v>11460</v>
       </c>
       <c r="F22" s="52">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_producto,F$16)</f>
+        <f t="shared" si="27"/>
         <v>16505</v>
       </c>
       <c r="G22" s="52">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_producto,G$16)</f>
+        <f t="shared" si="27"/>
         <v>25030</v>
       </c>
       <c r="H22" s="52">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_producto,H$16)</f>
+        <f t="shared" si="27"/>
         <v>5584</v>
       </c>
       <c r="I22" s="52">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_producto,I$16)</f>
+        <f t="shared" si="27"/>
         <v>41415</v>
       </c>
       <c r="J22" s="52">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>99994</v>
       </c>
       <c r="L22" s="102">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_producto,L$16)</f>
+        <f t="shared" si="28"/>
         <v>49438827</v>
       </c>
       <c r="M22" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_producto,M$16)</f>
+        <f t="shared" si="28"/>
         <v>50806730</v>
       </c>
       <c r="N22" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_producto,N$16)</f>
+        <f t="shared" si="28"/>
         <v>167729464</v>
       </c>
       <c r="O22" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_producto,O$16)</f>
+        <f t="shared" si="28"/>
         <v>17788927</v>
       </c>
       <c r="P22" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_producto,P$16)</f>
+        <f t="shared" si="28"/>
         <v>276189776</v>
       </c>
       <c r="Q22" s="58">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>561953724</v>
       </c>
       <c r="S22" s="94"/>
@@ -8009,51 +8009,51 @@
       <c r="AF22" s="68"/>
       <c r="AG22" s="68"/>
       <c r="AI22" s="83">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>8851</v>
       </c>
       <c r="AJ22" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>16505</v>
       </c>
       <c r="AK22" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>27768</v>
       </c>
       <c r="AL22" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>7382</v>
       </c>
       <c r="AM22" s="18">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>39488</v>
       </c>
       <c r="AN22" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>99994</v>
       </c>
       <c r="AP22" s="98">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>49797905</v>
       </c>
       <c r="AQ22" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>50806730</v>
       </c>
       <c r="AR22" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>168574296</v>
       </c>
       <c r="AS22" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>17133409</v>
       </c>
       <c r="AT22" s="60">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>275641384</v>
       </c>
       <c r="AU22" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>561953724</v>
       </c>
     </row>
@@ -8074,23 +8074,23 @@
         <v>110903</v>
       </c>
       <c r="F23" s="51">
-        <f t="shared" ref="F23:J23" si="33">SUM(F17:F22)</f>
+        <f t="shared" ref="F23:J23" si="35">SUM(F17:F22)</f>
         <v>304519</v>
       </c>
       <c r="G23" s="51">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>118380</v>
       </c>
       <c r="H23" s="51">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>115644</v>
       </c>
       <c r="I23" s="51">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>208781</v>
       </c>
       <c r="J23" s="118">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>858227</v>
       </c>
       <c r="L23" s="109">
@@ -8098,23 +8098,23 @@
         <v>650543568</v>
       </c>
       <c r="M23" s="69">
-        <f t="shared" ref="M23:Q23" si="34">SUM(M17:M22)</f>
+        <f t="shared" ref="M23:Q23" si="36">SUM(M17:M22)</f>
         <v>578124392</v>
       </c>
       <c r="N23" s="69">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>690157736</v>
       </c>
       <c r="O23" s="69">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>654943915</v>
       </c>
       <c r="P23" s="69">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>656247934</v>
       </c>
       <c r="Q23" s="115">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>3230017545</v>
       </c>
       <c r="S23" s="94"/>
@@ -8136,23 +8136,23 @@
         <v>110109</v>
       </c>
       <c r="AJ23" s="51">
-        <f t="shared" ref="AJ23:AN23" si="35">SUM(AJ17:AJ22)</f>
+        <f t="shared" ref="AJ23:AN23" si="37">SUM(AJ17:AJ22)</f>
         <v>213260</v>
       </c>
       <c r="AK23" s="51">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v>116030</v>
       </c>
       <c r="AL23" s="51">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v>312792</v>
       </c>
       <c r="AM23" s="51">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v>106036</v>
       </c>
       <c r="AN23" s="118">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v>858227</v>
       </c>
       <c r="AP23" s="109">
@@ -8160,23 +8160,23 @@
         <v>646106962</v>
       </c>
       <c r="AQ23" s="69">
-        <f t="shared" ref="AQ23" si="36">SUM(AQ17:AQ22)</f>
+        <f t="shared" ref="AQ23" si="38">SUM(AQ17:AQ22)</f>
         <v>576804336</v>
       </c>
       <c r="AR23" s="69">
-        <f t="shared" ref="AR23" si="37">SUM(AR17:AR22)</f>
+        <f t="shared" ref="AR23" si="39">SUM(AR17:AR22)</f>
         <v>687706530</v>
       </c>
       <c r="AS23" s="69">
-        <f t="shared" ref="AS23" si="38">SUM(AS17:AS22)</f>
+        <f t="shared" ref="AS23" si="40">SUM(AS17:AS22)</f>
         <v>654677692</v>
       </c>
       <c r="AT23" s="69">
-        <f t="shared" ref="AT23" si="39">SUM(AT17:AT22)</f>
+        <f t="shared" ref="AT23" si="41">SUM(AT17:AT22)</f>
         <v>664722025</v>
       </c>
       <c r="AU23" s="115">
-        <f t="shared" ref="AU23" si="40">SUM(AU17:AU22)</f>
+        <f t="shared" ref="AU23" si="42">SUM(AU17:AU22)</f>
         <v>3230017545</v>
       </c>
     </row>
@@ -8295,23 +8295,23 @@
         <v>646106962</v>
       </c>
       <c r="E26" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,E$25)</f>
+        <f t="shared" ref="E26:I30" si="43">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,E$25)</f>
         <v>101037</v>
       </c>
       <c r="F26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,F$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="G26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,G$25)</f>
+        <f t="shared" si="43"/>
         <v>8943</v>
       </c>
       <c r="H26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,H$25)</f>
+        <f t="shared" si="43"/>
         <v>129</v>
       </c>
       <c r="I26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,I$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="J26" s="17">
@@ -8319,23 +8319,23 @@
         <v>858227</v>
       </c>
       <c r="L26" s="97">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,L$25)</f>
+        <f t="shared" ref="L26:P30" si="44">SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,L$25)</f>
         <v>640574818</v>
       </c>
       <c r="M26" s="59">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,M$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="N26" s="59">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,N$25)</f>
+        <f t="shared" si="44"/>
         <v>4328234</v>
       </c>
       <c r="O26" s="59">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,O$25)</f>
+        <f t="shared" si="44"/>
         <v>1203910</v>
       </c>
       <c r="P26" s="59">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,P$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="Q26" s="59">
@@ -8343,27 +8343,27 @@
         <v>646106962</v>
       </c>
       <c r="S26" s="82">
-        <f t="shared" ref="S26:X30" si="41">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_vendedor,S$25)</f>
+        <f t="shared" ref="S26:X30" si="45">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_vendedor,S$25)</f>
         <v>23075</v>
       </c>
       <c r="T26" s="29">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>27346</v>
       </c>
       <c r="U26" s="29">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>9125</v>
       </c>
       <c r="V26" s="17">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>30665</v>
       </c>
       <c r="W26" s="29">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>11047</v>
       </c>
       <c r="X26" s="29">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>8851</v>
       </c>
       <c r="Y26" s="17">
@@ -8371,27 +8371,27 @@
         <v>110109</v>
       </c>
       <c r="AA26" s="97">
-        <f t="shared" ref="AA26:AF30" si="42">SUMIFS(ventas_total,ventas_region,$A26,ventas_vendedor,AA$25)</f>
+        <f t="shared" ref="AA26:AF30" si="46">SUMIFS(ventas_total,ventas_region,$A26,ventas_vendedor,AA$25)</f>
         <v>109144041</v>
       </c>
       <c r="AB26" s="64">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>193222871</v>
       </c>
       <c r="AC26" s="64">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>59797810</v>
       </c>
       <c r="AD26" s="59">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>139608342</v>
       </c>
       <c r="AE26" s="64">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>94535993</v>
       </c>
       <c r="AF26" s="64">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>49797905</v>
       </c>
       <c r="AG26" s="59">
@@ -8424,107 +8424,107 @@
         <v>576804336</v>
       </c>
       <c r="E27" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,E$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="F27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,F$25)</f>
+        <f t="shared" si="43"/>
         <v>105314</v>
       </c>
       <c r="G27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,G$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="H27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,H$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="I27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,I$25)</f>
+        <f t="shared" si="43"/>
         <v>107946</v>
       </c>
       <c r="J27" s="18">
-        <f t="shared" ref="J27:J30" si="43">SUM(E27:I31)</f>
+        <f t="shared" ref="J27:J30" si="47">SUM(E27:I31)</f>
         <v>1606345</v>
       </c>
       <c r="L27" s="98">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_producto,L$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="M27" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_producto,M$25)</f>
+        <f t="shared" si="44"/>
         <v>576702901</v>
       </c>
       <c r="N27" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_producto,N$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="O27" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_producto,O$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="P27" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_producto,P$25)</f>
+        <f t="shared" si="44"/>
         <v>101435</v>
       </c>
       <c r="Q27" s="60">
-        <f t="shared" ref="Q27:Q30" si="44">SUM(L27:P27)</f>
+        <f t="shared" ref="Q27:Q30" si="48">SUM(L27:P27)</f>
         <v>576804336</v>
       </c>
       <c r="S27" s="91">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>7195</v>
       </c>
       <c r="T27" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>51553</v>
       </c>
       <c r="U27" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>9023</v>
       </c>
       <c r="V27" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>103585</v>
       </c>
       <c r="W27" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>25399</v>
       </c>
       <c r="X27" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>16505</v>
       </c>
       <c r="Y27" s="30">
-        <f t="shared" ref="Y27:Y30" si="45">SUM(S27:X27)</f>
+        <f t="shared" ref="Y27:Y30" si="49">SUM(S27:X27)</f>
         <v>213260</v>
       </c>
       <c r="AA27" s="105">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>52631529</v>
       </c>
       <c r="AB27" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>271532147</v>
       </c>
       <c r="AC27" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>63246530</v>
       </c>
       <c r="AD27" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>44964557</v>
       </c>
       <c r="AE27" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>93622843</v>
       </c>
       <c r="AF27" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>50806730</v>
       </c>
       <c r="AG27" s="65">
-        <f t="shared" ref="AG27:AG30" si="46">SUM(AA27:AF27)</f>
+        <f t="shared" ref="AG27:AG30" si="50">SUM(AA27:AF27)</f>
         <v>576804336</v>
       </c>
       <c r="AI27" s="94"/>
@@ -8553,107 +8553,107 @@
         <v>687706530</v>
       </c>
       <c r="E28" s="84">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,E$25)</f>
+        <f t="shared" si="43"/>
         <v>2738</v>
       </c>
       <c r="F28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,F$25)</f>
+        <f t="shared" si="43"/>
         <v>1928</v>
       </c>
       <c r="G28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,G$25)</f>
+        <f t="shared" si="43"/>
         <v>109437</v>
       </c>
       <c r="H28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,H$25)</f>
+        <f t="shared" si="43"/>
         <v>1927</v>
       </c>
       <c r="I28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,I$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="J28" s="19">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>1393085</v>
       </c>
       <c r="L28" s="99">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_producto,L$25)</f>
+        <f t="shared" si="44"/>
         <v>844832</v>
       </c>
       <c r="M28" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_producto,M$25)</f>
+        <f t="shared" si="44"/>
         <v>108214</v>
       </c>
       <c r="N28" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_producto,N$25)</f>
+        <f t="shared" si="44"/>
         <v>685829502</v>
       </c>
       <c r="O28" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_producto,O$25)</f>
+        <f t="shared" si="44"/>
         <v>923982</v>
       </c>
       <c r="P28" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_producto,P$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="Q28" s="61">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>687706530</v>
       </c>
       <c r="S28" s="92">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>39170</v>
       </c>
       <c r="T28" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>19565</v>
       </c>
       <c r="U28" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>6969</v>
       </c>
       <c r="V28" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>9925</v>
       </c>
       <c r="W28" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>12633</v>
       </c>
       <c r="X28" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>27768</v>
       </c>
       <c r="Y28" s="31">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>116030</v>
       </c>
       <c r="AA28" s="106">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>240927099</v>
       </c>
       <c r="AB28" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>131950052</v>
       </c>
       <c r="AC28" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>40433106</v>
       </c>
       <c r="AD28" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>27153333</v>
       </c>
       <c r="AE28" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>78668644</v>
       </c>
       <c r="AF28" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>168574296</v>
       </c>
       <c r="AG28" s="66">
-        <f t="shared" si="46"/>
+        <f t="shared" si="50"/>
         <v>687706530</v>
       </c>
       <c r="AI28" s="94"/>
@@ -8682,107 +8682,107 @@
         <v>654677692</v>
       </c>
       <c r="E29" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,E$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="F29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,F$25)</f>
+        <f t="shared" si="43"/>
         <v>197277</v>
       </c>
       <c r="G29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,G$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="H29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,H$25)</f>
+        <f t="shared" si="43"/>
         <v>113588</v>
       </c>
       <c r="I29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,I$25)</f>
+        <f t="shared" si="43"/>
         <v>1927</v>
       </c>
       <c r="J29" s="18">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>1277055</v>
       </c>
       <c r="L29" s="98">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_producto,L$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="M29" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_producto,M$25)</f>
+        <f t="shared" si="44"/>
         <v>1313277</v>
       </c>
       <c r="N29" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_producto,N$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="O29" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_producto,O$25)</f>
+        <f t="shared" si="44"/>
         <v>652816023</v>
       </c>
       <c r="P29" s="60">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_producto,P$25)</f>
+        <f t="shared" si="44"/>
         <v>548392</v>
       </c>
       <c r="Q29" s="60">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>654677692</v>
       </c>
       <c r="S29" s="91">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>39255</v>
       </c>
       <c r="T29" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>12991</v>
       </c>
       <c r="U29" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>2096</v>
       </c>
       <c r="V29" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>197831</v>
       </c>
       <c r="W29" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>53237</v>
       </c>
       <c r="X29" s="30">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>7382</v>
       </c>
       <c r="Y29" s="30">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>312792</v>
       </c>
       <c r="AA29" s="105">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>170461858</v>
       </c>
       <c r="AB29" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>75839132</v>
       </c>
       <c r="AC29" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>31378227</v>
       </c>
       <c r="AD29" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>23830600</v>
       </c>
       <c r="AE29" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>336034466</v>
       </c>
       <c r="AF29" s="65">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>17133409</v>
       </c>
       <c r="AG29" s="65">
-        <f t="shared" si="46"/>
+        <f t="shared" si="50"/>
         <v>654677692</v>
       </c>
       <c r="AI29" s="94"/>
@@ -8811,107 +8811,107 @@
         <v>664722025</v>
       </c>
       <c r="E30" s="84">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,E$25)</f>
+        <f t="shared" si="43"/>
         <v>7128</v>
       </c>
       <c r="F30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,F$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="G30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,G$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="H30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,H$25)</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="I30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,I$25)</f>
+        <f t="shared" si="43"/>
         <v>98908</v>
       </c>
       <c r="J30" s="19">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>1146245</v>
       </c>
       <c r="L30" s="99">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_producto,L$25)</f>
+        <f t="shared" si="44"/>
         <v>9123918</v>
       </c>
       <c r="M30" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_producto,M$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="N30" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_producto,N$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="O30" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_producto,O$25)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="P30" s="61">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_producto,P$25)</f>
+        <f t="shared" si="44"/>
         <v>655598107</v>
       </c>
       <c r="Q30" s="61">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>664722025</v>
       </c>
       <c r="S30" s="92">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>12970</v>
       </c>
       <c r="T30" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>14165</v>
       </c>
       <c r="U30" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>5143</v>
       </c>
       <c r="V30" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>14291</v>
       </c>
       <c r="W30" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>19979</v>
       </c>
       <c r="X30" s="31">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>39488</v>
       </c>
       <c r="Y30" s="31">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>106036</v>
       </c>
       <c r="AA30" s="106">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>71950539</v>
       </c>
       <c r="AB30" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>88920515</v>
       </c>
       <c r="AC30" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>31867112</v>
       </c>
       <c r="AD30" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>76700859</v>
       </c>
       <c r="AE30" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>119641616</v>
       </c>
       <c r="AF30" s="66">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>275641384</v>
       </c>
       <c r="AG30" s="66">
-        <f t="shared" si="46"/>
+        <f t="shared" si="50"/>
         <v>664722025</v>
       </c>
       <c r="AI30" s="94"/>
@@ -8944,23 +8944,23 @@
         <v>110903</v>
       </c>
       <c r="F31" s="51">
-        <f t="shared" ref="F31:J31" si="47">SUM(F26:F30)</f>
+        <f t="shared" ref="F31:J31" si="51">SUM(F26:F30)</f>
         <v>304519</v>
       </c>
       <c r="G31" s="51">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>118380</v>
       </c>
       <c r="H31" s="51">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>115644</v>
       </c>
       <c r="I31" s="51">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>208781</v>
       </c>
       <c r="J31" s="118">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>6280957</v>
       </c>
       <c r="L31" s="109">
@@ -8968,23 +8968,23 @@
         <v>650543568</v>
       </c>
       <c r="M31" s="69">
-        <f t="shared" ref="M31" si="48">SUM(M26:M30)</f>
+        <f t="shared" ref="M31" si="52">SUM(M26:M30)</f>
         <v>578124392</v>
       </c>
       <c r="N31" s="69">
-        <f t="shared" ref="N31" si="49">SUM(N26:N30)</f>
+        <f t="shared" ref="N31" si="53">SUM(N26:N30)</f>
         <v>690157736</v>
       </c>
       <c r="O31" s="69">
-        <f t="shared" ref="O31" si="50">SUM(O26:O30)</f>
+        <f t="shared" ref="O31" si="54">SUM(O26:O30)</f>
         <v>654943915</v>
       </c>
       <c r="P31" s="69">
-        <f t="shared" ref="P31" si="51">SUM(P26:P30)</f>
+        <f t="shared" ref="P31" si="55">SUM(P26:P30)</f>
         <v>656247934</v>
       </c>
       <c r="Q31" s="115">
-        <f t="shared" ref="Q31" si="52">SUM(Q26:Q30)</f>
+        <f t="shared" ref="Q31" si="56">SUM(Q26:Q30)</f>
         <v>3230017545</v>
       </c>
       <c r="S31" s="93">
@@ -8992,27 +8992,27 @@
         <v>121665</v>
       </c>
       <c r="T31" s="40">
-        <f t="shared" ref="T31:Y31" si="53">SUM(T26:T30)</f>
+        <f t="shared" ref="T31:Y31" si="57">SUM(T26:T30)</f>
         <v>125620</v>
       </c>
       <c r="U31" s="40">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>32356</v>
       </c>
       <c r="V31" s="40">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>356297</v>
       </c>
       <c r="W31" s="40">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>122295</v>
       </c>
       <c r="X31" s="40">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>99994</v>
       </c>
       <c r="Y31" s="40">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>858227</v>
       </c>
       <c r="AA31" s="107">
@@ -9020,27 +9020,27 @@
         <v>645115066</v>
       </c>
       <c r="AB31" s="67">
-        <f t="shared" ref="AB31" si="54">SUM(AB26:AB30)</f>
+        <f t="shared" ref="AB31" si="58">SUM(AB26:AB30)</f>
         <v>761464717</v>
       </c>
       <c r="AC31" s="67">
-        <f t="shared" ref="AC31" si="55">SUM(AC26:AC30)</f>
+        <f t="shared" ref="AC31" si="59">SUM(AC26:AC30)</f>
         <v>226722785</v>
       </c>
       <c r="AD31" s="67">
-        <f t="shared" ref="AD31" si="56">SUM(AD26:AD30)</f>
+        <f t="shared" ref="AD31" si="60">SUM(AD26:AD30)</f>
         <v>312257691</v>
       </c>
       <c r="AE31" s="67">
-        <f t="shared" ref="AE31" si="57">SUM(AE26:AE30)</f>
+        <f t="shared" ref="AE31" si="61">SUM(AE26:AE30)</f>
         <v>722503562</v>
       </c>
       <c r="AF31" s="67">
-        <f t="shared" ref="AF31" si="58">SUM(AF26:AF30)</f>
+        <f t="shared" ref="AF31" si="62">SUM(AF26:AF30)</f>
         <v>561953724</v>
       </c>
       <c r="AG31" s="115">
-        <f t="shared" ref="AG31" si="59">SUM(AG26:AG30)</f>
+        <f t="shared" ref="AG31" si="63">SUM(AG26:AG30)</f>
         <v>3230017545</v>
       </c>
       <c r="AI31" s="94"/>
@@ -9195,23 +9195,23 @@
         <v>1007244151</v>
       </c>
       <c r="E34" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,E$25)</f>
+        <f t="shared" ref="E34:I38" si="64">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,E$25)</f>
         <v>33032</v>
       </c>
       <c r="F34" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,F$25)</f>
+        <f t="shared" si="64"/>
         <v>32696</v>
       </c>
       <c r="G34" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,G$25)</f>
+        <f t="shared" si="64"/>
         <v>39124</v>
       </c>
       <c r="H34" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,H$25)</f>
+        <f t="shared" si="64"/>
         <v>40573</v>
       </c>
       <c r="I34" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,I$25)</f>
+        <f t="shared" si="64"/>
         <v>36557</v>
       </c>
       <c r="J34" s="17">
@@ -9219,23 +9219,23 @@
         <v>858227</v>
       </c>
       <c r="L34" s="97">
-        <f>SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,L$25)</f>
+        <f t="shared" ref="L34:P38" si="65">SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,L$25)</f>
         <v>218669111</v>
       </c>
       <c r="M34" s="59">
-        <f>SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,M$25)</f>
+        <f t="shared" si="65"/>
         <v>160364763</v>
       </c>
       <c r="N34" s="59">
-        <f>SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,N$25)</f>
+        <f t="shared" si="65"/>
         <v>220801841</v>
       </c>
       <c r="O34" s="59">
-        <f>SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,O$25)</f>
+        <f t="shared" si="65"/>
         <v>190929354</v>
       </c>
       <c r="P34" s="59">
-        <f>SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,P$25)</f>
+        <f t="shared" si="65"/>
         <v>216479082</v>
       </c>
       <c r="Q34" s="59">
@@ -9243,27 +9243,27 @@
         <v>1007244151</v>
       </c>
       <c r="S34" s="90">
-        <f t="shared" ref="S34:X38" si="60">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,S$33)</f>
+        <f t="shared" ref="S34:X38" si="66">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,S$33)</f>
         <v>33623</v>
       </c>
       <c r="T34" s="29">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>45235</v>
       </c>
       <c r="U34" s="29">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>12423</v>
       </c>
       <c r="V34" s="29">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>20990</v>
       </c>
       <c r="W34" s="29">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>44558</v>
       </c>
       <c r="X34" s="29">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>25153</v>
       </c>
       <c r="Y34" s="29">
@@ -9271,27 +9271,27 @@
         <v>181982</v>
       </c>
       <c r="AA34" s="104">
-        <f t="shared" ref="AA34:AF38" si="61">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,AA$33)</f>
+        <f t="shared" ref="AA34:AF38" si="67">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,AA$33)</f>
         <v>33623</v>
       </c>
       <c r="AB34" s="64">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>45235</v>
       </c>
       <c r="AC34" s="64">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>12423</v>
       </c>
       <c r="AD34" s="64">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>20990</v>
       </c>
       <c r="AE34" s="64">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>44558</v>
       </c>
       <c r="AF34" s="64">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>25153</v>
       </c>
       <c r="AG34" s="64">
@@ -9299,23 +9299,23 @@
         <v>181982</v>
       </c>
       <c r="AI34" s="82">
-        <f t="shared" ref="AI34:AM38" si="62">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_region,AI$33)</f>
+        <f t="shared" ref="AI34:AM38" si="68">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_region,AI$33)</f>
         <v>33032</v>
       </c>
       <c r="AJ34" s="17">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>32696</v>
       </c>
       <c r="AK34" s="17">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>39124</v>
       </c>
       <c r="AL34" s="17">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>40573</v>
       </c>
       <c r="AM34" s="17">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>36557</v>
       </c>
       <c r="AN34" s="17">
@@ -9323,23 +9323,23 @@
         <v>181982</v>
       </c>
       <c r="AP34" s="111">
-        <f t="shared" ref="AP34:AT38" si="63">SUMIFS(ventas_total,ventas_año,$A34,ventas_region,AP$33)</f>
+        <f t="shared" ref="AP34:AT38" si="69">SUMIFS(ventas_total,ventas_año,$A34,ventas_region,AP$33)</f>
         <v>218669111</v>
       </c>
       <c r="AQ34" s="41">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>160364763</v>
       </c>
       <c r="AR34" s="41">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>220801841</v>
       </c>
       <c r="AS34" s="41">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>190929354</v>
       </c>
       <c r="AT34" s="41">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>216479082</v>
       </c>
       <c r="AU34" s="41">
@@ -9360,155 +9360,155 @@
         <v>1106846472</v>
       </c>
       <c r="E35" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A35,ventas_producto,E$25)</f>
+        <f t="shared" si="64"/>
         <v>32671</v>
       </c>
       <c r="F35" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A35,ventas_producto,F$25)</f>
+        <f t="shared" si="64"/>
         <v>31651</v>
       </c>
       <c r="G35" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A35,ventas_producto,G$25)</f>
+        <f t="shared" si="64"/>
         <v>34000</v>
       </c>
       <c r="H35" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A35,ventas_producto,H$25)</f>
+        <f t="shared" si="64"/>
         <v>39442</v>
       </c>
       <c r="I35" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A35,ventas_producto,I$25)</f>
+        <f t="shared" si="64"/>
         <v>28900</v>
       </c>
       <c r="J35" s="18">
-        <f t="shared" ref="J35:J38" si="64">SUM(E35:I39)</f>
+        <f t="shared" ref="J35:J38" si="70">SUM(E35:I39)</f>
         <v>1534472</v>
       </c>
       <c r="L35" s="98">
-        <f>SUMIFS(ventas_total,ventas_año,$A35,ventas_producto,L$25)</f>
+        <f t="shared" si="65"/>
         <v>203341463</v>
       </c>
       <c r="M35" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A35,ventas_producto,M$25)</f>
+        <f t="shared" si="65"/>
         <v>201880917</v>
       </c>
       <c r="N35" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A35,ventas_producto,N$25)</f>
+        <f t="shared" si="65"/>
         <v>239992813</v>
       </c>
       <c r="O35" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A35,ventas_producto,O$25)</f>
+        <f t="shared" si="65"/>
         <v>221383553</v>
       </c>
       <c r="P35" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A35,ventas_producto,P$25)</f>
+        <f t="shared" si="65"/>
         <v>240247726</v>
       </c>
       <c r="Q35" s="60">
-        <f t="shared" ref="Q35:Q38" si="65">SUM(L35:P35)</f>
+        <f t="shared" ref="Q35:Q38" si="71">SUM(L35:P35)</f>
         <v>1106846472</v>
       </c>
       <c r="S35" s="91">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>42339</v>
       </c>
       <c r="T35" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>39435</v>
       </c>
       <c r="U35" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>12194</v>
       </c>
       <c r="V35" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>11750</v>
       </c>
       <c r="W35" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>27319</v>
       </c>
       <c r="X35" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>33627</v>
       </c>
       <c r="Y35" s="30">
-        <f t="shared" ref="Y35:Y38" si="66">SUM(S35:X35)</f>
+        <f t="shared" ref="Y35:Y38" si="72">SUM(S35:X35)</f>
         <v>166664</v>
       </c>
       <c r="AA35" s="105">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>42339</v>
       </c>
       <c r="AB35" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>39435</v>
       </c>
       <c r="AC35" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>12194</v>
       </c>
       <c r="AD35" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>11750</v>
       </c>
       <c r="AE35" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>27319</v>
       </c>
       <c r="AF35" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>33627</v>
       </c>
       <c r="AG35" s="65">
-        <f t="shared" ref="AG35:AG38" si="67">SUM(AA35:AF35)</f>
+        <f t="shared" ref="AG35:AG38" si="73">SUM(AA35:AF35)</f>
         <v>166664</v>
       </c>
       <c r="AI35" s="83">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>32671</v>
       </c>
       <c r="AJ35" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>31651</v>
       </c>
       <c r="AK35" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>34000</v>
       </c>
       <c r="AL35" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>39442</v>
       </c>
       <c r="AM35" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>28900</v>
       </c>
       <c r="AN35" s="18">
-        <f t="shared" ref="AN35:AN38" si="68">SUM(AI35:AM35)</f>
+        <f t="shared" ref="AN35:AN38" si="74">SUM(AI35:AM35)</f>
         <v>166664</v>
       </c>
       <c r="AP35" s="112">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>203341463</v>
       </c>
       <c r="AQ35" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>201880917</v>
       </c>
       <c r="AR35" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>239992813</v>
       </c>
       <c r="AS35" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>221383553</v>
       </c>
       <c r="AT35" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>240247726</v>
       </c>
       <c r="AU35" s="45">
-        <f t="shared" ref="AU35:AU38" si="69">SUM(AP35:AT35)</f>
+        <f t="shared" ref="AU35:AU38" si="75">SUM(AP35:AT35)</f>
         <v>1106846472</v>
       </c>
     </row>
@@ -9525,155 +9525,155 @@
         <v>1089310347</v>
       </c>
       <c r="E36" s="84">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A36,ventas_producto,E$25)</f>
+        <f t="shared" si="64"/>
         <v>35334</v>
       </c>
       <c r="F36" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A36,ventas_producto,F$25)</f>
+        <f t="shared" si="64"/>
         <v>40967</v>
       </c>
       <c r="G36" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A36,ventas_producto,G$25)</f>
+        <f t="shared" si="64"/>
         <v>31330</v>
       </c>
       <c r="H36" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A36,ventas_producto,H$25)</f>
+        <f t="shared" si="64"/>
         <v>33573</v>
       </c>
       <c r="I36" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A36,ventas_producto,I$25)</f>
+        <f t="shared" si="64"/>
         <v>33451</v>
       </c>
       <c r="J36" s="19">
-        <f t="shared" si="64"/>
+        <f t="shared" si="70"/>
         <v>1367808</v>
       </c>
       <c r="L36" s="99">
-        <f>SUMIFS(ventas_total,ventas_año,$A36,ventas_producto,L$25)</f>
+        <f t="shared" si="65"/>
         <v>218564244</v>
       </c>
       <c r="M36" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A36,ventas_producto,M$25)</f>
+        <f t="shared" si="65"/>
         <v>214457221</v>
       </c>
       <c r="N36" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A36,ventas_producto,N$25)</f>
+        <f t="shared" si="65"/>
         <v>216914467</v>
       </c>
       <c r="O36" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A36,ventas_producto,O$25)</f>
+        <f t="shared" si="65"/>
         <v>240503116</v>
       </c>
       <c r="P36" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A36,ventas_producto,P$25)</f>
+        <f t="shared" si="65"/>
         <v>198871299</v>
       </c>
       <c r="Q36" s="61">
-        <f t="shared" si="65"/>
+        <f t="shared" si="71"/>
         <v>1089310347</v>
       </c>
       <c r="S36" s="92">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>33889</v>
       </c>
       <c r="T36" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>40950</v>
       </c>
       <c r="U36" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>7739</v>
       </c>
       <c r="V36" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>24117</v>
       </c>
       <c r="W36" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>31540</v>
       </c>
       <c r="X36" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>36420</v>
       </c>
       <c r="Y36" s="31">
-        <f t="shared" si="66"/>
+        <f t="shared" si="72"/>
         <v>174655</v>
       </c>
       <c r="AA36" s="106">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>33889</v>
       </c>
       <c r="AB36" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>40950</v>
       </c>
       <c r="AC36" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>7739</v>
       </c>
       <c r="AD36" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>24117</v>
       </c>
       <c r="AE36" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>31540</v>
       </c>
       <c r="AF36" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>36420</v>
       </c>
       <c r="AG36" s="66">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>174655</v>
       </c>
       <c r="AI36" s="84">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>35334</v>
       </c>
       <c r="AJ36" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>40967</v>
       </c>
       <c r="AK36" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>31330</v>
       </c>
       <c r="AL36" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>33573</v>
       </c>
       <c r="AM36" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>33451</v>
       </c>
       <c r="AN36" s="19">
-        <f t="shared" si="68"/>
+        <f t="shared" si="74"/>
         <v>174655</v>
       </c>
       <c r="AP36" s="113">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>218564244</v>
       </c>
       <c r="AQ36" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>214457221</v>
       </c>
       <c r="AR36" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>216914467</v>
       </c>
       <c r="AS36" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>240503116</v>
       </c>
       <c r="AT36" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>198871299</v>
       </c>
       <c r="AU36" s="46">
-        <f t="shared" si="69"/>
+        <f t="shared" si="75"/>
         <v>1089310347</v>
       </c>
     </row>
@@ -9690,155 +9690,155 @@
         <v>15082721</v>
       </c>
       <c r="E37" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A37,ventas_producto,E$25)</f>
+        <f t="shared" si="64"/>
         <v>2738</v>
       </c>
       <c r="F37" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A37,ventas_producto,F$25)</f>
+        <f t="shared" si="64"/>
         <v>4903</v>
       </c>
       <c r="G37" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A37,ventas_producto,G$25)</f>
+        <f t="shared" si="64"/>
         <v>13926</v>
       </c>
       <c r="H37" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A37,ventas_producto,H$25)</f>
+        <f t="shared" si="64"/>
         <v>129</v>
       </c>
       <c r="I37" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A37,ventas_producto,I$25)</f>
+        <f t="shared" si="64"/>
         <v>107946</v>
       </c>
       <c r="J37" s="18">
-        <f t="shared" si="64"/>
+        <f t="shared" si="70"/>
         <v>1193153</v>
       </c>
       <c r="L37" s="98">
-        <f>SUMIFS(ventas_total,ventas_año,$A37,ventas_producto,L$25)</f>
+        <f t="shared" si="65"/>
         <v>844832</v>
       </c>
       <c r="M37" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A37,ventas_producto,M$25)</f>
+        <f t="shared" si="65"/>
         <v>483929</v>
       </c>
       <c r="N37" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A37,ventas_producto,N$25)</f>
+        <f t="shared" si="65"/>
         <v>12448615</v>
       </c>
       <c r="O37" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A37,ventas_producto,O$25)</f>
+        <f t="shared" si="65"/>
         <v>1203910</v>
       </c>
       <c r="P37" s="60">
-        <f>SUMIFS(ventas_total,ventas_año,$A37,ventas_producto,P$25)</f>
+        <f t="shared" si="65"/>
         <v>101435</v>
       </c>
       <c r="Q37" s="60">
-        <f t="shared" si="65"/>
+        <f t="shared" si="71"/>
         <v>15082721</v>
       </c>
       <c r="S37" s="91">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>9886</v>
       </c>
       <c r="T37" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>0</v>
       </c>
       <c r="U37" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>0</v>
       </c>
       <c r="V37" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>107066</v>
       </c>
       <c r="W37" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>9823</v>
       </c>
       <c r="X37" s="30">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>2867</v>
       </c>
       <c r="Y37" s="30">
-        <f t="shared" si="66"/>
+        <f t="shared" si="72"/>
         <v>129642</v>
       </c>
       <c r="AA37" s="105">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>9886</v>
       </c>
       <c r="AB37" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="AC37" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="AD37" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>107066</v>
       </c>
       <c r="AE37" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>9823</v>
       </c>
       <c r="AF37" s="65">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>2867</v>
       </c>
       <c r="AG37" s="65">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>129642</v>
       </c>
       <c r="AI37" s="83">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>9072</v>
       </c>
       <c r="AJ37" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>107946</v>
       </c>
       <c r="AK37" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>7721</v>
       </c>
       <c r="AL37" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>4903</v>
       </c>
       <c r="AM37" s="18">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>0</v>
       </c>
       <c r="AN37" s="18">
-        <f t="shared" si="68"/>
+        <f t="shared" si="74"/>
         <v>129642</v>
       </c>
       <c r="AP37" s="112">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>5532144</v>
       </c>
       <c r="AQ37" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>101435</v>
       </c>
       <c r="AR37" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>8965213</v>
       </c>
       <c r="AS37" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>483929</v>
       </c>
       <c r="AT37" s="45">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>0</v>
       </c>
       <c r="AU37" s="45">
-        <f t="shared" si="69"/>
+        <f t="shared" si="75"/>
         <v>15082721</v>
       </c>
     </row>
@@ -9855,155 +9855,155 @@
         <v>11533854</v>
       </c>
       <c r="E38" s="84">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A38,ventas_producto,E$25)</f>
+        <f t="shared" si="64"/>
         <v>7128</v>
       </c>
       <c r="F38" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A38,ventas_producto,F$25)</f>
+        <f t="shared" si="64"/>
         <v>194302</v>
       </c>
       <c r="G38" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A38,ventas_producto,G$25)</f>
+        <f t="shared" si="64"/>
         <v>0</v>
       </c>
       <c r="H38" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A38,ventas_producto,H$25)</f>
+        <f t="shared" si="64"/>
         <v>1927</v>
       </c>
       <c r="I38" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_año,$A38,ventas_producto,I$25)</f>
+        <f t="shared" si="64"/>
         <v>1927</v>
       </c>
       <c r="J38" s="19">
-        <f t="shared" si="64"/>
+        <f t="shared" si="70"/>
         <v>1063511</v>
       </c>
       <c r="L38" s="99">
-        <f>SUMIFS(ventas_total,ventas_año,$A38,ventas_producto,L$25)</f>
+        <f t="shared" si="65"/>
         <v>9123918</v>
       </c>
       <c r="M38" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A38,ventas_producto,M$25)</f>
+        <f t="shared" si="65"/>
         <v>937562</v>
       </c>
       <c r="N38" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A38,ventas_producto,N$25)</f>
+        <f t="shared" si="65"/>
         <v>0</v>
       </c>
       <c r="O38" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A38,ventas_producto,O$25)</f>
+        <f t="shared" si="65"/>
         <v>923982</v>
       </c>
       <c r="P38" s="61">
-        <f>SUMIFS(ventas_total,ventas_año,$A38,ventas_producto,P$25)</f>
+        <f t="shared" si="65"/>
         <v>548392</v>
       </c>
       <c r="Q38" s="61">
-        <f t="shared" si="65"/>
+        <f t="shared" si="71"/>
         <v>11533854</v>
       </c>
       <c r="S38" s="92">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>1928</v>
       </c>
       <c r="T38" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>0</v>
       </c>
       <c r="U38" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>0</v>
       </c>
       <c r="V38" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>192374</v>
       </c>
       <c r="W38" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>9055</v>
       </c>
       <c r="X38" s="31">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>1927</v>
       </c>
       <c r="Y38" s="31">
-        <f t="shared" si="66"/>
+        <f t="shared" si="72"/>
         <v>205284</v>
       </c>
       <c r="AA38" s="106">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>1928</v>
       </c>
       <c r="AB38" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="AC38" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="AD38" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>192374</v>
       </c>
       <c r="AE38" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>9055</v>
       </c>
       <c r="AF38" s="66">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>1927</v>
       </c>
       <c r="AG38" s="66">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>205284</v>
       </c>
       <c r="AI38" s="84">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>0</v>
       </c>
       <c r="AJ38" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>0</v>
       </c>
       <c r="AK38" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>3855</v>
       </c>
       <c r="AL38" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>194301</v>
       </c>
       <c r="AM38" s="19">
-        <f t="shared" si="62"/>
+        <f t="shared" si="68"/>
         <v>7128</v>
       </c>
       <c r="AN38" s="19">
-        <f t="shared" si="68"/>
+        <f t="shared" si="74"/>
         <v>205284</v>
       </c>
       <c r="AP38" s="113">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>0</v>
       </c>
       <c r="AQ38" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>0</v>
       </c>
       <c r="AR38" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>1032196</v>
       </c>
       <c r="AS38" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>1377740</v>
       </c>
       <c r="AT38" s="46">
-        <f t="shared" si="63"/>
+        <f t="shared" si="69"/>
         <v>9123918</v>
       </c>
       <c r="AU38" s="46">
-        <f t="shared" si="69"/>
+        <f t="shared" si="75"/>
         <v>11533854</v>
       </c>
     </row>
@@ -10024,23 +10024,23 @@
         <v>110903</v>
       </c>
       <c r="F39" s="51">
-        <f t="shared" ref="F39" si="70">SUM(F34:F38)</f>
+        <f t="shared" ref="F39" si="76">SUM(F34:F38)</f>
         <v>304519</v>
       </c>
       <c r="G39" s="51">
-        <f t="shared" ref="G39" si="71">SUM(G34:G38)</f>
+        <f t="shared" ref="G39" si="77">SUM(G34:G38)</f>
         <v>118380</v>
       </c>
       <c r="H39" s="51">
-        <f t="shared" ref="H39" si="72">SUM(H34:H38)</f>
+        <f t="shared" ref="H39" si="78">SUM(H34:H38)</f>
         <v>115644</v>
       </c>
       <c r="I39" s="51">
-        <f t="shared" ref="I39" si="73">SUM(I34:I38)</f>
+        <f t="shared" ref="I39" si="79">SUM(I34:I38)</f>
         <v>208781</v>
       </c>
       <c r="J39" s="118">
-        <f t="shared" ref="J39" si="74">SUM(J34:J38)</f>
+        <f t="shared" ref="J39" si="80">SUM(J34:J38)</f>
         <v>6017171</v>
       </c>
       <c r="L39" s="109">
@@ -10048,19 +10048,19 @@
         <v>650543568</v>
       </c>
       <c r="M39" s="69">
-        <f t="shared" ref="M39" si="75">SUM(M34:M38)</f>
+        <f t="shared" ref="M39" si="81">SUM(M34:M38)</f>
         <v>578124392</v>
       </c>
       <c r="N39" s="69">
-        <f t="shared" ref="N39" si="76">SUM(N34:N38)</f>
+        <f t="shared" ref="N39" si="82">SUM(N34:N38)</f>
         <v>690157736</v>
       </c>
       <c r="O39" s="69">
-        <f t="shared" ref="O39" si="77">SUM(O34:O38)</f>
+        <f t="shared" ref="O39" si="83">SUM(O34:O38)</f>
         <v>654943915</v>
       </c>
       <c r="P39" s="69">
-        <f t="shared" ref="P39" si="78">SUM(P34:P38)</f>
+        <f t="shared" ref="P39" si="84">SUM(P34:P38)</f>
         <v>656247934</v>
       </c>
       <c r="Q39" s="115">
@@ -10072,27 +10072,27 @@
         <v>121665</v>
       </c>
       <c r="T39" s="40">
-        <f t="shared" ref="T39:Y39" si="79">SUM(T34:T38)</f>
+        <f t="shared" ref="T39:Y39" si="85">SUM(T34:T38)</f>
         <v>125620</v>
       </c>
       <c r="U39" s="40">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>32356</v>
       </c>
       <c r="V39" s="40">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>356297</v>
       </c>
       <c r="W39" s="40">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>122295</v>
       </c>
       <c r="X39" s="40">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>99994</v>
       </c>
       <c r="Y39" s="40">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>858227</v>
       </c>
       <c r="AA39" s="107">
@@ -10100,27 +10100,27 @@
         <v>121665</v>
       </c>
       <c r="AB39" s="67">
-        <f t="shared" ref="AB39" si="80">SUM(AB34:AB38)</f>
+        <f t="shared" ref="AB39" si="86">SUM(AB34:AB38)</f>
         <v>125620</v>
       </c>
       <c r="AC39" s="67">
-        <f t="shared" ref="AC39" si="81">SUM(AC34:AC38)</f>
+        <f t="shared" ref="AC39" si="87">SUM(AC34:AC38)</f>
         <v>32356</v>
       </c>
       <c r="AD39" s="67">
-        <f t="shared" ref="AD39" si="82">SUM(AD34:AD38)</f>
+        <f t="shared" ref="AD39" si="88">SUM(AD34:AD38)</f>
         <v>356297</v>
       </c>
       <c r="AE39" s="67">
-        <f t="shared" ref="AE39" si="83">SUM(AE34:AE38)</f>
+        <f t="shared" ref="AE39" si="89">SUM(AE34:AE38)</f>
         <v>122295</v>
       </c>
       <c r="AF39" s="67">
-        <f t="shared" ref="AF39" si="84">SUM(AF34:AF38)</f>
+        <f t="shared" ref="AF39" si="90">SUM(AF34:AF38)</f>
         <v>99994</v>
       </c>
       <c r="AG39" s="115">
-        <f t="shared" ref="AG39" si="85">SUM(AG34:AG38)</f>
+        <f t="shared" ref="AG39" si="91">SUM(AG34:AG38)</f>
         <v>858227</v>
       </c>
       <c r="AI39" s="95">
@@ -10128,23 +10128,23 @@
         <v>110109</v>
       </c>
       <c r="AJ39" s="51">
-        <f t="shared" ref="AJ39:AN39" si="86">SUM(AJ34:AJ38)</f>
+        <f t="shared" ref="AJ39:AN39" si="92">SUM(AJ34:AJ38)</f>
         <v>213260</v>
       </c>
       <c r="AK39" s="51">
-        <f t="shared" si="86"/>
+        <f t="shared" si="92"/>
         <v>116030</v>
       </c>
       <c r="AL39" s="51">
-        <f t="shared" si="86"/>
+        <f t="shared" si="92"/>
         <v>312792</v>
       </c>
       <c r="AM39" s="51">
-        <f t="shared" si="86"/>
+        <f t="shared" si="92"/>
         <v>106036</v>
       </c>
       <c r="AN39" s="118">
-        <f t="shared" si="86"/>
+        <f t="shared" si="92"/>
         <v>858227</v>
       </c>
       <c r="AP39" s="114">
@@ -10152,23 +10152,23 @@
         <v>646106962</v>
       </c>
       <c r="AQ39" s="49">
-        <f t="shared" ref="AQ39" si="87">SUM(AQ34:AQ38)</f>
+        <f t="shared" ref="AQ39" si="93">SUM(AQ34:AQ38)</f>
         <v>576804336</v>
       </c>
       <c r="AR39" s="49">
-        <f t="shared" ref="AR39" si="88">SUM(AR34:AR38)</f>
+        <f t="shared" ref="AR39" si="94">SUM(AR34:AR38)</f>
         <v>687706530</v>
       </c>
       <c r="AS39" s="49">
-        <f t="shared" ref="AS39" si="89">SUM(AS34:AS38)</f>
+        <f t="shared" ref="AS39" si="95">SUM(AS34:AS38)</f>
         <v>654677692</v>
       </c>
       <c r="AT39" s="49">
-        <f t="shared" ref="AT39" si="90">SUM(AT34:AT38)</f>
+        <f t="shared" ref="AT39" si="96">SUM(AT34:AT38)</f>
         <v>664722025</v>
       </c>
       <c r="AU39" s="119">
-        <f t="shared" ref="AU39" si="91">SUM(AU34:AU38)</f>
+        <f t="shared" ref="AU39" si="97">SUM(AU34:AU38)</f>
         <v>3230017545</v>
       </c>
     </row>

</xml_diff>

<commit_message>
implementacion funciones base de datos
</commit_message>
<xml_diff>
--- a/examples/DB_Supermercado.xlsx
+++ b/examples/DB_Supermercado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EducacionIT\Documents\office\Excel\xls-mj15\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A3AA43-0965-484F-88A4-DE87CEE6109D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6231D298-2DDF-4F12-898F-084AB5DE28D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -439,7 +439,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -575,15 +575,14 @@
     <xf numFmtId="44" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="10" fillId="3" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="10" fillId="5" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="10" fillId="5" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="10" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Énfasis5" xfId="3" builtinId="45"/>
@@ -6459,7 +6458,7 @@
         <f>SUMIF(ventas_producto,I$1,ventas_unidades)</f>
         <v>208781</v>
       </c>
-      <c r="J6" s="131">
+      <c r="J6" s="130">
         <f>SUM(E6:I6)</f>
         <v>858227</v>
       </c>
@@ -6483,7 +6482,7 @@
         <f>SUMIF(ventas_producto,P$1,ventas_total)</f>
         <v>656247934</v>
       </c>
-      <c r="Q6" s="132">
+      <c r="Q6" s="131">
         <f>SUM(L6:P6)</f>
         <v>3230017545</v>
       </c>
@@ -6511,8 +6510,11 @@
         <f t="shared" si="6"/>
         <v>99994</v>
       </c>
-      <c r="Y6" s="131"/>
-      <c r="Z6" s="133"/>
+      <c r="Y6" s="130">
+        <f>SUM(S6:X6)</f>
+        <v>858227</v>
+      </c>
+      <c r="Z6" s="132"/>
       <c r="AA6" s="99">
         <f t="shared" ref="AA6:AF6" si="7">SUMIF(ventas_vendedor,AA$1,ventas_total)</f>
         <v>645115066</v>
@@ -6537,7 +6539,10 @@
         <f t="shared" si="7"/>
         <v>561953724</v>
       </c>
-      <c r="AG6" s="132"/>
+      <c r="AG6" s="131">
+        <f>SUM(AA6:AF6)</f>
+        <v>3230017545</v>
+      </c>
       <c r="AI6" s="84">
         <f>SUMIF(ventas_region,AI$1,ventas_unidades)</f>
         <v>110109</v>
@@ -6558,7 +6563,10 @@
         <f>SUMIF(ventas_region,AM$1,ventas_unidades)</f>
         <v>106036</v>
       </c>
-      <c r="AN6" s="134"/>
+      <c r="AN6" s="134">
+        <f>SUM(AI6:AM6)</f>
+        <v>858227</v>
+      </c>
       <c r="AP6" s="99">
         <f>SUMIF(ventas_region,AP$1,ventas_total)</f>
         <v>646106962</v>
@@ -6579,7 +6587,7 @@
         <f>SUMIF(ventas_region,AT$1,ventas_total)</f>
         <v>664722025</v>
       </c>
-      <c r="AU6" s="135">
+      <c r="AU6" s="133">
         <f>SUM(AP6:AT6)</f>
         <v>3230017545</v>
       </c>
@@ -6603,7 +6611,7 @@
         <f>SUMIF(ventas_año,BA$1,ventas_unidades)</f>
         <v>205284</v>
       </c>
-      <c r="BB6" s="130">
+      <c r="BB6" s="129">
         <f>SUM(AW6:BA6)</f>
         <v>858227</v>
       </c>
@@ -6627,7 +6635,7 @@
         <f>SUMIF(ventas_año,BH$1,ventas_total)</f>
         <v>11533854</v>
       </c>
-      <c r="BI6" s="135">
+      <c r="BI6" s="133">
         <f>SUM(BD6:BH6)</f>
         <v>3230017545</v>
       </c>
@@ -6902,23 +6910,23 @@
         <v>650543568</v>
       </c>
       <c r="AW9" s="81">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A9,ventas_año,AW$8)</f>
+        <f t="shared" ref="AW9:BA13" si="12">SUMIFS(ventas_unidades,ventas_producto,$A9,ventas_año,AW$8)</f>
         <v>33032</v>
       </c>
       <c r="AX9" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A9,ventas_año,AX$8)</f>
+        <f t="shared" si="12"/>
         <v>32671</v>
       </c>
       <c r="AY9" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A9,ventas_año,AY$8)</f>
+        <f t="shared" si="12"/>
         <v>35334</v>
       </c>
       <c r="AZ9" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A9,ventas_año,AZ$8)</f>
+        <f t="shared" si="12"/>
         <v>2738</v>
       </c>
       <c r="BA9" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A9,ventas_año,BA$8)</f>
+        <f t="shared" si="12"/>
         <v>7128</v>
       </c>
       <c r="BB9" s="17">
@@ -6926,23 +6934,23 @@
         <v>110903</v>
       </c>
       <c r="BD9" s="96">
-        <f>SUMIFS(ventas_total,ventas_producto,$A9,ventas_año,BD$8)</f>
+        <f t="shared" ref="BD9:BH13" si="13">SUMIFS(ventas_total,ventas_producto,$A9,ventas_año,BD$8)</f>
         <v>218669111</v>
       </c>
       <c r="BE9" s="58">
-        <f>SUMIFS(ventas_total,ventas_producto,$A9,ventas_año,BE$8)</f>
+        <f t="shared" si="13"/>
         <v>203341463</v>
       </c>
       <c r="BF9" s="58">
-        <f>SUMIFS(ventas_total,ventas_producto,$A9,ventas_año,BF$8)</f>
+        <f t="shared" si="13"/>
         <v>218564244</v>
       </c>
       <c r="BG9" s="58">
-        <f>SUMIFS(ventas_total,ventas_producto,$A9,ventas_año,BG$8)</f>
+        <f t="shared" si="13"/>
         <v>844832</v>
       </c>
       <c r="BH9" s="58">
-        <f>SUMIFS(ventas_total,ventas_producto,$A9,ventas_año,BH$8)</f>
+        <f t="shared" si="13"/>
         <v>9123918</v>
       </c>
       <c r="BI9" s="58">
@@ -7000,7 +7008,7 @@
         <v>16505</v>
       </c>
       <c r="Y10" s="30">
-        <f t="shared" ref="Y10:Y13" si="12">SUM(S10:X10)</f>
+        <f t="shared" ref="Y10:Y13" si="14">SUM(S10:X10)</f>
         <v>304519</v>
       </c>
       <c r="AA10" s="104">
@@ -7028,7 +7036,7 @@
         <v>50806730</v>
       </c>
       <c r="AG10" s="64">
-        <f t="shared" ref="AG10:AG13" si="13">SUM(AA10:AF10)</f>
+        <f t="shared" ref="AG10:AG13" si="15">SUM(AA10:AF10)</f>
         <v>578124392</v>
       </c>
       <c r="AI10" s="82">
@@ -7052,7 +7060,7 @@
         <v>0</v>
       </c>
       <c r="AN10" s="46">
-        <f t="shared" ref="AN10:AN13" si="14">SUM(AI10:AM10)</f>
+        <f t="shared" ref="AN10:AN13" si="16">SUM(AI10:AM10)</f>
         <v>304519</v>
       </c>
       <c r="AP10" s="97">
@@ -7076,55 +7084,55 @@
         <v>0</v>
       </c>
       <c r="AU10" s="69">
-        <f t="shared" ref="AU10:AU13" si="15">SUM(AP10:AT10)</f>
+        <f t="shared" ref="AU10:AU13" si="17">SUM(AP10:AT10)</f>
         <v>578124392</v>
       </c>
       <c r="AW10" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A10,ventas_año,AW$8)</f>
+        <f t="shared" si="12"/>
         <v>32696</v>
       </c>
       <c r="AX10" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A10,ventas_año,AX$8)</f>
+        <f t="shared" si="12"/>
         <v>31651</v>
       </c>
       <c r="AY10" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A10,ventas_año,AY$8)</f>
+        <f t="shared" si="12"/>
         <v>40967</v>
       </c>
       <c r="AZ10" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A10,ventas_año,AZ$8)</f>
+        <f t="shared" si="12"/>
         <v>4903</v>
       </c>
       <c r="BA10" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A10,ventas_año,BA$8)</f>
+        <f t="shared" si="12"/>
         <v>194302</v>
       </c>
       <c r="BB10" s="46">
-        <f t="shared" ref="BB10:BB13" si="16">SUM(AW10:BA10)</f>
+        <f t="shared" ref="BB10:BB13" si="18">SUM(AW10:BA10)</f>
         <v>304519</v>
       </c>
       <c r="BD10" s="97">
-        <f>SUMIFS(ventas_total,ventas_producto,$A10,ventas_año,BD$8)</f>
+        <f t="shared" si="13"/>
         <v>160364763</v>
       </c>
       <c r="BE10" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A10,ventas_año,BE$8)</f>
+        <f t="shared" si="13"/>
         <v>201880917</v>
       </c>
       <c r="BF10" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A10,ventas_año,BF$8)</f>
+        <f t="shared" si="13"/>
         <v>214457221</v>
       </c>
       <c r="BG10" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A10,ventas_año,BG$8)</f>
+        <f t="shared" si="13"/>
         <v>483929</v>
       </c>
       <c r="BH10" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A10,ventas_año,BH$8)</f>
+        <f t="shared" si="13"/>
         <v>937562</v>
       </c>
       <c r="BI10" s="69">
-        <f t="shared" ref="BI10:BI13" si="17">SUM(BD10:BH10)</f>
+        <f t="shared" ref="BI10:BI13" si="19">SUM(BD10:BH10)</f>
         <v>578124392</v>
       </c>
     </row>
@@ -7178,7 +7186,7 @@
         <v>25030</v>
       </c>
       <c r="Y11" s="31">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>118380</v>
       </c>
       <c r="AA11" s="105">
@@ -7206,7 +7214,7 @@
         <v>167729464</v>
       </c>
       <c r="AG11" s="65">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>690157736</v>
       </c>
       <c r="AI11" s="83">
@@ -7230,7 +7238,7 @@
         <v>0</v>
       </c>
       <c r="AN11" s="47">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>118380</v>
       </c>
       <c r="AP11" s="98">
@@ -7254,55 +7262,55 @@
         <v>0</v>
       </c>
       <c r="AU11" s="70">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>690157736</v>
       </c>
       <c r="AW11" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A11,ventas_año,AW$8)</f>
+        <f t="shared" si="12"/>
         <v>39124</v>
       </c>
       <c r="AX11" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A11,ventas_año,AX$8)</f>
+        <f t="shared" si="12"/>
         <v>34000</v>
       </c>
       <c r="AY11" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A11,ventas_año,AY$8)</f>
+        <f t="shared" si="12"/>
         <v>31330</v>
       </c>
       <c r="AZ11" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A11,ventas_año,AZ$8)</f>
+        <f t="shared" si="12"/>
         <v>13926</v>
       </c>
       <c r="BA11" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A11,ventas_año,BA$8)</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="BB11" s="47">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>118380</v>
       </c>
       <c r="BD11" s="98">
-        <f>SUMIFS(ventas_total,ventas_producto,$A11,ventas_año,BD$8)</f>
+        <f t="shared" si="13"/>
         <v>220801841</v>
       </c>
       <c r="BE11" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A11,ventas_año,BE$8)</f>
+        <f t="shared" si="13"/>
         <v>239992813</v>
       </c>
       <c r="BF11" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A11,ventas_año,BF$8)</f>
+        <f t="shared" si="13"/>
         <v>216914467</v>
       </c>
       <c r="BG11" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A11,ventas_año,BG$8)</f>
+        <f t="shared" si="13"/>
         <v>12448615</v>
       </c>
       <c r="BH11" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A11,ventas_año,BH$8)</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="BI11" s="70">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>690157736</v>
       </c>
     </row>
@@ -7356,7 +7364,7 @@
         <v>5584</v>
       </c>
       <c r="Y12" s="30">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>115644</v>
       </c>
       <c r="AA12" s="104">
@@ -7384,7 +7392,7 @@
         <v>17788927</v>
       </c>
       <c r="AG12" s="64">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>654943915</v>
       </c>
       <c r="AI12" s="82">
@@ -7408,7 +7416,7 @@
         <v>0</v>
       </c>
       <c r="AN12" s="46">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>115644</v>
       </c>
       <c r="AP12" s="97">
@@ -7432,55 +7440,55 @@
         <v>0</v>
       </c>
       <c r="AU12" s="69">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>654943915</v>
       </c>
       <c r="AW12" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A12,ventas_año,AW$8)</f>
+        <f t="shared" si="12"/>
         <v>40573</v>
       </c>
       <c r="AX12" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A12,ventas_año,AX$8)</f>
+        <f t="shared" si="12"/>
         <v>39442</v>
       </c>
       <c r="AY12" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A12,ventas_año,AY$8)</f>
+        <f t="shared" si="12"/>
         <v>33573</v>
       </c>
       <c r="AZ12" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A12,ventas_año,AZ$8)</f>
+        <f t="shared" si="12"/>
         <v>129</v>
       </c>
       <c r="BA12" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A12,ventas_año,BA$8)</f>
+        <f t="shared" si="12"/>
         <v>1927</v>
       </c>
       <c r="BB12" s="46">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>115644</v>
       </c>
       <c r="BD12" s="97">
-        <f>SUMIFS(ventas_total,ventas_producto,$A12,ventas_año,BD$8)</f>
+        <f t="shared" si="13"/>
         <v>190929354</v>
       </c>
       <c r="BE12" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A12,ventas_año,BE$8)</f>
+        <f t="shared" si="13"/>
         <v>221383553</v>
       </c>
       <c r="BF12" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A12,ventas_año,BF$8)</f>
+        <f t="shared" si="13"/>
         <v>240503116</v>
       </c>
       <c r="BG12" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A12,ventas_año,BG$8)</f>
+        <f t="shared" si="13"/>
         <v>1203910</v>
       </c>
       <c r="BH12" s="69">
-        <f>SUMIFS(ventas_total,ventas_producto,$A12,ventas_año,BH$8)</f>
+        <f t="shared" si="13"/>
         <v>923982</v>
       </c>
       <c r="BI12" s="69">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>654943915</v>
       </c>
     </row>
@@ -7534,7 +7542,7 @@
         <v>41415</v>
       </c>
       <c r="Y13" s="31">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>208781</v>
       </c>
       <c r="AA13" s="105">
@@ -7562,7 +7570,7 @@
         <v>276189776</v>
       </c>
       <c r="AG13" s="65">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>656247934</v>
       </c>
       <c r="AI13" s="83">
@@ -7586,7 +7594,7 @@
         <v>98908</v>
       </c>
       <c r="AN13" s="47">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>208781</v>
       </c>
       <c r="AP13" s="98">
@@ -7610,55 +7618,55 @@
         <v>655598107</v>
       </c>
       <c r="AU13" s="70">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>656247934</v>
       </c>
       <c r="AW13" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A13,ventas_año,AW$8)</f>
+        <f t="shared" si="12"/>
         <v>36557</v>
       </c>
       <c r="AX13" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A13,ventas_año,AX$8)</f>
+        <f t="shared" si="12"/>
         <v>28900</v>
       </c>
       <c r="AY13" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A13,ventas_año,AY$8)</f>
+        <f t="shared" si="12"/>
         <v>33451</v>
       </c>
       <c r="AZ13" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A13,ventas_año,AZ$8)</f>
+        <f t="shared" si="12"/>
         <v>107946</v>
       </c>
       <c r="BA13" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_producto,$A13,ventas_año,BA$8)</f>
+        <f t="shared" si="12"/>
         <v>1927</v>
       </c>
       <c r="BB13" s="47">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>208781</v>
       </c>
       <c r="BD13" s="98">
-        <f>SUMIFS(ventas_total,ventas_producto,$A13,ventas_año,BD$8)</f>
+        <f t="shared" si="13"/>
         <v>216479082</v>
       </c>
       <c r="BE13" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A13,ventas_año,BE$8)</f>
+        <f t="shared" si="13"/>
         <v>240247726</v>
       </c>
       <c r="BF13" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A13,ventas_año,BF$8)</f>
+        <f t="shared" si="13"/>
         <v>198871299</v>
       </c>
       <c r="BG13" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A13,ventas_año,BG$8)</f>
+        <f t="shared" si="13"/>
         <v>101435</v>
       </c>
       <c r="BH13" s="70">
-        <f>SUMIFS(ventas_total,ventas_producto,$A13,ventas_año,BH$8)</f>
+        <f t="shared" si="13"/>
         <v>548392</v>
       </c>
       <c r="BI13" s="70">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>656247934</v>
       </c>
     </row>
@@ -7692,23 +7700,23 @@
         <v>121665</v>
       </c>
       <c r="T14" s="40">
-        <f t="shared" ref="T14:X14" si="18">SUM(T9:T13)</f>
+        <f t="shared" ref="T14:X14" si="20">SUM(T9:T13)</f>
         <v>125620</v>
       </c>
       <c r="U14" s="40">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>32356</v>
       </c>
       <c r="V14" s="40">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>356297</v>
       </c>
       <c r="W14" s="40">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>122295</v>
       </c>
       <c r="X14" s="40">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>99994</v>
       </c>
       <c r="Y14" s="117">
@@ -7720,47 +7728,47 @@
         <v>645115066</v>
       </c>
       <c r="AB14" s="66">
-        <f t="shared" ref="AB14" si="19">SUM(AB9:AB13)</f>
+        <f t="shared" ref="AB14" si="21">SUM(AB9:AB13)</f>
         <v>761464717</v>
       </c>
       <c r="AC14" s="66">
-        <f t="shared" ref="AC14" si="20">SUM(AC9:AC13)</f>
+        <f t="shared" ref="AC14" si="22">SUM(AC9:AC13)</f>
         <v>226722785</v>
       </c>
       <c r="AD14" s="66">
-        <f t="shared" ref="AD14" si="21">SUM(AD9:AD13)</f>
+        <f t="shared" ref="AD14" si="23">SUM(AD9:AD13)</f>
         <v>312257691</v>
       </c>
       <c r="AE14" s="66">
-        <f t="shared" ref="AE14" si="22">SUM(AE9:AE13)</f>
+        <f t="shared" ref="AE14" si="24">SUM(AE9:AE13)</f>
         <v>722503562</v>
       </c>
       <c r="AF14" s="66">
-        <f t="shared" ref="AF14" si="23">SUM(AF9:AF13)</f>
+        <f t="shared" ref="AF14" si="25">SUM(AF9:AF13)</f>
         <v>561953724</v>
       </c>
       <c r="AG14" s="114">
-        <f t="shared" ref="AG14" si="24">SUM(AG9:AG13)</f>
+        <f t="shared" ref="AG14" si="26">SUM(AG9:AG13)</f>
         <v>3230017545</v>
       </c>
       <c r="AI14" s="94">
-        <f t="shared" ref="AI14:AM14" si="25">SUM(AI10:AI13)</f>
+        <f t="shared" ref="AI14:AM14" si="27">SUM(AI10:AI13)</f>
         <v>9072</v>
       </c>
       <c r="AJ14" s="50">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>213260</v>
       </c>
       <c r="AK14" s="50">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>113292</v>
       </c>
       <c r="AL14" s="50">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>312792</v>
       </c>
       <c r="AM14" s="50">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>98908</v>
       </c>
       <c r="AN14" s="117">
@@ -7772,43 +7780,43 @@
         <v>646106962</v>
       </c>
       <c r="AQ14" s="68">
-        <f t="shared" ref="AQ14:AU14" si="26">SUM(AQ9:AQ13)</f>
+        <f t="shared" ref="AQ14:AU14" si="28">SUM(AQ9:AQ13)</f>
         <v>576804336</v>
       </c>
       <c r="AR14" s="68">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>687706530</v>
       </c>
       <c r="AS14" s="68">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>654677692</v>
       </c>
       <c r="AT14" s="68">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>664722025</v>
       </c>
       <c r="AU14" s="114">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>3230017545</v>
       </c>
       <c r="AW14" s="94">
-        <f t="shared" ref="AW14:BA14" si="27">SUM(AW10:AW13)</f>
+        <f t="shared" ref="AW14:BA14" si="29">SUM(AW10:AW13)</f>
         <v>148950</v>
       </c>
       <c r="AX14" s="50">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>133993</v>
       </c>
       <c r="AY14" s="50">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>139321</v>
       </c>
       <c r="AZ14" s="50">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>126904</v>
       </c>
       <c r="BA14" s="50">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>198156</v>
       </c>
       <c r="BB14" s="117">
@@ -7820,23 +7828,23 @@
         <v>1007244151</v>
       </c>
       <c r="BE14" s="68">
-        <f t="shared" ref="BE14:BI14" si="28">SUM(BE9:BE13)</f>
+        <f t="shared" ref="BE14:BI14" si="30">SUM(BE9:BE13)</f>
         <v>1106846472</v>
       </c>
       <c r="BF14" s="68">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>1089310347</v>
       </c>
       <c r="BG14" s="68">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>15082721</v>
       </c>
       <c r="BH14" s="68">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>11533854</v>
       </c>
       <c r="BI14" s="114">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>3230017545</v>
       </c>
     </row>
@@ -7980,31 +7988,31 @@
         <v>28</v>
       </c>
       <c r="B17" s="29">
-        <f t="shared" ref="B17:B22" si="29">SUMIF(ventas_vendedor,$A17,ventas_unidades)</f>
+        <f t="shared" ref="B17:B22" si="31">SUMIF(ventas_vendedor,$A17,ventas_unidades)</f>
         <v>121665</v>
       </c>
       <c r="C17" s="37">
-        <f t="shared" ref="C17:C22" si="30">SUMIF(ventas_vendedor,$A17,ventas_total)</f>
+        <f t="shared" ref="C17:C22" si="32">SUMIF(ventas_vendedor,$A17,ventas_total)</f>
         <v>645115066</v>
       </c>
       <c r="E17" s="81">
-        <f t="shared" ref="E17:I22" si="31">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,E$16)</f>
+        <f t="shared" ref="E17:I22" si="33">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_producto,E$16)</f>
         <v>23075</v>
       </c>
       <c r="F17" s="17">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>14026</v>
       </c>
       <c r="G17" s="17">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>37242</v>
       </c>
       <c r="H17" s="17">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>34352</v>
       </c>
       <c r="I17" s="17">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>12970</v>
       </c>
       <c r="J17" s="17">
@@ -8012,23 +8020,23 @@
         <v>121665</v>
       </c>
       <c r="L17" s="96">
-        <f t="shared" ref="L17:P22" si="32">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,L$16)</f>
+        <f t="shared" ref="L17:P22" si="34">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_producto,L$16)</f>
         <v>109144041</v>
       </c>
       <c r="M17" s="58">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>53223672</v>
       </c>
       <c r="N17" s="58">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>240818885</v>
       </c>
       <c r="O17" s="58">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>169977929</v>
       </c>
       <c r="P17" s="58">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>71950539</v>
       </c>
       <c r="Q17" s="58">
@@ -8050,23 +8058,23 @@
       <c r="AF17" s="67"/>
       <c r="AG17" s="67"/>
       <c r="AI17" s="81">
-        <f t="shared" ref="AI17:AM22" si="33">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_region,AI$16)</f>
+        <f t="shared" ref="AI17:AM22" si="35">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_region,AI$16)</f>
         <v>23075</v>
       </c>
       <c r="AJ17" s="17">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>7195</v>
       </c>
       <c r="AK17" s="17">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>39170</v>
       </c>
       <c r="AL17" s="17">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>39255</v>
       </c>
       <c r="AM17" s="17">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>12970</v>
       </c>
       <c r="AN17" s="17">
@@ -8074,23 +8082,23 @@
         <v>121665</v>
       </c>
       <c r="AP17" s="96">
-        <f t="shared" ref="AP17:AT22" si="34">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_region,AP$16)</f>
+        <f t="shared" ref="AP17:AT22" si="36">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_region,AP$16)</f>
         <v>109144041</v>
       </c>
       <c r="AQ17" s="58">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>52631529</v>
       </c>
       <c r="AR17" s="58">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>240927099</v>
       </c>
       <c r="AS17" s="58">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>170461858</v>
       </c>
       <c r="AT17" s="58">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>71950539</v>
       </c>
       <c r="AU17" s="58">
@@ -8098,23 +8106,23 @@
         <v>645115066</v>
       </c>
       <c r="AW17" s="81">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_año,AW$16)</f>
+        <f t="shared" ref="AW17:BA22" si="37">SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_año,AW$16)</f>
         <v>33623</v>
       </c>
       <c r="AX17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_año,AX$16)</f>
+        <f t="shared" si="37"/>
         <v>42339</v>
       </c>
       <c r="AY17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_año,AY$16)</f>
+        <f t="shared" si="37"/>
         <v>33889</v>
       </c>
       <c r="AZ17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_año,AZ$16)</f>
+        <f t="shared" si="37"/>
         <v>9886</v>
       </c>
       <c r="BA17" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A17,ventas_año,BA$16)</f>
+        <f t="shared" si="37"/>
         <v>1928</v>
       </c>
       <c r="BB17" s="17">
@@ -8122,23 +8130,23 @@
         <v>121665</v>
       </c>
       <c r="BD17" s="96">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_año,BD$8)</f>
+        <f t="shared" ref="BD17:BH22" si="38">SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_año,BD$8)</f>
         <v>175048265</v>
       </c>
       <c r="BE17" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_año,BE$8)</f>
+        <f t="shared" si="38"/>
         <v>244791087</v>
       </c>
       <c r="BF17" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_año,BF$8)</f>
+        <f t="shared" si="38"/>
         <v>216563190</v>
       </c>
       <c r="BG17" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_año,BG$8)</f>
+        <f t="shared" si="38"/>
         <v>8604310</v>
       </c>
       <c r="BH17" s="58">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A17,ventas_año,BH$8)</f>
+        <f t="shared" si="38"/>
         <v>108214</v>
       </c>
       <c r="BI17" s="58">
@@ -8151,59 +8159,59 @@
         <v>8</v>
       </c>
       <c r="B18" s="30">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>125620</v>
       </c>
       <c r="C18" s="38">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>761464717</v>
       </c>
       <c r="E18" s="82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>27346</v>
       </c>
       <c r="F18" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>51553</v>
       </c>
       <c r="G18" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>19565</v>
       </c>
       <c r="H18" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>12991</v>
       </c>
       <c r="I18" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>14165</v>
       </c>
       <c r="J18" s="18">
-        <f t="shared" ref="J18:J22" si="35">SUM(E18:I18)</f>
+        <f t="shared" ref="J18:J22" si="39">SUM(E18:I18)</f>
         <v>125620</v>
       </c>
       <c r="L18" s="97">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>193222871</v>
       </c>
       <c r="M18" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>271532147</v>
       </c>
       <c r="N18" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>131950052</v>
       </c>
       <c r="O18" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>75839132</v>
       </c>
       <c r="P18" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>88920515</v>
       </c>
       <c r="Q18" s="59">
-        <f t="shared" ref="Q18:Q22" si="36">SUM(L18:P18)</f>
+        <f t="shared" ref="Q18:Q22" si="40">SUM(L18:P18)</f>
         <v>761464717</v>
       </c>
       <c r="S18" s="93"/>
@@ -8221,99 +8229,99 @@
       <c r="AF18" s="67"/>
       <c r="AG18" s="67"/>
       <c r="AI18" s="82">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>27346</v>
       </c>
       <c r="AJ18" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>51553</v>
       </c>
       <c r="AK18" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>19565</v>
       </c>
       <c r="AL18" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>12991</v>
       </c>
       <c r="AM18" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>14165</v>
       </c>
       <c r="AN18" s="18">
-        <f t="shared" ref="AN18:AN22" si="37">SUM(AI18:AM18)</f>
+        <f t="shared" ref="AN18:AN22" si="41">SUM(AI18:AM18)</f>
         <v>125620</v>
       </c>
       <c r="AP18" s="97">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>193222871</v>
       </c>
       <c r="AQ18" s="59">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>271532147</v>
       </c>
       <c r="AR18" s="59">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>131950052</v>
       </c>
       <c r="AS18" s="59">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>75839132</v>
       </c>
       <c r="AT18" s="59">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>88920515</v>
       </c>
       <c r="AU18" s="59">
-        <f t="shared" ref="AU18:AU22" si="38">SUM(AP18:AT18)</f>
+        <f t="shared" ref="AU18:AU22" si="42">SUM(AP18:AT18)</f>
         <v>761464717</v>
       </c>
       <c r="AW18" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_año,AW$16)</f>
+        <f t="shared" si="37"/>
         <v>45235</v>
       </c>
       <c r="AX18" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_año,AX$16)</f>
+        <f t="shared" si="37"/>
         <v>39435</v>
       </c>
       <c r="AY18" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_año,AY$16)</f>
+        <f t="shared" si="37"/>
         <v>40950</v>
       </c>
       <c r="AZ18" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_año,AZ$16)</f>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="BA18" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A18,ventas_año,BA$16)</f>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="BB18" s="46">
-        <f t="shared" ref="BB18:BB21" si="39">SUM(AW18:BA18)</f>
+        <f t="shared" ref="BB18:BB21" si="43">SUM(AW18:BA18)</f>
         <v>125620</v>
       </c>
       <c r="BD18" s="97">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_año,BD$8)</f>
+        <f t="shared" si="38"/>
         <v>275531995</v>
       </c>
       <c r="BE18" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_año,BE$8)</f>
+        <f t="shared" si="38"/>
         <v>271002529</v>
       </c>
       <c r="BF18" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_año,BF$8)</f>
+        <f t="shared" si="38"/>
         <v>214930193</v>
       </c>
       <c r="BG18" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_año,BG$8)</f>
+        <f t="shared" si="38"/>
         <v>0</v>
       </c>
       <c r="BH18" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A18,ventas_año,BH$8)</f>
+        <f t="shared" si="38"/>
         <v>0</v>
       </c>
       <c r="BI18" s="69">
-        <f t="shared" ref="BI18:BI21" si="40">SUM(BD18:BH18)</f>
+        <f t="shared" ref="BI18:BI21" si="44">SUM(BD18:BH18)</f>
         <v>761464717</v>
       </c>
     </row>
@@ -8322,59 +8330,59 @@
         <v>11</v>
       </c>
       <c r="B19" s="31">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>32356</v>
       </c>
       <c r="C19" s="39">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>226722785</v>
       </c>
       <c r="E19" s="83">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>9125</v>
       </c>
       <c r="F19" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>9023</v>
       </c>
       <c r="G19" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>6969</v>
       </c>
       <c r="H19" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>2096</v>
       </c>
       <c r="I19" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>5143</v>
       </c>
       <c r="J19" s="19">
-        <f t="shared" si="35"/>
+        <f t="shared" si="39"/>
         <v>32356</v>
       </c>
       <c r="L19" s="98">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>59797810</v>
       </c>
       <c r="M19" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>63246530</v>
       </c>
       <c r="N19" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>40433106</v>
       </c>
       <c r="O19" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>31378227</v>
       </c>
       <c r="P19" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>31867112</v>
       </c>
       <c r="Q19" s="60">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>226722785</v>
       </c>
       <c r="S19" s="93"/>
@@ -8392,99 +8400,99 @@
       <c r="AF19" s="67"/>
       <c r="AG19" s="67"/>
       <c r="AI19" s="83">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>9125</v>
       </c>
       <c r="AJ19" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>9023</v>
       </c>
       <c r="AK19" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>6969</v>
       </c>
       <c r="AL19" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>2096</v>
       </c>
       <c r="AM19" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>5143</v>
       </c>
       <c r="AN19" s="19">
+        <f t="shared" si="41"/>
+        <v>32356</v>
+      </c>
+      <c r="AP19" s="98">
+        <f t="shared" si="36"/>
+        <v>59797810</v>
+      </c>
+      <c r="AQ19" s="60">
+        <f t="shared" si="36"/>
+        <v>63246530</v>
+      </c>
+      <c r="AR19" s="60">
+        <f t="shared" si="36"/>
+        <v>40433106</v>
+      </c>
+      <c r="AS19" s="60">
+        <f t="shared" si="36"/>
+        <v>31378227</v>
+      </c>
+      <c r="AT19" s="60">
+        <f t="shared" si="36"/>
+        <v>31867112</v>
+      </c>
+      <c r="AU19" s="60">
+        <f t="shared" si="42"/>
+        <v>226722785</v>
+      </c>
+      <c r="AW19" s="83">
         <f t="shared" si="37"/>
+        <v>12423</v>
+      </c>
+      <c r="AX19" s="47">
+        <f t="shared" si="37"/>
+        <v>12194</v>
+      </c>
+      <c r="AY19" s="47">
+        <f t="shared" si="37"/>
+        <v>7739</v>
+      </c>
+      <c r="AZ19" s="47">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+      <c r="BA19" s="47">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+      <c r="BB19" s="47">
+        <f t="shared" si="43"/>
         <v>32356</v>
       </c>
-      <c r="AP19" s="98">
-        <f t="shared" si="34"/>
-        <v>59797810</v>
-      </c>
-      <c r="AQ19" s="60">
-        <f t="shared" si="34"/>
-        <v>63246530</v>
-      </c>
-      <c r="AR19" s="60">
-        <f t="shared" si="34"/>
-        <v>40433106</v>
-      </c>
-      <c r="AS19" s="60">
-        <f t="shared" si="34"/>
-        <v>31378227</v>
-      </c>
-      <c r="AT19" s="60">
-        <f t="shared" si="34"/>
-        <v>31867112</v>
-      </c>
-      <c r="AU19" s="60">
+      <c r="BD19" s="98">
         <f t="shared" si="38"/>
-        <v>226722785</v>
-      </c>
-      <c r="AW19" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_año,AW$16)</f>
-        <v>12423</v>
-      </c>
-      <c r="AX19" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_año,AX$16)</f>
-        <v>12194</v>
-      </c>
-      <c r="AY19" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_año,AY$16)</f>
-        <v>7739</v>
-      </c>
-      <c r="AZ19" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_año,AZ$16)</f>
+        <v>48322205</v>
+      </c>
+      <c r="BE19" s="70">
+        <f t="shared" si="38"/>
+        <v>131956162</v>
+      </c>
+      <c r="BF19" s="70">
+        <f t="shared" si="38"/>
+        <v>46444418</v>
+      </c>
+      <c r="BG19" s="70">
+        <f t="shared" si="38"/>
         <v>0</v>
       </c>
-      <c r="BA19" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A19,ventas_año,BA$16)</f>
+      <c r="BH19" s="70">
+        <f t="shared" si="38"/>
         <v>0</v>
       </c>
-      <c r="BB19" s="47">
-        <f t="shared" si="39"/>
-        <v>32356</v>
-      </c>
-      <c r="BD19" s="98">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_año,BD$8)</f>
-        <v>48322205</v>
-      </c>
-      <c r="BE19" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_año,BE$8)</f>
-        <v>131956162</v>
-      </c>
-      <c r="BF19" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_año,BF$8)</f>
-        <v>46444418</v>
-      </c>
-      <c r="BG19" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_año,BG$8)</f>
-        <v>0</v>
-      </c>
-      <c r="BH19" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A19,ventas_año,BH$8)</f>
-        <v>0</v>
-      </c>
       <c r="BI19" s="70">
-        <f t="shared" si="40"/>
+        <f t="shared" si="44"/>
         <v>226722785</v>
       </c>
     </row>
@@ -8493,59 +8501,59 @@
         <v>13</v>
       </c>
       <c r="B20" s="30">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>356297</v>
       </c>
       <c r="C20" s="38">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>312257691</v>
       </c>
       <c r="E20" s="82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>21722</v>
       </c>
       <c r="F20" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>197836</v>
       </c>
       <c r="G20" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>18868</v>
       </c>
       <c r="H20" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>5457</v>
       </c>
       <c r="I20" s="18">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>112414</v>
       </c>
       <c r="J20" s="18">
-        <f t="shared" si="35"/>
+        <f t="shared" si="39"/>
         <v>356297</v>
       </c>
       <c r="L20" s="97">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>135280108</v>
       </c>
       <c r="M20" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>45710704</v>
       </c>
       <c r="N20" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>31481567</v>
       </c>
       <c r="O20" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>23001252</v>
       </c>
       <c r="P20" s="59">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>76784060</v>
       </c>
       <c r="Q20" s="59">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>312257691</v>
       </c>
       <c r="S20" s="93"/>
@@ -8563,99 +8571,99 @@
       <c r="AF20" s="67"/>
       <c r="AG20" s="67"/>
       <c r="AI20" s="82">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>30665</v>
       </c>
       <c r="AJ20" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>103585</v>
       </c>
       <c r="AK20" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>9925</v>
       </c>
       <c r="AL20" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>197831</v>
       </c>
       <c r="AM20" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>14291</v>
       </c>
       <c r="AN20" s="18">
+        <f t="shared" si="41"/>
+        <v>356297</v>
+      </c>
+      <c r="AP20" s="97">
+        <f t="shared" si="36"/>
+        <v>139608342</v>
+      </c>
+      <c r="AQ20" s="59">
+        <f t="shared" si="36"/>
+        <v>44964557</v>
+      </c>
+      <c r="AR20" s="59">
+        <f t="shared" si="36"/>
+        <v>27153333</v>
+      </c>
+      <c r="AS20" s="59">
+        <f t="shared" si="36"/>
+        <v>23830600</v>
+      </c>
+      <c r="AT20" s="59">
+        <f t="shared" si="36"/>
+        <v>76700859</v>
+      </c>
+      <c r="AU20" s="59">
+        <f t="shared" si="42"/>
+        <v>312257691</v>
+      </c>
+      <c r="AW20" s="82">
         <f t="shared" si="37"/>
+        <v>20990</v>
+      </c>
+      <c r="AX20" s="46">
+        <f t="shared" si="37"/>
+        <v>11750</v>
+      </c>
+      <c r="AY20" s="46">
+        <f t="shared" si="37"/>
+        <v>24117</v>
+      </c>
+      <c r="AZ20" s="46">
+        <f t="shared" si="37"/>
+        <v>107066</v>
+      </c>
+      <c r="BA20" s="46">
+        <f t="shared" si="37"/>
+        <v>192374</v>
+      </c>
+      <c r="BB20" s="46">
+        <f t="shared" si="43"/>
         <v>356297</v>
       </c>
-      <c r="AP20" s="97">
-        <f t="shared" si="34"/>
-        <v>139608342</v>
-      </c>
-      <c r="AQ20" s="59">
-        <f t="shared" si="34"/>
-        <v>44964557</v>
-      </c>
-      <c r="AR20" s="59">
-        <f t="shared" si="34"/>
-        <v>27153333</v>
-      </c>
-      <c r="AS20" s="59">
-        <f t="shared" si="34"/>
-        <v>23830600</v>
-      </c>
-      <c r="AT20" s="59">
-        <f t="shared" si="34"/>
-        <v>76700859</v>
-      </c>
-      <c r="AU20" s="59">
+      <c r="BD20" s="97">
         <f t="shared" si="38"/>
-        <v>312257691</v>
-      </c>
-      <c r="AW20" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_año,AW$16)</f>
-        <v>20990</v>
-      </c>
-      <c r="AX20" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_año,AX$16)</f>
-        <v>11750</v>
-      </c>
-      <c r="AY20" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_año,AY$16)</f>
-        <v>24117</v>
-      </c>
-      <c r="AZ20" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_año,AZ$16)</f>
-        <v>107066</v>
-      </c>
-      <c r="BA20" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A20,ventas_año,BA$16)</f>
-        <v>192374</v>
-      </c>
-      <c r="BB20" s="46">
-        <f t="shared" si="39"/>
-        <v>356297</v>
-      </c>
-      <c r="BD20" s="97">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_año,BD$8)</f>
         <v>109777406</v>
       </c>
       <c r="BE20" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_año,BE$8)</f>
+        <f t="shared" si="38"/>
         <v>63876055</v>
       </c>
       <c r="BF20" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_año,BF$8)</f>
+        <f t="shared" si="38"/>
         <v>133363447</v>
       </c>
       <c r="BG20" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_año,BG$8)</f>
+        <f t="shared" si="38"/>
         <v>4411435</v>
       </c>
       <c r="BH20" s="69">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A20,ventas_año,BH$8)</f>
+        <f t="shared" si="38"/>
         <v>829348</v>
       </c>
       <c r="BI20" s="69">
-        <f t="shared" si="40"/>
+        <f t="shared" si="44"/>
         <v>312257691</v>
       </c>
     </row>
@@ -8664,59 +8672,59 @@
         <v>29</v>
       </c>
       <c r="B21" s="31">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>122295</v>
       </c>
       <c r="C21" s="39">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>722503562</v>
       </c>
       <c r="E21" s="83">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>18175</v>
       </c>
       <c r="F21" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>15576</v>
       </c>
       <c r="G21" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>10706</v>
       </c>
       <c r="H21" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>55164</v>
       </c>
       <c r="I21" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>22674</v>
       </c>
       <c r="J21" s="19">
-        <f t="shared" si="35"/>
+        <f t="shared" si="39"/>
         <v>122295</v>
       </c>
       <c r="L21" s="98">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>103659911</v>
       </c>
       <c r="M21" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>93604609</v>
       </c>
       <c r="N21" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>77744662</v>
       </c>
       <c r="O21" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>336958448</v>
       </c>
       <c r="P21" s="60">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>110535932</v>
       </c>
       <c r="Q21" s="60">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>722503562</v>
       </c>
       <c r="S21" s="93"/>
@@ -8734,99 +8742,99 @@
       <c r="AF21" s="67"/>
       <c r="AG21" s="67"/>
       <c r="AI21" s="83">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>11047</v>
       </c>
       <c r="AJ21" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>25399</v>
       </c>
       <c r="AK21" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>12633</v>
       </c>
       <c r="AL21" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>53237</v>
       </c>
       <c r="AM21" s="19">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>19979</v>
       </c>
       <c r="AN21" s="19">
+        <f t="shared" si="41"/>
+        <v>122295</v>
+      </c>
+      <c r="AP21" s="98">
+        <f t="shared" si="36"/>
+        <v>94535993</v>
+      </c>
+      <c r="AQ21" s="60">
+        <f t="shared" si="36"/>
+        <v>93622843</v>
+      </c>
+      <c r="AR21" s="60">
+        <f t="shared" si="36"/>
+        <v>78668644</v>
+      </c>
+      <c r="AS21" s="60">
+        <f t="shared" si="36"/>
+        <v>336034466</v>
+      </c>
+      <c r="AT21" s="60">
+        <f t="shared" si="36"/>
+        <v>119641616</v>
+      </c>
+      <c r="AU21" s="60">
+        <f t="shared" si="42"/>
+        <v>722503562</v>
+      </c>
+      <c r="AW21" s="83">
         <f t="shared" si="37"/>
+        <v>44558</v>
+      </c>
+      <c r="AX21" s="47">
+        <f t="shared" si="37"/>
+        <v>27319</v>
+      </c>
+      <c r="AY21" s="47">
+        <f t="shared" si="37"/>
+        <v>31540</v>
+      </c>
+      <c r="AZ21" s="47">
+        <f t="shared" si="37"/>
+        <v>9823</v>
+      </c>
+      <c r="BA21" s="47">
+        <f t="shared" si="37"/>
+        <v>9055</v>
+      </c>
+      <c r="BB21" s="47">
+        <f t="shared" si="43"/>
         <v>122295</v>
       </c>
-      <c r="AP21" s="98">
-        <f t="shared" si="34"/>
-        <v>94535993</v>
-      </c>
-      <c r="AQ21" s="60">
-        <f t="shared" si="34"/>
-        <v>93622843</v>
-      </c>
-      <c r="AR21" s="60">
-        <f t="shared" si="34"/>
-        <v>78668644</v>
-      </c>
-      <c r="AS21" s="60">
-        <f t="shared" si="34"/>
-        <v>336034466</v>
-      </c>
-      <c r="AT21" s="60">
-        <f t="shared" si="34"/>
-        <v>119641616</v>
-      </c>
-      <c r="AU21" s="60">
+      <c r="BD21" s="98">
         <f t="shared" si="38"/>
-        <v>722503562</v>
-      </c>
-      <c r="AW21" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_año,AW$16)</f>
-        <v>44558</v>
-      </c>
-      <c r="AX21" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_año,AX$16)</f>
-        <v>27319</v>
-      </c>
-      <c r="AY21" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_año,AY$16)</f>
-        <v>31540</v>
-      </c>
-      <c r="AZ21" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_año,AZ$16)</f>
-        <v>9823</v>
-      </c>
-      <c r="BA21" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A21,ventas_año,BA$16)</f>
-        <v>9055</v>
-      </c>
-      <c r="BB21" s="47">
-        <f t="shared" si="39"/>
-        <v>122295</v>
-      </c>
-      <c r="BD21" s="98">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_año,BD$8)</f>
         <v>223098228</v>
       </c>
       <c r="BE21" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_año,BE$8)</f>
+        <f t="shared" si="38"/>
         <v>217807965</v>
       </c>
       <c r="BF21" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_año,BF$8)</f>
+        <f t="shared" si="38"/>
         <v>271531235</v>
       </c>
       <c r="BG21" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_año,BG$8)</f>
+        <f t="shared" si="38"/>
         <v>18234</v>
       </c>
       <c r="BH21" s="70">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A21,ventas_año,BH$8)</f>
+        <f t="shared" si="38"/>
         <v>10047900</v>
       </c>
       <c r="BI21" s="70">
-        <f t="shared" si="40"/>
+        <f t="shared" si="44"/>
         <v>722503562</v>
       </c>
     </row>
@@ -8835,59 +8843,59 @@
         <v>30</v>
       </c>
       <c r="B22" s="30">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v>99994</v>
       </c>
       <c r="C22" s="38">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>561953724</v>
       </c>
       <c r="E22" s="87">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>11460</v>
       </c>
       <c r="F22" s="51">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>16505</v>
       </c>
       <c r="G22" s="51">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>25030</v>
       </c>
       <c r="H22" s="51">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>5584</v>
       </c>
       <c r="I22" s="51">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>41415</v>
       </c>
       <c r="J22" s="51">
-        <f t="shared" si="35"/>
+        <f t="shared" si="39"/>
         <v>99994</v>
       </c>
       <c r="L22" s="101">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>49438827</v>
       </c>
       <c r="M22" s="57">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>50806730</v>
       </c>
       <c r="N22" s="57">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>167729464</v>
       </c>
       <c r="O22" s="57">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>17788927</v>
       </c>
       <c r="P22" s="57">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>276189776</v>
       </c>
       <c r="Q22" s="57">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>561953724</v>
       </c>
       <c r="S22" s="93"/>
@@ -8905,100 +8913,99 @@
       <c r="AF22" s="67"/>
       <c r="AG22" s="67"/>
       <c r="AI22" s="82">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>8851</v>
       </c>
       <c r="AJ22" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>16505</v>
       </c>
       <c r="AK22" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>27768</v>
       </c>
       <c r="AL22" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>7382</v>
       </c>
       <c r="AM22" s="18">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>39488</v>
       </c>
       <c r="AN22" s="18">
+        <f t="shared" si="41"/>
+        <v>99994</v>
+      </c>
+      <c r="AP22" s="97">
+        <f t="shared" si="36"/>
+        <v>49797905</v>
+      </c>
+      <c r="AQ22" s="59">
+        <f t="shared" si="36"/>
+        <v>50806730</v>
+      </c>
+      <c r="AR22" s="59">
+        <f t="shared" si="36"/>
+        <v>168574296</v>
+      </c>
+      <c r="AS22" s="59">
+        <f t="shared" si="36"/>
+        <v>17133409</v>
+      </c>
+      <c r="AT22" s="59">
+        <f t="shared" si="36"/>
+        <v>275641384</v>
+      </c>
+      <c r="AU22" s="59">
+        <f t="shared" si="42"/>
+        <v>561953724</v>
+      </c>
+      <c r="AW22" s="126">
         <f t="shared" si="37"/>
+        <v>25153</v>
+      </c>
+      <c r="AX22" s="78">
+        <f t="shared" si="37"/>
+        <v>33627</v>
+      </c>
+      <c r="AY22" s="78">
+        <f t="shared" si="37"/>
+        <v>36420</v>
+      </c>
+      <c r="AZ22" s="78">
+        <f t="shared" si="37"/>
+        <v>2867</v>
+      </c>
+      <c r="BA22" s="78">
+        <f t="shared" si="37"/>
+        <v>1927</v>
+      </c>
+      <c r="BB22" s="78">
+        <f t="shared" ref="BB22" si="45">SUM(AW22:BA22)</f>
         <v>99994</v>
       </c>
-      <c r="AP22" s="97">
-        <f t="shared" si="34"/>
-        <v>49797905</v>
-      </c>
-      <c r="AQ22" s="59">
-        <f t="shared" si="34"/>
-        <v>50806730</v>
-      </c>
-      <c r="AR22" s="59">
-        <f t="shared" si="34"/>
-        <v>168574296</v>
-      </c>
-      <c r="AS22" s="59">
-        <f t="shared" si="34"/>
-        <v>17133409</v>
-      </c>
-      <c r="AT22" s="59">
-        <f t="shared" si="34"/>
-        <v>275641384</v>
-      </c>
-      <c r="AU22" s="59">
+      <c r="BD22" s="127">
         <f t="shared" si="38"/>
-        <v>561953724</v>
-      </c>
-      <c r="AW22" s="126">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_año,AW$16)</f>
-        <v>25153</v>
-      </c>
-      <c r="AX22" s="78">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_año,AX$16)</f>
-        <v>33627</v>
-      </c>
-      <c r="AY22" s="78">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_año,AY$16)</f>
-        <v>36420</v>
-      </c>
-      <c r="AZ22" s="78">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_año,AZ$16)</f>
-        <v>2867</v>
-      </c>
-      <c r="BA22" s="78">
-        <f>SUMIFS(ventas_unidades,ventas_vendedor,$A22,ventas_año,BA$16)</f>
-        <v>1927</v>
-      </c>
-      <c r="BB22" s="78">
-        <f t="shared" ref="BB22" si="41">SUM(AW22:BA22)</f>
-        <v>99994</v>
-      </c>
-      <c r="BC22" s="127"/>
-      <c r="BD22" s="128">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_año,BD$8)</f>
         <v>175466052</v>
       </c>
-      <c r="BE22" s="129">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_año,BE$8)</f>
+      <c r="BE22" s="128">
+        <f t="shared" si="38"/>
         <v>177412674</v>
       </c>
-      <c r="BF22" s="129">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_año,BF$8)</f>
+      <c r="BF22" s="128">
+        <f t="shared" si="38"/>
         <v>206477864</v>
       </c>
-      <c r="BG22" s="129">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_año,BG$8)</f>
+      <c r="BG22" s="128">
+        <f t="shared" si="38"/>
         <v>2048742</v>
       </c>
-      <c r="BH22" s="129">
-        <f>SUMIFS(ventas_total,ventas_vendedor,$A22,ventas_año,BH$8)</f>
+      <c r="BH22" s="128">
+        <f t="shared" si="38"/>
         <v>548392</v>
       </c>
-      <c r="BI22" s="129">
-        <f t="shared" ref="BI22" si="42">SUM(BD22:BH22)</f>
+      <c r="BI22" s="128">
+        <f t="shared" ref="BI22" si="46">SUM(BD22:BH22)</f>
         <v>561953724</v>
       </c>
     </row>
@@ -9019,23 +9026,23 @@
         <v>110903</v>
       </c>
       <c r="F23" s="50">
-        <f t="shared" ref="F23:J23" si="43">SUM(F17:F22)</f>
+        <f t="shared" ref="F23:J23" si="47">SUM(F17:F22)</f>
         <v>304519</v>
       </c>
       <c r="G23" s="50">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>118380</v>
       </c>
       <c r="H23" s="50">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>115644</v>
       </c>
       <c r="I23" s="50">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>208781</v>
       </c>
       <c r="J23" s="117">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>858227</v>
       </c>
       <c r="L23" s="108">
@@ -9043,23 +9050,23 @@
         <v>650543568</v>
       </c>
       <c r="M23" s="68">
-        <f t="shared" ref="M23:Q23" si="44">SUM(M17:M22)</f>
+        <f t="shared" ref="M23:Q23" si="48">SUM(M17:M22)</f>
         <v>578124392</v>
       </c>
       <c r="N23" s="68">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>690157736</v>
       </c>
       <c r="O23" s="68">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>654943915</v>
       </c>
       <c r="P23" s="68">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>656247934</v>
       </c>
       <c r="Q23" s="114">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>3230017545</v>
       </c>
       <c r="S23" s="93"/>
@@ -9081,23 +9088,23 @@
         <v>110109</v>
       </c>
       <c r="AJ23" s="50">
-        <f t="shared" ref="AJ23:AN23" si="45">SUM(AJ17:AJ22)</f>
+        <f t="shared" ref="AJ23:AN23" si="49">SUM(AJ17:AJ22)</f>
         <v>213260</v>
       </c>
       <c r="AK23" s="50">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>116030</v>
       </c>
       <c r="AL23" s="50">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>312792</v>
       </c>
       <c r="AM23" s="50">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>106036</v>
       </c>
       <c r="AN23" s="117">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>858227</v>
       </c>
       <c r="AP23" s="108">
@@ -9105,23 +9112,23 @@
         <v>646106962</v>
       </c>
       <c r="AQ23" s="68">
-        <f t="shared" ref="AQ23" si="46">SUM(AQ17:AQ22)</f>
+        <f t="shared" ref="AQ23" si="50">SUM(AQ17:AQ22)</f>
         <v>576804336</v>
       </c>
       <c r="AR23" s="68">
-        <f t="shared" ref="AR23" si="47">SUM(AR17:AR22)</f>
+        <f t="shared" ref="AR23" si="51">SUM(AR17:AR22)</f>
         <v>687706530</v>
       </c>
       <c r="AS23" s="68">
-        <f t="shared" ref="AS23" si="48">SUM(AS17:AS22)</f>
+        <f t="shared" ref="AS23" si="52">SUM(AS17:AS22)</f>
         <v>654677692</v>
       </c>
       <c r="AT23" s="68">
-        <f t="shared" ref="AT23" si="49">SUM(AT17:AT22)</f>
+        <f t="shared" ref="AT23" si="53">SUM(AT17:AT22)</f>
         <v>664722025</v>
       </c>
       <c r="AU23" s="114">
-        <f t="shared" ref="AU23" si="50">SUM(AU17:AU22)</f>
+        <f t="shared" ref="AU23" si="54">SUM(AU17:AU22)</f>
         <v>3230017545</v>
       </c>
       <c r="AW23" s="94">
@@ -9149,27 +9156,27 @@
         <v>758233</v>
       </c>
       <c r="BD23" s="108">
-        <f>SUM(BD17:BD21)</f>
+        <f t="shared" ref="BD23:BI23" si="55">SUM(BD17:BD21)</f>
         <v>831778099</v>
       </c>
       <c r="BE23" s="68">
-        <f>SUM(BE17:BE21)</f>
+        <f t="shared" si="55"/>
         <v>929433798</v>
       </c>
       <c r="BF23" s="68">
-        <f>SUM(BF17:BF21)</f>
+        <f t="shared" si="55"/>
         <v>882832483</v>
       </c>
       <c r="BG23" s="68">
-        <f>SUM(BG17:BG21)</f>
+        <f t="shared" si="55"/>
         <v>13033979</v>
       </c>
       <c r="BH23" s="68">
-        <f>SUM(BH17:BH21)</f>
+        <f t="shared" si="55"/>
         <v>10985462</v>
       </c>
       <c r="BI23" s="114">
-        <f>SUM(BI17:BI21)</f>
+        <f t="shared" si="55"/>
         <v>2668063821</v>
       </c>
     </row>
@@ -9325,47 +9332,47 @@
         <v>646106962</v>
       </c>
       <c r="E26" s="81">
-        <f t="shared" ref="E26:I30" si="51">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,E$25)</f>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,E$25)</f>
         <v>101037</v>
       </c>
       <c r="F26" s="17">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,F$25)</f>
         <v>0</v>
       </c>
       <c r="G26" s="17">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,G$25)</f>
         <v>8943</v>
       </c>
       <c r="H26" s="17">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,H$25)</f>
         <v>129</v>
       </c>
       <c r="I26" s="17">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,I$25)</f>
         <v>0</v>
       </c>
       <c r="J26" s="17">
-        <f>SUM(E26:I30)</f>
-        <v>858227</v>
+        <f>SUM(E26:I26)</f>
+        <v>110109</v>
       </c>
       <c r="L26" s="96">
-        <f t="shared" ref="L26:P30" si="52">SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,L$25)</f>
+        <f t="shared" ref="L26:P30" si="56">SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,L$25)</f>
         <v>640574818</v>
       </c>
       <c r="M26" s="58">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="N26" s="58">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>4328234</v>
       </c>
       <c r="O26" s="58">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>1203910</v>
       </c>
       <c r="P26" s="58">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="Q26" s="58">
@@ -9373,27 +9380,27 @@
         <v>646106962</v>
       </c>
       <c r="S26" s="81">
-        <f t="shared" ref="S26:X30" si="53">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_vendedor,S$25)</f>
+        <f t="shared" ref="S26:X30" si="57">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_vendedor,S$25)</f>
         <v>23075</v>
       </c>
       <c r="T26" s="29">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>27346</v>
       </c>
       <c r="U26" s="29">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>9125</v>
       </c>
       <c r="V26" s="17">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>30665</v>
       </c>
       <c r="W26" s="29">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>11047</v>
       </c>
       <c r="X26" s="29">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>8851</v>
       </c>
       <c r="Y26" s="17">
@@ -9401,27 +9408,27 @@
         <v>110109</v>
       </c>
       <c r="AA26" s="96">
-        <f t="shared" ref="AA26:AF30" si="54">SUMIFS(ventas_total,ventas_region,$A26,ventas_vendedor,AA$25)</f>
+        <f t="shared" ref="AA26:AF30" si="58">SUMIFS(ventas_total,ventas_region,$A26,ventas_vendedor,AA$25)</f>
         <v>109144041</v>
       </c>
       <c r="AB26" s="63">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>193222871</v>
       </c>
       <c r="AC26" s="63">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>59797810</v>
       </c>
       <c r="AD26" s="58">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>139608342</v>
       </c>
       <c r="AE26" s="63">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>94535993</v>
       </c>
       <c r="AF26" s="63">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>49797905</v>
       </c>
       <c r="AG26" s="58">
@@ -9441,23 +9448,23 @@
       <c r="AT26" s="49"/>
       <c r="AU26" s="49"/>
       <c r="AW26" s="81">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,AW$8)</f>
+        <f t="shared" ref="AW26:BA30" si="59">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,AW$8)</f>
         <v>33032</v>
       </c>
       <c r="AX26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,AX$8)</f>
+        <f t="shared" si="59"/>
         <v>32671</v>
       </c>
       <c r="AY26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,AY$8)</f>
+        <f t="shared" si="59"/>
         <v>35334</v>
       </c>
       <c r="AZ26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,AZ$8)</f>
+        <f t="shared" si="59"/>
         <v>9072</v>
       </c>
       <c r="BA26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,BA$8)</f>
+        <f t="shared" si="59"/>
         <v>0</v>
       </c>
       <c r="BB26" s="17">
@@ -9465,23 +9472,23 @@
         <v>110109</v>
       </c>
       <c r="BD26" s="96">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BD$8)</f>
+        <f t="shared" ref="BD26:BH30" si="60">SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BD$8)</f>
         <v>218669111</v>
       </c>
       <c r="BE26" s="58">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BE$8)</f>
+        <f t="shared" si="60"/>
         <v>203341463</v>
       </c>
       <c r="BF26" s="58">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BF$8)</f>
+        <f t="shared" si="60"/>
         <v>218564244</v>
       </c>
       <c r="BG26" s="58">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BG$8)</f>
+        <f t="shared" si="60"/>
         <v>5532144</v>
       </c>
       <c r="BH26" s="58">
-        <f>SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BH$8)</f>
+        <f t="shared" si="60"/>
         <v>0</v>
       </c>
       <c r="BI26" s="58">
@@ -9502,107 +9509,107 @@
         <v>576804336</v>
       </c>
       <c r="E27" s="82">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,E$25)</f>
         <v>0</v>
       </c>
       <c r="F27" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,F$25)</f>
         <v>105314</v>
       </c>
       <c r="G27" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,G$25)</f>
         <v>0</v>
       </c>
       <c r="H27" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,H$25)</f>
         <v>0</v>
       </c>
       <c r="I27" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,I$25)</f>
         <v>107946</v>
       </c>
       <c r="J27" s="18">
-        <f t="shared" ref="J27:J30" si="55">SUM(E27:I31)</f>
-        <v>1606345</v>
+        <f t="shared" ref="J27:J30" si="61">SUM(E27:I27)</f>
+        <v>213260</v>
       </c>
       <c r="L27" s="97">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="M27" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>576702901</v>
       </c>
       <c r="N27" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="O27" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="P27" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>101435</v>
       </c>
       <c r="Q27" s="59">
-        <f t="shared" ref="Q27:Q30" si="56">SUM(L27:P27)</f>
+        <f t="shared" ref="Q27:Q30" si="62">SUM(L27:P27)</f>
         <v>576804336</v>
       </c>
       <c r="S27" s="90">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>7195</v>
       </c>
       <c r="T27" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>51553</v>
       </c>
       <c r="U27" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>9023</v>
       </c>
       <c r="V27" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>103585</v>
       </c>
       <c r="W27" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>25399</v>
       </c>
       <c r="X27" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>16505</v>
       </c>
       <c r="Y27" s="30">
-        <f t="shared" ref="Y27:Y30" si="57">SUM(S27:X27)</f>
+        <f t="shared" ref="Y27:Y30" si="63">SUM(S27:X27)</f>
         <v>213260</v>
       </c>
       <c r="AA27" s="104">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>52631529</v>
       </c>
       <c r="AB27" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>271532147</v>
       </c>
       <c r="AC27" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>63246530</v>
       </c>
       <c r="AD27" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>44964557</v>
       </c>
       <c r="AE27" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>93622843</v>
       </c>
       <c r="AF27" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>50806730</v>
       </c>
       <c r="AG27" s="64">
-        <f t="shared" ref="AG27:AG30" si="58">SUM(AA27:AF27)</f>
+        <f t="shared" ref="AG27:AG30" si="64">SUM(AA27:AF27)</f>
         <v>576804336</v>
       </c>
       <c r="AI27" s="93"/>
@@ -9618,51 +9625,51 @@
       <c r="AT27" s="49"/>
       <c r="AU27" s="49"/>
       <c r="AW27" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_año,AW$8)</f>
+        <f t="shared" si="59"/>
         <v>32696</v>
       </c>
       <c r="AX27" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_año,AX$8)</f>
+        <f t="shared" si="59"/>
         <v>31651</v>
       </c>
       <c r="AY27" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_año,AY$8)</f>
+        <f t="shared" si="59"/>
         <v>40967</v>
       </c>
       <c r="AZ27" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_año,AZ$8)</f>
+        <f t="shared" si="59"/>
         <v>107946</v>
       </c>
       <c r="BA27" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_año,BA$8)</f>
+        <f t="shared" si="59"/>
         <v>0</v>
       </c>
       <c r="BB27" s="46">
-        <f t="shared" ref="BB27:BB30" si="59">SUM(AW27:BA27)</f>
+        <f t="shared" ref="BB27:BB30" si="65">SUM(AW27:BA27)</f>
         <v>213260</v>
       </c>
       <c r="BD27" s="97">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_año,BD$8)</f>
+        <f t="shared" si="60"/>
         <v>160364763</v>
       </c>
       <c r="BE27" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_año,BE$8)</f>
+        <f t="shared" si="60"/>
         <v>201880917</v>
       </c>
       <c r="BF27" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_año,BF$8)</f>
+        <f t="shared" si="60"/>
         <v>214457221</v>
       </c>
       <c r="BG27" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_año,BG$8)</f>
+        <f t="shared" si="60"/>
         <v>101435</v>
       </c>
       <c r="BH27" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A27,ventas_año,BH$8)</f>
+        <f t="shared" si="60"/>
         <v>0</v>
       </c>
       <c r="BI27" s="69">
-        <f t="shared" ref="BI27:BI30" si="60">SUM(BD27:BH27)</f>
+        <f t="shared" ref="BI27:BI30" si="66">SUM(BD27:BH27)</f>
         <v>576804336</v>
       </c>
     </row>
@@ -9679,107 +9686,107 @@
         <v>687706530</v>
       </c>
       <c r="E28" s="83">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,E$25)</f>
         <v>2738</v>
       </c>
       <c r="F28" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,F$25)</f>
         <v>1928</v>
       </c>
       <c r="G28" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,G$25)</f>
         <v>109437</v>
       </c>
       <c r="H28" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,H$25)</f>
         <v>1927</v>
       </c>
       <c r="I28" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,I$25)</f>
         <v>0</v>
       </c>
       <c r="J28" s="19">
-        <f t="shared" si="55"/>
-        <v>1393085</v>
+        <f t="shared" si="61"/>
+        <v>116030</v>
       </c>
       <c r="L28" s="98">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>844832</v>
       </c>
       <c r="M28" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>108214</v>
       </c>
       <c r="N28" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>685829502</v>
       </c>
       <c r="O28" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>923982</v>
       </c>
       <c r="P28" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="Q28" s="60">
-        <f t="shared" si="56"/>
+        <f t="shared" si="62"/>
         <v>687706530</v>
       </c>
       <c r="S28" s="91">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>39170</v>
       </c>
       <c r="T28" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>19565</v>
       </c>
       <c r="U28" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>6969</v>
       </c>
       <c r="V28" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>9925</v>
       </c>
       <c r="W28" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>12633</v>
       </c>
       <c r="X28" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>27768</v>
       </c>
       <c r="Y28" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="63"/>
         <v>116030</v>
       </c>
       <c r="AA28" s="105">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>240927099</v>
       </c>
       <c r="AB28" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>131950052</v>
       </c>
       <c r="AC28" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>40433106</v>
       </c>
       <c r="AD28" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>27153333</v>
       </c>
       <c r="AE28" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>78668644</v>
       </c>
       <c r="AF28" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>168574296</v>
       </c>
       <c r="AG28" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="64"/>
         <v>687706530</v>
       </c>
       <c r="AI28" s="93"/>
@@ -9795,51 +9802,51 @@
       <c r="AT28" s="49"/>
       <c r="AU28" s="49"/>
       <c r="AW28" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_año,AW$8)</f>
+        <f t="shared" si="59"/>
         <v>39124</v>
       </c>
       <c r="AX28" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_año,AX$8)</f>
+        <f t="shared" si="59"/>
         <v>34000</v>
       </c>
       <c r="AY28" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_año,AY$8)</f>
+        <f t="shared" si="59"/>
         <v>31330</v>
       </c>
       <c r="AZ28" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_año,AZ$8)</f>
+        <f t="shared" si="59"/>
         <v>7721</v>
       </c>
       <c r="BA28" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_año,BA$8)</f>
+        <f t="shared" si="59"/>
         <v>3855</v>
       </c>
       <c r="BB28" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="65"/>
         <v>116030</v>
       </c>
       <c r="BD28" s="98">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_año,BD$8)</f>
+        <f t="shared" si="60"/>
         <v>220801841</v>
       </c>
       <c r="BE28" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_año,BE$8)</f>
+        <f t="shared" si="60"/>
         <v>239992813</v>
       </c>
       <c r="BF28" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_año,BF$8)</f>
+        <f t="shared" si="60"/>
         <v>216914467</v>
       </c>
       <c r="BG28" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_año,BG$8)</f>
+        <f t="shared" si="60"/>
         <v>8965213</v>
       </c>
       <c r="BH28" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A28,ventas_año,BH$8)</f>
+        <f t="shared" si="60"/>
         <v>1032196</v>
       </c>
       <c r="BI28" s="70">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>687706530</v>
       </c>
     </row>
@@ -9856,107 +9863,107 @@
         <v>654677692</v>
       </c>
       <c r="E29" s="82">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,E$25)</f>
         <v>0</v>
       </c>
       <c r="F29" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,F$25)</f>
         <v>197277</v>
       </c>
       <c r="G29" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,G$25)</f>
         <v>0</v>
       </c>
       <c r="H29" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,H$25)</f>
         <v>113588</v>
       </c>
       <c r="I29" s="18">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,I$25)</f>
         <v>1927</v>
       </c>
       <c r="J29" s="18">
-        <f t="shared" si="55"/>
-        <v>1277055</v>
+        <f t="shared" si="61"/>
+        <v>312792</v>
       </c>
       <c r="L29" s="97">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="M29" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>1313277</v>
       </c>
       <c r="N29" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="O29" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>652816023</v>
       </c>
       <c r="P29" s="59">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>548392</v>
       </c>
       <c r="Q29" s="59">
-        <f t="shared" si="56"/>
+        <f t="shared" si="62"/>
         <v>654677692</v>
       </c>
       <c r="S29" s="90">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>39255</v>
       </c>
       <c r="T29" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>12991</v>
       </c>
       <c r="U29" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>2096</v>
       </c>
       <c r="V29" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>197831</v>
       </c>
       <c r="W29" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>53237</v>
       </c>
       <c r="X29" s="30">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>7382</v>
       </c>
       <c r="Y29" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="63"/>
         <v>312792</v>
       </c>
       <c r="AA29" s="104">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>170461858</v>
       </c>
       <c r="AB29" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>75839132</v>
       </c>
       <c r="AC29" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>31378227</v>
       </c>
       <c r="AD29" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>23830600</v>
       </c>
       <c r="AE29" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>336034466</v>
       </c>
       <c r="AF29" s="64">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>17133409</v>
       </c>
       <c r="AG29" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="64"/>
         <v>654677692</v>
       </c>
       <c r="AI29" s="93"/>
@@ -9972,51 +9979,51 @@
       <c r="AT29" s="49"/>
       <c r="AU29" s="49"/>
       <c r="AW29" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_año,AW$8)</f>
+        <f t="shared" si="59"/>
         <v>40573</v>
       </c>
       <c r="AX29" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_año,AX$8)</f>
+        <f t="shared" si="59"/>
         <v>39442</v>
       </c>
       <c r="AY29" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_año,AY$8)</f>
+        <f t="shared" si="59"/>
         <v>33573</v>
       </c>
       <c r="AZ29" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_año,AZ$8)</f>
+        <f t="shared" si="59"/>
         <v>4903</v>
       </c>
       <c r="BA29" s="46">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_año,BA$8)</f>
+        <f t="shared" si="59"/>
         <v>194301</v>
       </c>
       <c r="BB29" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="65"/>
         <v>312792</v>
       </c>
       <c r="BD29" s="97">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_año,BD$8)</f>
+        <f t="shared" si="60"/>
         <v>190929354</v>
       </c>
       <c r="BE29" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_año,BE$8)</f>
+        <f t="shared" si="60"/>
         <v>221383553</v>
       </c>
       <c r="BF29" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_año,BF$8)</f>
+        <f t="shared" si="60"/>
         <v>240503116</v>
       </c>
       <c r="BG29" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_año,BG$8)</f>
+        <f t="shared" si="60"/>
         <v>483929</v>
       </c>
       <c r="BH29" s="69">
-        <f>SUMIFS(ventas_total,ventas_region,$A29,ventas_año,BH$8)</f>
+        <f t="shared" si="60"/>
         <v>1377740</v>
       </c>
       <c r="BI29" s="69">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>654677692</v>
       </c>
     </row>
@@ -10033,107 +10040,107 @@
         <v>664722025</v>
       </c>
       <c r="E30" s="83">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,E$25)</f>
         <v>7128</v>
       </c>
       <c r="F30" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,F$25)</f>
         <v>0</v>
       </c>
       <c r="G30" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,G$25)</f>
         <v>0</v>
       </c>
       <c r="H30" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,H$25)</f>
         <v>0</v>
       </c>
       <c r="I30" s="19">
-        <f t="shared" si="51"/>
+        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,I$25)</f>
         <v>98908</v>
       </c>
       <c r="J30" s="19">
-        <f t="shared" si="55"/>
-        <v>1146245</v>
+        <f t="shared" si="61"/>
+        <v>106036</v>
       </c>
       <c r="L30" s="98">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>9123918</v>
       </c>
       <c r="M30" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="N30" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="O30" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="P30" s="60">
-        <f t="shared" si="52"/>
+        <f t="shared" si="56"/>
         <v>655598107</v>
       </c>
       <c r="Q30" s="60">
-        <f t="shared" si="56"/>
+        <f t="shared" si="62"/>
         <v>664722025</v>
       </c>
       <c r="S30" s="91">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>12970</v>
       </c>
       <c r="T30" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>14165</v>
       </c>
       <c r="U30" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>5143</v>
       </c>
       <c r="V30" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>14291</v>
       </c>
       <c r="W30" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>19979</v>
       </c>
       <c r="X30" s="31">
-        <f t="shared" si="53"/>
+        <f t="shared" si="57"/>
         <v>39488</v>
       </c>
       <c r="Y30" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="63"/>
         <v>106036</v>
       </c>
       <c r="AA30" s="105">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>71950539</v>
       </c>
       <c r="AB30" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>88920515</v>
       </c>
       <c r="AC30" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>31867112</v>
       </c>
       <c r="AD30" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>76700859</v>
       </c>
       <c r="AE30" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>119641616</v>
       </c>
       <c r="AF30" s="65">
-        <f t="shared" si="54"/>
+        <f t="shared" si="58"/>
         <v>275641384</v>
       </c>
       <c r="AG30" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="64"/>
         <v>664722025</v>
       </c>
       <c r="AI30" s="93"/>
@@ -10149,51 +10156,51 @@
       <c r="AT30" s="49"/>
       <c r="AU30" s="49"/>
       <c r="AW30" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_año,AW$8)</f>
+        <f t="shared" si="59"/>
         <v>36557</v>
       </c>
       <c r="AX30" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_año,AX$8)</f>
+        <f t="shared" si="59"/>
         <v>28900</v>
       </c>
       <c r="AY30" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_año,AY$8)</f>
+        <f t="shared" si="59"/>
         <v>33451</v>
       </c>
       <c r="AZ30" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_año,AZ$8)</f>
+        <f t="shared" si="59"/>
         <v>0</v>
       </c>
       <c r="BA30" s="47">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_año,BA$8)</f>
+        <f t="shared" si="59"/>
         <v>7128</v>
       </c>
       <c r="BB30" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="65"/>
         <v>106036</v>
       </c>
       <c r="BD30" s="98">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_año,BD$8)</f>
+        <f t="shared" si="60"/>
         <v>216479082</v>
       </c>
       <c r="BE30" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_año,BE$8)</f>
+        <f t="shared" si="60"/>
         <v>240247726</v>
       </c>
       <c r="BF30" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_año,BF$8)</f>
+        <f t="shared" si="60"/>
         <v>198871299</v>
       </c>
       <c r="BG30" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_año,BG$8)</f>
+        <f t="shared" si="60"/>
         <v>0</v>
       </c>
       <c r="BH30" s="70">
-        <f>SUMIFS(ventas_total,ventas_region,$A30,ventas_año,BH$8)</f>
+        <f t="shared" si="60"/>
         <v>9123918</v>
       </c>
       <c r="BI30" s="70">
-        <f t="shared" si="60"/>
+        <f t="shared" si="66"/>
         <v>664722025</v>
       </c>
     </row>
@@ -10214,47 +10221,47 @@
         <v>110903</v>
       </c>
       <c r="F31" s="50">
-        <f t="shared" ref="F31:J31" si="61">SUM(F26:F30)</f>
+        <f t="shared" ref="F31:J31" si="67">SUM(F26:F30)</f>
         <v>304519</v>
       </c>
       <c r="G31" s="50">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>118380</v>
       </c>
       <c r="H31" s="50">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>115644</v>
       </c>
       <c r="I31" s="50">
-        <f t="shared" si="61"/>
+        <f t="shared" si="67"/>
         <v>208781</v>
       </c>
       <c r="J31" s="117">
-        <f t="shared" si="61"/>
-        <v>6280957</v>
+        <f t="shared" si="67"/>
+        <v>858227</v>
       </c>
       <c r="L31" s="108">
         <f>SUM(L26:L30)</f>
         <v>650543568</v>
       </c>
       <c r="M31" s="68">
-        <f t="shared" ref="M31" si="62">SUM(M26:M30)</f>
+        <f t="shared" ref="M31" si="68">SUM(M26:M30)</f>
         <v>578124392</v>
       </c>
       <c r="N31" s="68">
-        <f t="shared" ref="N31" si="63">SUM(N26:N30)</f>
+        <f t="shared" ref="N31" si="69">SUM(N26:N30)</f>
         <v>690157736</v>
       </c>
       <c r="O31" s="68">
-        <f t="shared" ref="O31" si="64">SUM(O26:O30)</f>
+        <f t="shared" ref="O31" si="70">SUM(O26:O30)</f>
         <v>654943915</v>
       </c>
       <c r="P31" s="68">
-        <f t="shared" ref="P31" si="65">SUM(P26:P30)</f>
+        <f t="shared" ref="P31" si="71">SUM(P26:P30)</f>
         <v>656247934</v>
       </c>
       <c r="Q31" s="114">
-        <f t="shared" ref="Q31" si="66">SUM(Q26:Q30)</f>
+        <f t="shared" ref="Q31" si="72">SUM(Q26:Q30)</f>
         <v>3230017545</v>
       </c>
       <c r="S31" s="92">
@@ -10262,27 +10269,27 @@
         <v>121665</v>
       </c>
       <c r="T31" s="40">
-        <f t="shared" ref="T31:Y31" si="67">SUM(T26:T30)</f>
+        <f t="shared" ref="T31:Y31" si="73">SUM(T26:T30)</f>
         <v>125620</v>
       </c>
       <c r="U31" s="40">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>32356</v>
       </c>
       <c r="V31" s="40">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>356297</v>
       </c>
       <c r="W31" s="40">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>122295</v>
       </c>
       <c r="X31" s="40">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>99994</v>
       </c>
       <c r="Y31" s="40">
-        <f t="shared" si="67"/>
+        <f t="shared" si="73"/>
         <v>858227</v>
       </c>
       <c r="AA31" s="106">
@@ -10290,27 +10297,27 @@
         <v>645115066</v>
       </c>
       <c r="AB31" s="66">
-        <f t="shared" ref="AB31" si="68">SUM(AB26:AB30)</f>
+        <f t="shared" ref="AB31" si="74">SUM(AB26:AB30)</f>
         <v>761464717</v>
       </c>
       <c r="AC31" s="66">
-        <f t="shared" ref="AC31" si="69">SUM(AC26:AC30)</f>
+        <f t="shared" ref="AC31" si="75">SUM(AC26:AC30)</f>
         <v>226722785</v>
       </c>
       <c r="AD31" s="66">
-        <f t="shared" ref="AD31" si="70">SUM(AD26:AD30)</f>
+        <f t="shared" ref="AD31" si="76">SUM(AD26:AD30)</f>
         <v>312257691</v>
       </c>
       <c r="AE31" s="66">
-        <f t="shared" ref="AE31" si="71">SUM(AE26:AE30)</f>
+        <f t="shared" ref="AE31" si="77">SUM(AE26:AE30)</f>
         <v>722503562</v>
       </c>
       <c r="AF31" s="66">
-        <f t="shared" ref="AF31" si="72">SUM(AF26:AF30)</f>
+        <f t="shared" ref="AF31" si="78">SUM(AF26:AF30)</f>
         <v>561953724</v>
       </c>
       <c r="AG31" s="114">
-        <f t="shared" ref="AG31" si="73">SUM(AG26:AG30)</f>
+        <f t="shared" ref="AG31" si="79">SUM(AG26:AG30)</f>
         <v>3230017545</v>
       </c>
       <c r="AI31" s="93"/>
@@ -10326,23 +10333,23 @@
       <c r="AT31" s="49"/>
       <c r="AU31" s="49"/>
       <c r="AW31" s="94">
-        <f t="shared" ref="AW31:BA31" si="74">SUM(AW27:AW30)</f>
+        <f t="shared" ref="AW31:BA31" si="80">SUM(AW27:AW30)</f>
         <v>148950</v>
       </c>
       <c r="AX31" s="50">
-        <f t="shared" si="74"/>
+        <f t="shared" si="80"/>
         <v>133993</v>
       </c>
       <c r="AY31" s="50">
-        <f t="shared" si="74"/>
+        <f t="shared" si="80"/>
         <v>139321</v>
       </c>
       <c r="AZ31" s="50">
-        <f t="shared" si="74"/>
+        <f t="shared" si="80"/>
         <v>120570</v>
       </c>
       <c r="BA31" s="50">
-        <f t="shared" si="74"/>
+        <f t="shared" si="80"/>
         <v>205284</v>
       </c>
       <c r="BB31" s="117">
@@ -10354,23 +10361,23 @@
         <v>1007244151</v>
       </c>
       <c r="BE31" s="68">
-        <f t="shared" ref="BE31:BI31" si="75">SUM(BE26:BE30)</f>
+        <f t="shared" ref="BE31:BI31" si="81">SUM(BE26:BE30)</f>
         <v>1106846472</v>
       </c>
       <c r="BF31" s="68">
-        <f t="shared" si="75"/>
+        <f t="shared" si="81"/>
         <v>1089310347</v>
       </c>
       <c r="BG31" s="68">
-        <f t="shared" si="75"/>
+        <f t="shared" si="81"/>
         <v>15082721</v>
       </c>
       <c r="BH31" s="68">
-        <f t="shared" si="75"/>
+        <f t="shared" si="81"/>
         <v>11533854</v>
       </c>
       <c r="BI31" s="114">
-        <f t="shared" si="75"/>
+        <f t="shared" si="81"/>
         <v>3230017545</v>
       </c>
     </row>
@@ -10525,47 +10532,47 @@
         <v>1007244151</v>
       </c>
       <c r="E34" s="81">
-        <f t="shared" ref="E34:I38" si="76">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,E$25)</f>
+        <f t="shared" ref="E34:I38" si="82">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,E$25)</f>
         <v>33032</v>
       </c>
       <c r="F34" s="17">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>32696</v>
       </c>
       <c r="G34" s="17">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>39124</v>
       </c>
       <c r="H34" s="17">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>40573</v>
       </c>
       <c r="I34" s="17">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>36557</v>
       </c>
       <c r="J34" s="17">
-        <f>SUM(E34:I38)</f>
-        <v>858227</v>
+        <f>SUM(E34:I34)</f>
+        <v>181982</v>
       </c>
       <c r="L34" s="96">
-        <f t="shared" ref="L34:P38" si="77">SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,L$25)</f>
+        <f t="shared" ref="L34:P38" si="83">SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,L$25)</f>
         <v>218669111</v>
       </c>
       <c r="M34" s="58">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>160364763</v>
       </c>
       <c r="N34" s="58">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>220801841</v>
       </c>
       <c r="O34" s="58">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>190929354</v>
       </c>
       <c r="P34" s="58">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>216479082</v>
       </c>
       <c r="Q34" s="58">
@@ -10573,27 +10580,27 @@
         <v>1007244151</v>
       </c>
       <c r="S34" s="89">
-        <f t="shared" ref="S34:X38" si="78">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,S$33)</f>
+        <f t="shared" ref="S34:X38" si="84">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,S$33)</f>
         <v>33623</v>
       </c>
       <c r="T34" s="29">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>45235</v>
       </c>
       <c r="U34" s="29">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>12423</v>
       </c>
       <c r="V34" s="29">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>20990</v>
       </c>
       <c r="W34" s="29">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>44558</v>
       </c>
       <c r="X34" s="29">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>25153</v>
       </c>
       <c r="Y34" s="29">
@@ -10601,27 +10608,27 @@
         <v>181982</v>
       </c>
       <c r="AA34" s="103">
-        <f t="shared" ref="AA34:AF38" si="79">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,AA$33)</f>
+        <f t="shared" ref="AA34:AF38" si="85">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,AA$33)</f>
         <v>33623</v>
       </c>
       <c r="AB34" s="63">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>45235</v>
       </c>
       <c r="AC34" s="63">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>12423</v>
       </c>
       <c r="AD34" s="63">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>20990</v>
       </c>
       <c r="AE34" s="63">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>44558</v>
       </c>
       <c r="AF34" s="63">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>25153</v>
       </c>
       <c r="AG34" s="63">
@@ -10629,23 +10636,23 @@
         <v>181982</v>
       </c>
       <c r="AI34" s="81">
-        <f t="shared" ref="AI34:AM38" si="80">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_region,AI$33)</f>
+        <f t="shared" ref="AI34:AM38" si="86">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_region,AI$33)</f>
         <v>33032</v>
       </c>
       <c r="AJ34" s="17">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>32696</v>
       </c>
       <c r="AK34" s="17">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>39124</v>
       </c>
       <c r="AL34" s="17">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>40573</v>
       </c>
       <c r="AM34" s="17">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>36557</v>
       </c>
       <c r="AN34" s="17">
@@ -10653,23 +10660,23 @@
         <v>181982</v>
       </c>
       <c r="AP34" s="110">
-        <f t="shared" ref="AP34:AT38" si="81">SUMIFS(ventas_total,ventas_año,$A34,ventas_region,AP$33)</f>
+        <f t="shared" ref="AP34:AT38" si="87">SUMIFS(ventas_total,ventas_año,$A34,ventas_region,AP$33)</f>
         <v>218669111</v>
       </c>
       <c r="AQ34" s="41">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>160364763</v>
       </c>
       <c r="AR34" s="41">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>220801841</v>
       </c>
       <c r="AS34" s="41">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>190929354</v>
       </c>
       <c r="AT34" s="41">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>216479082</v>
       </c>
       <c r="AU34" s="41">
@@ -10702,155 +10709,155 @@
         <v>1106846472</v>
       </c>
       <c r="E35" s="82">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>32671</v>
       </c>
       <c r="F35" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>31651</v>
       </c>
       <c r="G35" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>34000</v>
       </c>
       <c r="H35" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>39442</v>
       </c>
       <c r="I35" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>28900</v>
       </c>
       <c r="J35" s="18">
-        <f t="shared" ref="J35:J38" si="82">SUM(E35:I39)</f>
-        <v>1534472</v>
+        <f t="shared" ref="J35:J38" si="88">SUM(E35:I35)</f>
+        <v>166664</v>
       </c>
       <c r="L35" s="97">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>203341463</v>
       </c>
       <c r="M35" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>201880917</v>
       </c>
       <c r="N35" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>239992813</v>
       </c>
       <c r="O35" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>221383553</v>
       </c>
       <c r="P35" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>240247726</v>
       </c>
       <c r="Q35" s="59">
-        <f t="shared" ref="Q35:Q38" si="83">SUM(L35:P35)</f>
+        <f t="shared" ref="Q35:Q38" si="89">SUM(L35:P35)</f>
         <v>1106846472</v>
       </c>
       <c r="S35" s="90">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>42339</v>
       </c>
       <c r="T35" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>39435</v>
       </c>
       <c r="U35" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>12194</v>
       </c>
       <c r="V35" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>11750</v>
       </c>
       <c r="W35" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>27319</v>
       </c>
       <c r="X35" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>33627</v>
       </c>
       <c r="Y35" s="30">
-        <f t="shared" ref="Y35:Y38" si="84">SUM(S35:X35)</f>
+        <f t="shared" ref="Y35:Y38" si="90">SUM(S35:X35)</f>
         <v>166664</v>
       </c>
       <c r="AA35" s="104">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>42339</v>
       </c>
       <c r="AB35" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>39435</v>
       </c>
       <c r="AC35" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>12194</v>
       </c>
       <c r="AD35" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>11750</v>
       </c>
       <c r="AE35" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>27319</v>
       </c>
       <c r="AF35" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>33627</v>
       </c>
       <c r="AG35" s="64">
-        <f t="shared" ref="AG35:AG38" si="85">SUM(AA35:AF35)</f>
+        <f t="shared" ref="AG35:AG38" si="91">SUM(AA35:AF35)</f>
         <v>166664</v>
       </c>
       <c r="AI35" s="82">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>32671</v>
       </c>
       <c r="AJ35" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>31651</v>
       </c>
       <c r="AK35" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>34000</v>
       </c>
       <c r="AL35" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>39442</v>
       </c>
       <c r="AM35" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>28900</v>
       </c>
       <c r="AN35" s="18">
-        <f t="shared" ref="AN35:AN38" si="86">SUM(AI35:AM35)</f>
+        <f t="shared" ref="AN35:AN38" si="92">SUM(AI35:AM35)</f>
         <v>166664</v>
       </c>
       <c r="AP35" s="111">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>203341463</v>
       </c>
       <c r="AQ35" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>201880917</v>
       </c>
       <c r="AR35" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>239992813</v>
       </c>
       <c r="AS35" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>221383553</v>
       </c>
       <c r="AT35" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>240247726</v>
       </c>
       <c r="AU35" s="44">
-        <f t="shared" ref="AU35:AU38" si="87">SUM(AP35:AT35)</f>
+        <f t="shared" ref="AU35:AU38" si="93">SUM(AP35:AT35)</f>
         <v>1106846472</v>
       </c>
       <c r="AW35" s="93"/>
@@ -10879,155 +10886,155 @@
         <v>1089310347</v>
       </c>
       <c r="E36" s="83">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>35334</v>
       </c>
       <c r="F36" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>40967</v>
       </c>
       <c r="G36" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>31330</v>
       </c>
       <c r="H36" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>33573</v>
       </c>
       <c r="I36" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>33451</v>
       </c>
       <c r="J36" s="19">
-        <f t="shared" si="82"/>
-        <v>1367808</v>
+        <f t="shared" si="88"/>
+        <v>174655</v>
       </c>
       <c r="L36" s="98">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>218564244</v>
       </c>
       <c r="M36" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>214457221</v>
       </c>
       <c r="N36" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>216914467</v>
       </c>
       <c r="O36" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>240503116</v>
       </c>
       <c r="P36" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>198871299</v>
       </c>
       <c r="Q36" s="60">
-        <f t="shared" si="83"/>
+        <f t="shared" si="89"/>
         <v>1089310347</v>
       </c>
       <c r="S36" s="91">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>33889</v>
       </c>
       <c r="T36" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>40950</v>
       </c>
       <c r="U36" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>7739</v>
       </c>
       <c r="V36" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>24117</v>
       </c>
       <c r="W36" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>31540</v>
       </c>
       <c r="X36" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>36420</v>
       </c>
       <c r="Y36" s="31">
-        <f t="shared" si="84"/>
+        <f t="shared" si="90"/>
         <v>174655</v>
       </c>
       <c r="AA36" s="105">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>33889</v>
       </c>
       <c r="AB36" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>40950</v>
       </c>
       <c r="AC36" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>7739</v>
       </c>
       <c r="AD36" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>24117</v>
       </c>
       <c r="AE36" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>31540</v>
       </c>
       <c r="AF36" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>36420</v>
       </c>
       <c r="AG36" s="65">
-        <f t="shared" si="85"/>
+        <f t="shared" si="91"/>
         <v>174655</v>
       </c>
       <c r="AI36" s="83">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>35334</v>
       </c>
       <c r="AJ36" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>40967</v>
       </c>
       <c r="AK36" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>31330</v>
       </c>
       <c r="AL36" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>33573</v>
       </c>
       <c r="AM36" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>33451</v>
       </c>
       <c r="AN36" s="19">
-        <f t="shared" si="86"/>
+        <f t="shared" si="92"/>
         <v>174655</v>
       </c>
       <c r="AP36" s="112">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>218564244</v>
       </c>
       <c r="AQ36" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>214457221</v>
       </c>
       <c r="AR36" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>216914467</v>
       </c>
       <c r="AS36" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>240503116</v>
       </c>
       <c r="AT36" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>198871299</v>
       </c>
       <c r="AU36" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="93"/>
         <v>1089310347</v>
       </c>
       <c r="AW36" s="93"/>
@@ -11056,155 +11063,155 @@
         <v>15082721</v>
       </c>
       <c r="E37" s="82">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>2738</v>
       </c>
       <c r="F37" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>4903</v>
       </c>
       <c r="G37" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>13926</v>
       </c>
       <c r="H37" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>129</v>
       </c>
       <c r="I37" s="18">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>107946</v>
       </c>
       <c r="J37" s="18">
-        <f t="shared" si="82"/>
-        <v>1193153</v>
+        <f t="shared" si="88"/>
+        <v>129642</v>
       </c>
       <c r="L37" s="97">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>844832</v>
       </c>
       <c r="M37" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>483929</v>
       </c>
       <c r="N37" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>12448615</v>
       </c>
       <c r="O37" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>1203910</v>
       </c>
       <c r="P37" s="59">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>101435</v>
       </c>
       <c r="Q37" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="89"/>
         <v>15082721</v>
       </c>
       <c r="S37" s="90">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>9886</v>
       </c>
       <c r="T37" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="U37" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="V37" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>107066</v>
       </c>
       <c r="W37" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>9823</v>
       </c>
       <c r="X37" s="30">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>2867</v>
       </c>
       <c r="Y37" s="30">
-        <f t="shared" si="84"/>
+        <f t="shared" si="90"/>
         <v>129642</v>
       </c>
       <c r="AA37" s="104">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>9886</v>
       </c>
       <c r="AB37" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>0</v>
       </c>
       <c r="AC37" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>0</v>
       </c>
       <c r="AD37" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>107066</v>
       </c>
       <c r="AE37" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>9823</v>
       </c>
       <c r="AF37" s="64">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>2867</v>
       </c>
       <c r="AG37" s="64">
-        <f t="shared" si="85"/>
+        <f t="shared" si="91"/>
         <v>129642</v>
       </c>
       <c r="AI37" s="82">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>9072</v>
       </c>
       <c r="AJ37" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>107946</v>
       </c>
       <c r="AK37" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>7721</v>
       </c>
       <c r="AL37" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>4903</v>
       </c>
       <c r="AM37" s="18">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>0</v>
       </c>
       <c r="AN37" s="18">
-        <f t="shared" si="86"/>
+        <f t="shared" si="92"/>
         <v>129642</v>
       </c>
       <c r="AP37" s="111">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>5532144</v>
       </c>
       <c r="AQ37" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>101435</v>
       </c>
       <c r="AR37" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>8965213</v>
       </c>
       <c r="AS37" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>483929</v>
       </c>
       <c r="AT37" s="44">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>0</v>
       </c>
       <c r="AU37" s="44">
-        <f t="shared" si="87"/>
+        <f t="shared" si="93"/>
         <v>15082721</v>
       </c>
       <c r="AW37" s="93"/>
@@ -11233,155 +11240,155 @@
         <v>11533854</v>
       </c>
       <c r="E38" s="83">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>7128</v>
       </c>
       <c r="F38" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>194302</v>
       </c>
       <c r="G38" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>0</v>
       </c>
       <c r="H38" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>1927</v>
       </c>
       <c r="I38" s="19">
-        <f t="shared" si="76"/>
+        <f t="shared" si="82"/>
         <v>1927</v>
       </c>
       <c r="J38" s="19">
-        <f t="shared" si="82"/>
-        <v>1063511</v>
+        <f t="shared" si="88"/>
+        <v>205284</v>
       </c>
       <c r="L38" s="98">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>9123918</v>
       </c>
       <c r="M38" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>937562</v>
       </c>
       <c r="N38" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>0</v>
       </c>
       <c r="O38" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>923982</v>
       </c>
       <c r="P38" s="60">
-        <f t="shared" si="77"/>
+        <f t="shared" si="83"/>
         <v>548392</v>
       </c>
       <c r="Q38" s="60">
-        <f t="shared" si="83"/>
+        <f t="shared" si="89"/>
         <v>11533854</v>
       </c>
       <c r="S38" s="91">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>1928</v>
       </c>
       <c r="T38" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="U38" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="V38" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>192374</v>
       </c>
       <c r="W38" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>9055</v>
       </c>
       <c r="X38" s="31">
-        <f t="shared" si="78"/>
+        <f t="shared" si="84"/>
         <v>1927</v>
       </c>
       <c r="Y38" s="31">
-        <f t="shared" si="84"/>
+        <f t="shared" si="90"/>
         <v>205284</v>
       </c>
       <c r="AA38" s="105">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>1928</v>
       </c>
       <c r="AB38" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>0</v>
       </c>
       <c r="AC38" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>0</v>
       </c>
       <c r="AD38" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>192374</v>
       </c>
       <c r="AE38" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>9055</v>
       </c>
       <c r="AF38" s="65">
-        <f t="shared" si="79"/>
+        <f t="shared" si="85"/>
         <v>1927</v>
       </c>
       <c r="AG38" s="65">
-        <f t="shared" si="85"/>
+        <f t="shared" si="91"/>
         <v>205284</v>
       </c>
       <c r="AI38" s="83">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>0</v>
       </c>
       <c r="AJ38" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>0</v>
       </c>
       <c r="AK38" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>3855</v>
       </c>
       <c r="AL38" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>194301</v>
       </c>
       <c r="AM38" s="19">
-        <f t="shared" si="80"/>
+        <f t="shared" si="86"/>
         <v>7128</v>
       </c>
       <c r="AN38" s="19">
-        <f t="shared" si="86"/>
+        <f t="shared" si="92"/>
         <v>205284</v>
       </c>
       <c r="AP38" s="112">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>0</v>
       </c>
       <c r="AQ38" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>0</v>
       </c>
       <c r="AR38" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>1032196</v>
       </c>
       <c r="AS38" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>1377740</v>
       </c>
       <c r="AT38" s="45">
-        <f t="shared" si="81"/>
+        <f t="shared" si="87"/>
         <v>9123918</v>
       </c>
       <c r="AU38" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="93"/>
         <v>11533854</v>
       </c>
       <c r="AW38" s="93"/>
@@ -11414,43 +11421,43 @@
         <v>110903</v>
       </c>
       <c r="F39" s="50">
-        <f t="shared" ref="F39" si="88">SUM(F34:F38)</f>
+        <f t="shared" ref="F39" si="94">SUM(F34:F38)</f>
         <v>304519</v>
       </c>
       <c r="G39" s="50">
-        <f t="shared" ref="G39" si="89">SUM(G34:G38)</f>
+        <f t="shared" ref="G39" si="95">SUM(G34:G38)</f>
         <v>118380</v>
       </c>
       <c r="H39" s="50">
-        <f t="shared" ref="H39" si="90">SUM(H34:H38)</f>
+        <f t="shared" ref="H39" si="96">SUM(H34:H38)</f>
         <v>115644</v>
       </c>
       <c r="I39" s="50">
-        <f t="shared" ref="I39" si="91">SUM(I34:I38)</f>
+        <f t="shared" ref="I39" si="97">SUM(I34:I38)</f>
         <v>208781</v>
       </c>
       <c r="J39" s="117">
-        <f t="shared" ref="J39" si="92">SUM(J34:J38)</f>
-        <v>6017171</v>
+        <f t="shared" ref="J39" si="98">SUM(J34:J38)</f>
+        <v>858227</v>
       </c>
       <c r="L39" s="108">
         <f>SUM(L34:L38)</f>
         <v>650543568</v>
       </c>
       <c r="M39" s="68">
-        <f t="shared" ref="M39" si="93">SUM(M34:M38)</f>
+        <f t="shared" ref="M39" si="99">SUM(M34:M38)</f>
         <v>578124392</v>
       </c>
       <c r="N39" s="68">
-        <f t="shared" ref="N39" si="94">SUM(N34:N38)</f>
+        <f t="shared" ref="N39" si="100">SUM(N34:N38)</f>
         <v>690157736</v>
       </c>
       <c r="O39" s="68">
-        <f t="shared" ref="O39" si="95">SUM(O34:O38)</f>
+        <f t="shared" ref="O39" si="101">SUM(O34:O38)</f>
         <v>654943915</v>
       </c>
       <c r="P39" s="68">
-        <f t="shared" ref="P39" si="96">SUM(P34:P38)</f>
+        <f t="shared" ref="P39" si="102">SUM(P34:P38)</f>
         <v>656247934</v>
       </c>
       <c r="Q39" s="114">
@@ -11462,27 +11469,27 @@
         <v>121665</v>
       </c>
       <c r="T39" s="40">
-        <f t="shared" ref="T39:Y39" si="97">SUM(T34:T38)</f>
+        <f t="shared" ref="T39:Y39" si="103">SUM(T34:T38)</f>
         <v>125620</v>
       </c>
       <c r="U39" s="40">
-        <f t="shared" si="97"/>
+        <f t="shared" si="103"/>
         <v>32356</v>
       </c>
       <c r="V39" s="40">
-        <f t="shared" si="97"/>
+        <f t="shared" si="103"/>
         <v>356297</v>
       </c>
       <c r="W39" s="40">
-        <f t="shared" si="97"/>
+        <f t="shared" si="103"/>
         <v>122295</v>
       </c>
       <c r="X39" s="40">
-        <f t="shared" si="97"/>
+        <f t="shared" si="103"/>
         <v>99994</v>
       </c>
       <c r="Y39" s="40">
-        <f t="shared" si="97"/>
+        <f t="shared" si="103"/>
         <v>858227</v>
       </c>
       <c r="AA39" s="106">
@@ -11490,27 +11497,27 @@
         <v>121665</v>
       </c>
       <c r="AB39" s="66">
-        <f t="shared" ref="AB39" si="98">SUM(AB34:AB38)</f>
+        <f t="shared" ref="AB39" si="104">SUM(AB34:AB38)</f>
         <v>125620</v>
       </c>
       <c r="AC39" s="66">
-        <f t="shared" ref="AC39" si="99">SUM(AC34:AC38)</f>
+        <f t="shared" ref="AC39" si="105">SUM(AC34:AC38)</f>
         <v>32356</v>
       </c>
       <c r="AD39" s="66">
-        <f t="shared" ref="AD39" si="100">SUM(AD34:AD38)</f>
+        <f t="shared" ref="AD39" si="106">SUM(AD34:AD38)</f>
         <v>356297</v>
       </c>
       <c r="AE39" s="66">
-        <f t="shared" ref="AE39" si="101">SUM(AE34:AE38)</f>
+        <f t="shared" ref="AE39" si="107">SUM(AE34:AE38)</f>
         <v>122295</v>
       </c>
       <c r="AF39" s="66">
-        <f t="shared" ref="AF39" si="102">SUM(AF34:AF38)</f>
+        <f t="shared" ref="AF39" si="108">SUM(AF34:AF38)</f>
         <v>99994</v>
       </c>
       <c r="AG39" s="114">
-        <f t="shared" ref="AG39" si="103">SUM(AG34:AG38)</f>
+        <f t="shared" ref="AG39" si="109">SUM(AG34:AG38)</f>
         <v>858227</v>
       </c>
       <c r="AI39" s="94">
@@ -11518,23 +11525,23 @@
         <v>110109</v>
       </c>
       <c r="AJ39" s="50">
-        <f t="shared" ref="AJ39:AN39" si="104">SUM(AJ34:AJ38)</f>
+        <f t="shared" ref="AJ39:AN39" si="110">SUM(AJ34:AJ38)</f>
         <v>213260</v>
       </c>
       <c r="AK39" s="50">
-        <f t="shared" si="104"/>
+        <f t="shared" si="110"/>
         <v>116030</v>
       </c>
       <c r="AL39" s="50">
-        <f t="shared" si="104"/>
+        <f t="shared" si="110"/>
         <v>312792</v>
       </c>
       <c r="AM39" s="50">
-        <f t="shared" si="104"/>
+        <f t="shared" si="110"/>
         <v>106036</v>
       </c>
       <c r="AN39" s="117">
-        <f t="shared" si="104"/>
+        <f t="shared" si="110"/>
         <v>858227</v>
       </c>
       <c r="AP39" s="113">
@@ -11542,23 +11549,23 @@
         <v>646106962</v>
       </c>
       <c r="AQ39" s="48">
-        <f t="shared" ref="AQ39" si="105">SUM(AQ34:AQ38)</f>
+        <f t="shared" ref="AQ39" si="111">SUM(AQ34:AQ38)</f>
         <v>576804336</v>
       </c>
       <c r="AR39" s="48">
-        <f t="shared" ref="AR39" si="106">SUM(AR34:AR38)</f>
+        <f t="shared" ref="AR39" si="112">SUM(AR34:AR38)</f>
         <v>687706530</v>
       </c>
       <c r="AS39" s="48">
-        <f t="shared" ref="AS39" si="107">SUM(AS34:AS38)</f>
+        <f t="shared" ref="AS39" si="113">SUM(AS34:AS38)</f>
         <v>654677692</v>
       </c>
       <c r="AT39" s="48">
-        <f t="shared" ref="AT39" si="108">SUM(AT34:AT38)</f>
+        <f t="shared" ref="AT39" si="114">SUM(AT34:AT38)</f>
         <v>664722025</v>
       </c>
       <c r="AU39" s="118">
-        <f t="shared" ref="AU39" si="109">SUM(AU34:AU38)</f>
+        <f t="shared" ref="AU39" si="115">SUM(AU34:AU38)</f>
         <v>3230017545</v>
       </c>
       <c r="AW39" s="93"/>

</xml_diff>

<commit_message>
funciones base de datos y busqueda
</commit_message>
<xml_diff>
--- a/examples/DB_Supermercado.xlsx
+++ b/examples/DB_Supermercado.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EducacionIT\Documents\office\Excel\xls-mj15\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6231D298-2DDF-4F12-898F-084AB5DE28D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B21AB4E-B473-4246-8337-6D7FFB61AAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ventas" sheetId="6" r:id="rId1"/>
     <sheet name="listas" sheetId="7" state="hidden" r:id="rId2"/>
     <sheet name="estadisticas" sheetId="8" r:id="rId3"/>
+    <sheet name="comisiones" sheetId="9" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ventas!$A:$G</definedName>
+    <definedName name="vendedores">estadisticas!$A$16:$C$23</definedName>
     <definedName name="ventas_año">ventas!$B:$B</definedName>
     <definedName name="ventas_producto">ventas!$C:$C</definedName>
     <definedName name="ventas_region">ventas!$G:$G</definedName>
@@ -64,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="57">
   <si>
     <t>Mes</t>
   </si>
@@ -211,6 +213,30 @@
   </si>
   <si>
     <t>UNIDADES</t>
+  </si>
+  <si>
+    <t>Comision</t>
+  </si>
+  <si>
+    <t>porcentaje</t>
+  </si>
+  <si>
+    <t>objetivo</t>
+  </si>
+  <si>
+    <t>valor</t>
+  </si>
+  <si>
+    <t>unidad</t>
+  </si>
+  <si>
+    <t>venta</t>
+  </si>
+  <si>
+    <t>cumple</t>
+  </si>
+  <si>
+    <t>Objetivos</t>
   </si>
 </sst>
 </file>
@@ -439,7 +465,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -583,6 +609,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="10" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="10" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Énfasis5" xfId="3" builtinId="45"/>
@@ -8497,7 +8526,7 @@
       </c>
     </row>
     <row r="20" spans="1:61" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="30">
@@ -9332,23 +9361,23 @@
         <v>646106962</v>
       </c>
       <c r="E26" s="81">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,E$25)</f>
+        <f t="shared" ref="E26:I30" si="56">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,E$25)</f>
         <v>101037</v>
       </c>
       <c r="F26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,F$25)</f>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="G26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,G$25)</f>
+        <f t="shared" si="56"/>
         <v>8943</v>
       </c>
       <c r="H26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,H$25)</f>
+        <f t="shared" si="56"/>
         <v>129</v>
       </c>
       <c r="I26" s="17">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A26,ventas_producto,I$25)</f>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="J26" s="17">
@@ -9356,23 +9385,23 @@
         <v>110109</v>
       </c>
       <c r="L26" s="96">
-        <f t="shared" ref="L26:P30" si="56">SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,L$25)</f>
+        <f t="shared" ref="L26:P30" si="57">SUMIFS(ventas_total,ventas_region,$A26,ventas_producto,L$25)</f>
         <v>640574818</v>
       </c>
       <c r="M26" s="58">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>0</v>
       </c>
       <c r="N26" s="58">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>4328234</v>
       </c>
       <c r="O26" s="58">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>1203910</v>
       </c>
       <c r="P26" s="58">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>0</v>
       </c>
       <c r="Q26" s="58">
@@ -9380,27 +9409,27 @@
         <v>646106962</v>
       </c>
       <c r="S26" s="81">
-        <f t="shared" ref="S26:X30" si="57">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_vendedor,S$25)</f>
+        <f t="shared" ref="S26:X30" si="58">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_vendedor,S$25)</f>
         <v>23075</v>
       </c>
       <c r="T26" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>27346</v>
       </c>
       <c r="U26" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>9125</v>
       </c>
       <c r="V26" s="17">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>30665</v>
       </c>
       <c r="W26" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>11047</v>
       </c>
       <c r="X26" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>8851</v>
       </c>
       <c r="Y26" s="17">
@@ -9408,27 +9437,27 @@
         <v>110109</v>
       </c>
       <c r="AA26" s="96">
-        <f t="shared" ref="AA26:AF30" si="58">SUMIFS(ventas_total,ventas_region,$A26,ventas_vendedor,AA$25)</f>
+        <f t="shared" ref="AA26:AF30" si="59">SUMIFS(ventas_total,ventas_region,$A26,ventas_vendedor,AA$25)</f>
         <v>109144041</v>
       </c>
       <c r="AB26" s="63">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>193222871</v>
       </c>
       <c r="AC26" s="63">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>59797810</v>
       </c>
       <c r="AD26" s="58">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>139608342</v>
       </c>
       <c r="AE26" s="63">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>94535993</v>
       </c>
       <c r="AF26" s="63">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>49797905</v>
       </c>
       <c r="AG26" s="58">
@@ -9448,23 +9477,23 @@
       <c r="AT26" s="49"/>
       <c r="AU26" s="49"/>
       <c r="AW26" s="81">
-        <f t="shared" ref="AW26:BA30" si="59">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,AW$8)</f>
+        <f t="shared" ref="AW26:BA30" si="60">SUMIFS(ventas_unidades,ventas_region,$A26,ventas_año,AW$8)</f>
         <v>33032</v>
       </c>
       <c r="AX26" s="17">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>32671</v>
       </c>
       <c r="AY26" s="17">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>35334</v>
       </c>
       <c r="AZ26" s="17">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>9072</v>
       </c>
       <c r="BA26" s="17">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>0</v>
       </c>
       <c r="BB26" s="17">
@@ -9472,23 +9501,23 @@
         <v>110109</v>
       </c>
       <c r="BD26" s="96">
-        <f t="shared" ref="BD26:BH30" si="60">SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BD$8)</f>
+        <f t="shared" ref="BD26:BH30" si="61">SUMIFS(ventas_total,ventas_region,$A26,ventas_año,BD$8)</f>
         <v>218669111</v>
       </c>
       <c r="BE26" s="58">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>203341463</v>
       </c>
       <c r="BF26" s="58">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>218564244</v>
       </c>
       <c r="BG26" s="58">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>5532144</v>
       </c>
       <c r="BH26" s="58">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>0</v>
       </c>
       <c r="BI26" s="58">
@@ -9509,107 +9538,107 @@
         <v>576804336</v>
       </c>
       <c r="E27" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,E$25)</f>
-        <v>0</v>
-      </c>
-      <c r="F27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,F$25)</f>
-        <v>105314</v>
-      </c>
-      <c r="G27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,G$25)</f>
-        <v>0</v>
-      </c>
-      <c r="H27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,H$25)</f>
-        <v>0</v>
-      </c>
-      <c r="I27" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A27,ventas_producto,I$25)</f>
-        <v>107946</v>
-      </c>
-      <c r="J27" s="18">
-        <f t="shared" ref="J27:J30" si="61">SUM(E27:I27)</f>
-        <v>213260</v>
-      </c>
-      <c r="L27" s="97">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
-      <c r="M27" s="59">
+      <c r="F27" s="18">
         <f t="shared" si="56"/>
-        <v>576702901</v>
-      </c>
-      <c r="N27" s="59">
+        <v>105314</v>
+      </c>
+      <c r="G27" s="18">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
-      <c r="O27" s="59">
+      <c r="H27" s="18">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
+      <c r="I27" s="18">
+        <f t="shared" si="56"/>
+        <v>107946</v>
+      </c>
+      <c r="J27" s="18">
+        <f t="shared" ref="J27:J30" si="62">SUM(E27:I27)</f>
+        <v>213260</v>
+      </c>
+      <c r="L27" s="97">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
+      <c r="M27" s="59">
+        <f t="shared" si="57"/>
+        <v>576702901</v>
+      </c>
+      <c r="N27" s="59">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
+      <c r="O27" s="59">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
       <c r="P27" s="59">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>101435</v>
       </c>
       <c r="Q27" s="59">
-        <f t="shared" ref="Q27:Q30" si="62">SUM(L27:P27)</f>
+        <f t="shared" ref="Q27:Q30" si="63">SUM(L27:P27)</f>
         <v>576804336</v>
       </c>
       <c r="S27" s="90">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>7195</v>
       </c>
       <c r="T27" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>51553</v>
       </c>
       <c r="U27" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>9023</v>
       </c>
       <c r="V27" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>103585</v>
       </c>
       <c r="W27" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>25399</v>
       </c>
       <c r="X27" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>16505</v>
       </c>
       <c r="Y27" s="30">
-        <f t="shared" ref="Y27:Y30" si="63">SUM(S27:X27)</f>
+        <f t="shared" ref="Y27:Y30" si="64">SUM(S27:X27)</f>
         <v>213260</v>
       </c>
       <c r="AA27" s="104">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>52631529</v>
       </c>
       <c r="AB27" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>271532147</v>
       </c>
       <c r="AC27" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>63246530</v>
       </c>
       <c r="AD27" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>44964557</v>
       </c>
       <c r="AE27" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>93622843</v>
       </c>
       <c r="AF27" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>50806730</v>
       </c>
       <c r="AG27" s="64">
-        <f t="shared" ref="AG27:AG30" si="64">SUM(AA27:AF27)</f>
+        <f t="shared" ref="AG27:AG30" si="65">SUM(AA27:AF27)</f>
         <v>576804336</v>
       </c>
       <c r="AI27" s="93"/>
@@ -9625,51 +9654,51 @@
       <c r="AT27" s="49"/>
       <c r="AU27" s="49"/>
       <c r="AW27" s="82">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>32696</v>
       </c>
       <c r="AX27" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>31651</v>
       </c>
       <c r="AY27" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>40967</v>
       </c>
       <c r="AZ27" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>107946</v>
       </c>
       <c r="BA27" s="46">
-        <f t="shared" si="59"/>
-        <v>0</v>
-      </c>
-      <c r="BB27" s="46">
-        <f t="shared" ref="BB27:BB30" si="65">SUM(AW27:BA27)</f>
-        <v>213260</v>
-      </c>
-      <c r="BD27" s="97">
-        <f t="shared" si="60"/>
-        <v>160364763</v>
-      </c>
-      <c r="BE27" s="69">
-        <f t="shared" si="60"/>
-        <v>201880917</v>
-      </c>
-      <c r="BF27" s="69">
-        <f t="shared" si="60"/>
-        <v>214457221</v>
-      </c>
-      <c r="BG27" s="69">
-        <f t="shared" si="60"/>
-        <v>101435</v>
-      </c>
-      <c r="BH27" s="69">
         <f t="shared" si="60"/>
         <v>0</v>
       </c>
+      <c r="BB27" s="46">
+        <f t="shared" ref="BB27:BB30" si="66">SUM(AW27:BA27)</f>
+        <v>213260</v>
+      </c>
+      <c r="BD27" s="97">
+        <f t="shared" si="61"/>
+        <v>160364763</v>
+      </c>
+      <c r="BE27" s="69">
+        <f t="shared" si="61"/>
+        <v>201880917</v>
+      </c>
+      <c r="BF27" s="69">
+        <f t="shared" si="61"/>
+        <v>214457221</v>
+      </c>
+      <c r="BG27" s="69">
+        <f t="shared" si="61"/>
+        <v>101435</v>
+      </c>
+      <c r="BH27" s="69">
+        <f t="shared" si="61"/>
+        <v>0</v>
+      </c>
       <c r="BI27" s="69">
-        <f t="shared" ref="BI27:BI30" si="66">SUM(BD27:BH27)</f>
+        <f t="shared" ref="BI27:BI30" si="67">SUM(BD27:BH27)</f>
         <v>576804336</v>
       </c>
     </row>
@@ -9686,107 +9715,107 @@
         <v>687706530</v>
       </c>
       <c r="E28" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,E$25)</f>
+        <f t="shared" si="56"/>
         <v>2738</v>
       </c>
       <c r="F28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,F$25)</f>
+        <f t="shared" si="56"/>
         <v>1928</v>
       </c>
       <c r="G28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,G$25)</f>
+        <f t="shared" si="56"/>
         <v>109437</v>
       </c>
       <c r="H28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,H$25)</f>
+        <f t="shared" si="56"/>
         <v>1927</v>
       </c>
       <c r="I28" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A28,ventas_producto,I$25)</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="19">
-        <f t="shared" si="61"/>
-        <v>116030</v>
-      </c>
-      <c r="L28" s="98">
-        <f t="shared" si="56"/>
-        <v>844832</v>
-      </c>
-      <c r="M28" s="60">
-        <f t="shared" si="56"/>
-        <v>108214</v>
-      </c>
-      <c r="N28" s="60">
-        <f t="shared" si="56"/>
-        <v>685829502</v>
-      </c>
-      <c r="O28" s="60">
-        <f t="shared" si="56"/>
-        <v>923982</v>
-      </c>
-      <c r="P28" s="60">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
+      <c r="J28" s="19">
+        <f t="shared" si="62"/>
+        <v>116030</v>
+      </c>
+      <c r="L28" s="98">
+        <f t="shared" si="57"/>
+        <v>844832</v>
+      </c>
+      <c r="M28" s="60">
+        <f t="shared" si="57"/>
+        <v>108214</v>
+      </c>
+      <c r="N28" s="60">
+        <f t="shared" si="57"/>
+        <v>685829502</v>
+      </c>
+      <c r="O28" s="60">
+        <f t="shared" si="57"/>
+        <v>923982</v>
+      </c>
+      <c r="P28" s="60">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
       <c r="Q28" s="60">
-        <f t="shared" si="62"/>
+        <f t="shared" si="63"/>
         <v>687706530</v>
       </c>
       <c r="S28" s="91">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>39170</v>
       </c>
       <c r="T28" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>19565</v>
       </c>
       <c r="U28" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>6969</v>
       </c>
       <c r="V28" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>9925</v>
       </c>
       <c r="W28" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>12633</v>
       </c>
       <c r="X28" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>27768</v>
       </c>
       <c r="Y28" s="31">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>116030</v>
       </c>
       <c r="AA28" s="105">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>240927099</v>
       </c>
       <c r="AB28" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>131950052</v>
       </c>
       <c r="AC28" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>40433106</v>
       </c>
       <c r="AD28" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>27153333</v>
       </c>
       <c r="AE28" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>78668644</v>
       </c>
       <c r="AF28" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>168574296</v>
       </c>
       <c r="AG28" s="65">
-        <f t="shared" si="64"/>
+        <f t="shared" si="65"/>
         <v>687706530</v>
       </c>
       <c r="AI28" s="93"/>
@@ -9802,51 +9831,51 @@
       <c r="AT28" s="49"/>
       <c r="AU28" s="49"/>
       <c r="AW28" s="83">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>39124</v>
       </c>
       <c r="AX28" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>34000</v>
       </c>
       <c r="AY28" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>31330</v>
       </c>
       <c r="AZ28" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>7721</v>
       </c>
       <c r="BA28" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>3855</v>
       </c>
       <c r="BB28" s="47">
-        <f t="shared" si="65"/>
+        <f t="shared" si="66"/>
         <v>116030</v>
       </c>
       <c r="BD28" s="98">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>220801841</v>
       </c>
       <c r="BE28" s="70">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>239992813</v>
       </c>
       <c r="BF28" s="70">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>216914467</v>
       </c>
       <c r="BG28" s="70">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>8965213</v>
       </c>
       <c r="BH28" s="70">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>1032196</v>
       </c>
       <c r="BI28" s="70">
-        <f t="shared" si="66"/>
+        <f t="shared" si="67"/>
         <v>687706530</v>
       </c>
     </row>
@@ -9863,107 +9892,107 @@
         <v>654677692</v>
       </c>
       <c r="E29" s="82">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,E$25)</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,F$25)</f>
-        <v>197277</v>
-      </c>
-      <c r="G29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,G$25)</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,H$25)</f>
-        <v>113588</v>
-      </c>
-      <c r="I29" s="18">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A29,ventas_producto,I$25)</f>
-        <v>1927</v>
-      </c>
-      <c r="J29" s="18">
-        <f t="shared" si="61"/>
-        <v>312792</v>
-      </c>
-      <c r="L29" s="97">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
-      <c r="M29" s="59">
+      <c r="F29" s="18">
         <f t="shared" si="56"/>
-        <v>1313277</v>
-      </c>
-      <c r="N29" s="59">
+        <v>197277</v>
+      </c>
+      <c r="G29" s="18">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
+      <c r="H29" s="18">
+        <f t="shared" si="56"/>
+        <v>113588</v>
+      </c>
+      <c r="I29" s="18">
+        <f t="shared" si="56"/>
+        <v>1927</v>
+      </c>
+      <c r="J29" s="18">
+        <f t="shared" si="62"/>
+        <v>312792</v>
+      </c>
+      <c r="L29" s="97">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
+      <c r="M29" s="59">
+        <f t="shared" si="57"/>
+        <v>1313277</v>
+      </c>
+      <c r="N29" s="59">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
       <c r="O29" s="59">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>652816023</v>
       </c>
       <c r="P29" s="59">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>548392</v>
       </c>
       <c r="Q29" s="59">
-        <f t="shared" si="62"/>
+        <f t="shared" si="63"/>
         <v>654677692</v>
       </c>
       <c r="S29" s="90">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>39255</v>
       </c>
       <c r="T29" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>12991</v>
       </c>
       <c r="U29" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>2096</v>
       </c>
       <c r="V29" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>197831</v>
       </c>
       <c r="W29" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>53237</v>
       </c>
       <c r="X29" s="30">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>7382</v>
       </c>
       <c r="Y29" s="30">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>312792</v>
       </c>
       <c r="AA29" s="104">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>170461858</v>
       </c>
       <c r="AB29" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>75839132</v>
       </c>
       <c r="AC29" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>31378227</v>
       </c>
       <c r="AD29" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>23830600</v>
       </c>
       <c r="AE29" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>336034466</v>
       </c>
       <c r="AF29" s="64">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>17133409</v>
       </c>
       <c r="AG29" s="64">
-        <f t="shared" si="64"/>
+        <f t="shared" si="65"/>
         <v>654677692</v>
       </c>
       <c r="AI29" s="93"/>
@@ -9979,51 +10008,51 @@
       <c r="AT29" s="49"/>
       <c r="AU29" s="49"/>
       <c r="AW29" s="82">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>40573</v>
       </c>
       <c r="AX29" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>39442</v>
       </c>
       <c r="AY29" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>33573</v>
       </c>
       <c r="AZ29" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>4903</v>
       </c>
       <c r="BA29" s="46">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>194301</v>
       </c>
       <c r="BB29" s="46">
-        <f t="shared" si="65"/>
+        <f t="shared" si="66"/>
         <v>312792</v>
       </c>
       <c r="BD29" s="97">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>190929354</v>
       </c>
       <c r="BE29" s="69">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>221383553</v>
       </c>
       <c r="BF29" s="69">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>240503116</v>
       </c>
       <c r="BG29" s="69">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>483929</v>
       </c>
       <c r="BH29" s="69">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>1377740</v>
       </c>
       <c r="BI29" s="69">
-        <f t="shared" si="66"/>
+        <f t="shared" si="67"/>
         <v>654677692</v>
       </c>
     </row>
@@ -10040,107 +10069,107 @@
         <v>664722025</v>
       </c>
       <c r="E30" s="83">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,E$25)</f>
+        <f t="shared" si="56"/>
         <v>7128</v>
       </c>
       <c r="F30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,F$25)</f>
-        <v>0</v>
-      </c>
-      <c r="G30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,G$25)</f>
-        <v>0</v>
-      </c>
-      <c r="H30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,H$25)</f>
-        <v>0</v>
-      </c>
-      <c r="I30" s="19">
-        <f>SUMIFS(ventas_unidades,ventas_region,$A30,ventas_producto,I$25)</f>
-        <v>98908</v>
-      </c>
-      <c r="J30" s="19">
-        <f t="shared" si="61"/>
-        <v>106036</v>
-      </c>
-      <c r="L30" s="98">
-        <f t="shared" si="56"/>
-        <v>9123918</v>
-      </c>
-      <c r="M30" s="60">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
-      <c r="N30" s="60">
+      <c r="G30" s="19">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
-      <c r="O30" s="60">
+      <c r="H30" s="19">
         <f t="shared" si="56"/>
         <v>0</v>
       </c>
+      <c r="I30" s="19">
+        <f t="shared" si="56"/>
+        <v>98908</v>
+      </c>
+      <c r="J30" s="19">
+        <f t="shared" si="62"/>
+        <v>106036</v>
+      </c>
+      <c r="L30" s="98">
+        <f t="shared" si="57"/>
+        <v>9123918</v>
+      </c>
+      <c r="M30" s="60">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
+      <c r="N30" s="60">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
+      <c r="O30" s="60">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
       <c r="P30" s="60">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>655598107</v>
       </c>
       <c r="Q30" s="60">
-        <f t="shared" si="62"/>
+        <f t="shared" si="63"/>
         <v>664722025</v>
       </c>
       <c r="S30" s="91">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>12970</v>
       </c>
       <c r="T30" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>14165</v>
       </c>
       <c r="U30" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>5143</v>
       </c>
       <c r="V30" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>14291</v>
       </c>
       <c r="W30" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>19979</v>
       </c>
       <c r="X30" s="31">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>39488</v>
       </c>
       <c r="Y30" s="31">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>106036</v>
       </c>
       <c r="AA30" s="105">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>71950539</v>
       </c>
       <c r="AB30" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>88920515</v>
       </c>
       <c r="AC30" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>31867112</v>
       </c>
       <c r="AD30" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>76700859</v>
       </c>
       <c r="AE30" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>119641616</v>
       </c>
       <c r="AF30" s="65">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>275641384</v>
       </c>
       <c r="AG30" s="65">
-        <f t="shared" si="64"/>
+        <f t="shared" si="65"/>
         <v>664722025</v>
       </c>
       <c r="AI30" s="93"/>
@@ -10156,51 +10185,51 @@
       <c r="AT30" s="49"/>
       <c r="AU30" s="49"/>
       <c r="AW30" s="83">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>36557</v>
       </c>
       <c r="AX30" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>28900</v>
       </c>
       <c r="AY30" s="47">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>33451</v>
       </c>
       <c r="AZ30" s="47">
-        <f t="shared" si="59"/>
-        <v>0</v>
-      </c>
-      <c r="BA30" s="47">
-        <f t="shared" si="59"/>
-        <v>7128</v>
-      </c>
-      <c r="BB30" s="47">
-        <f t="shared" si="65"/>
-        <v>106036</v>
-      </c>
-      <c r="BD30" s="98">
-        <f t="shared" si="60"/>
-        <v>216479082</v>
-      </c>
-      <c r="BE30" s="70">
-        <f t="shared" si="60"/>
-        <v>240247726</v>
-      </c>
-      <c r="BF30" s="70">
-        <f t="shared" si="60"/>
-        <v>198871299</v>
-      </c>
-      <c r="BG30" s="70">
         <f t="shared" si="60"/>
         <v>0</v>
       </c>
+      <c r="BA30" s="47">
+        <f t="shared" si="60"/>
+        <v>7128</v>
+      </c>
+      <c r="BB30" s="47">
+        <f t="shared" si="66"/>
+        <v>106036</v>
+      </c>
+      <c r="BD30" s="98">
+        <f t="shared" si="61"/>
+        <v>216479082</v>
+      </c>
+      <c r="BE30" s="70">
+        <f t="shared" si="61"/>
+        <v>240247726</v>
+      </c>
+      <c r="BF30" s="70">
+        <f t="shared" si="61"/>
+        <v>198871299</v>
+      </c>
+      <c r="BG30" s="70">
+        <f t="shared" si="61"/>
+        <v>0</v>
+      </c>
       <c r="BH30" s="70">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>9123918</v>
       </c>
       <c r="BI30" s="70">
-        <f t="shared" si="66"/>
+        <f t="shared" si="67"/>
         <v>664722025</v>
       </c>
     </row>
@@ -10221,23 +10250,23 @@
         <v>110903</v>
       </c>
       <c r="F31" s="50">
-        <f t="shared" ref="F31:J31" si="67">SUM(F26:F30)</f>
+        <f t="shared" ref="F31:J31" si="68">SUM(F26:F30)</f>
         <v>304519</v>
       </c>
       <c r="G31" s="50">
-        <f t="shared" si="67"/>
+        <f t="shared" si="68"/>
         <v>118380</v>
       </c>
       <c r="H31" s="50">
-        <f t="shared" si="67"/>
+        <f t="shared" si="68"/>
         <v>115644</v>
       </c>
       <c r="I31" s="50">
-        <f t="shared" si="67"/>
+        <f t="shared" si="68"/>
         <v>208781</v>
       </c>
       <c r="J31" s="117">
-        <f t="shared" si="67"/>
+        <f t="shared" si="68"/>
         <v>858227</v>
       </c>
       <c r="L31" s="108">
@@ -10245,23 +10274,23 @@
         <v>650543568</v>
       </c>
       <c r="M31" s="68">
-        <f t="shared" ref="M31" si="68">SUM(M26:M30)</f>
+        <f t="shared" ref="M31" si="69">SUM(M26:M30)</f>
         <v>578124392</v>
       </c>
       <c r="N31" s="68">
-        <f t="shared" ref="N31" si="69">SUM(N26:N30)</f>
+        <f t="shared" ref="N31" si="70">SUM(N26:N30)</f>
         <v>690157736</v>
       </c>
       <c r="O31" s="68">
-        <f t="shared" ref="O31" si="70">SUM(O26:O30)</f>
+        <f t="shared" ref="O31" si="71">SUM(O26:O30)</f>
         <v>654943915</v>
       </c>
       <c r="P31" s="68">
-        <f t="shared" ref="P31" si="71">SUM(P26:P30)</f>
+        <f t="shared" ref="P31" si="72">SUM(P26:P30)</f>
         <v>656247934</v>
       </c>
       <c r="Q31" s="114">
-        <f t="shared" ref="Q31" si="72">SUM(Q26:Q30)</f>
+        <f t="shared" ref="Q31" si="73">SUM(Q26:Q30)</f>
         <v>3230017545</v>
       </c>
       <c r="S31" s="92">
@@ -10269,27 +10298,27 @@
         <v>121665</v>
       </c>
       <c r="T31" s="40">
-        <f t="shared" ref="T31:Y31" si="73">SUM(T26:T30)</f>
+        <f t="shared" ref="T31:Y31" si="74">SUM(T26:T30)</f>
         <v>125620</v>
       </c>
       <c r="U31" s="40">
-        <f t="shared" si="73"/>
+        <f t="shared" si="74"/>
         <v>32356</v>
       </c>
       <c r="V31" s="40">
-        <f t="shared" si="73"/>
+        <f t="shared" si="74"/>
         <v>356297</v>
       </c>
       <c r="W31" s="40">
-        <f t="shared" si="73"/>
+        <f t="shared" si="74"/>
         <v>122295</v>
       </c>
       <c r="X31" s="40">
-        <f t="shared" si="73"/>
+        <f t="shared" si="74"/>
         <v>99994</v>
       </c>
       <c r="Y31" s="40">
-        <f t="shared" si="73"/>
+        <f t="shared" si="74"/>
         <v>858227</v>
       </c>
       <c r="AA31" s="106">
@@ -10297,27 +10326,27 @@
         <v>645115066</v>
       </c>
       <c r="AB31" s="66">
-        <f t="shared" ref="AB31" si="74">SUM(AB26:AB30)</f>
+        <f t="shared" ref="AB31" si="75">SUM(AB26:AB30)</f>
         <v>761464717</v>
       </c>
       <c r="AC31" s="66">
-        <f t="shared" ref="AC31" si="75">SUM(AC26:AC30)</f>
+        <f t="shared" ref="AC31" si="76">SUM(AC26:AC30)</f>
         <v>226722785</v>
       </c>
       <c r="AD31" s="66">
-        <f t="shared" ref="AD31" si="76">SUM(AD26:AD30)</f>
+        <f t="shared" ref="AD31" si="77">SUM(AD26:AD30)</f>
         <v>312257691</v>
       </c>
       <c r="AE31" s="66">
-        <f t="shared" ref="AE31" si="77">SUM(AE26:AE30)</f>
+        <f t="shared" ref="AE31" si="78">SUM(AE26:AE30)</f>
         <v>722503562</v>
       </c>
       <c r="AF31" s="66">
-        <f t="shared" ref="AF31" si="78">SUM(AF26:AF30)</f>
+        <f t="shared" ref="AF31" si="79">SUM(AF26:AF30)</f>
         <v>561953724</v>
       </c>
       <c r="AG31" s="114">
-        <f t="shared" ref="AG31" si="79">SUM(AG26:AG30)</f>
+        <f t="shared" ref="AG31" si="80">SUM(AG26:AG30)</f>
         <v>3230017545</v>
       </c>
       <c r="AI31" s="93"/>
@@ -10333,23 +10362,23 @@
       <c r="AT31" s="49"/>
       <c r="AU31" s="49"/>
       <c r="AW31" s="94">
-        <f t="shared" ref="AW31:BA31" si="80">SUM(AW27:AW30)</f>
+        <f t="shared" ref="AW31:BA31" si="81">SUM(AW27:AW30)</f>
         <v>148950</v>
       </c>
       <c r="AX31" s="50">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>133993</v>
       </c>
       <c r="AY31" s="50">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>139321</v>
       </c>
       <c r="AZ31" s="50">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>120570</v>
       </c>
       <c r="BA31" s="50">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>205284</v>
       </c>
       <c r="BB31" s="117">
@@ -10361,23 +10390,23 @@
         <v>1007244151</v>
       </c>
       <c r="BE31" s="68">
-        <f t="shared" ref="BE31:BI31" si="81">SUM(BE26:BE30)</f>
+        <f t="shared" ref="BE31:BI31" si="82">SUM(BE26:BE30)</f>
         <v>1106846472</v>
       </c>
       <c r="BF31" s="68">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>1089310347</v>
       </c>
       <c r="BG31" s="68">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>15082721</v>
       </c>
       <c r="BH31" s="68">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>11533854</v>
       </c>
       <c r="BI31" s="114">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>3230017545</v>
       </c>
     </row>
@@ -10532,23 +10561,23 @@
         <v>1007244151</v>
       </c>
       <c r="E34" s="81">
-        <f t="shared" ref="E34:I38" si="82">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,E$25)</f>
+        <f t="shared" ref="E34:I38" si="83">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_producto,E$25)</f>
         <v>33032</v>
       </c>
       <c r="F34" s="17">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>32696</v>
       </c>
       <c r="G34" s="17">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>39124</v>
       </c>
       <c r="H34" s="17">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>40573</v>
       </c>
       <c r="I34" s="17">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>36557</v>
       </c>
       <c r="J34" s="17">
@@ -10556,23 +10585,23 @@
         <v>181982</v>
       </c>
       <c r="L34" s="96">
-        <f t="shared" ref="L34:P38" si="83">SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,L$25)</f>
+        <f t="shared" ref="L34:P38" si="84">SUMIFS(ventas_total,ventas_año,$A34,ventas_producto,L$25)</f>
         <v>218669111</v>
       </c>
       <c r="M34" s="58">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>160364763</v>
       </c>
       <c r="N34" s="58">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>220801841</v>
       </c>
       <c r="O34" s="58">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>190929354</v>
       </c>
       <c r="P34" s="58">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>216479082</v>
       </c>
       <c r="Q34" s="58">
@@ -10580,27 +10609,27 @@
         <v>1007244151</v>
       </c>
       <c r="S34" s="89">
-        <f t="shared" ref="S34:X38" si="84">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,S$33)</f>
+        <f t="shared" ref="S34:X38" si="85">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,S$33)</f>
         <v>33623</v>
       </c>
       <c r="T34" s="29">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>45235</v>
       </c>
       <c r="U34" s="29">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>12423</v>
       </c>
       <c r="V34" s="29">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>20990</v>
       </c>
       <c r="W34" s="29">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>44558</v>
       </c>
       <c r="X34" s="29">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>25153</v>
       </c>
       <c r="Y34" s="29">
@@ -10608,27 +10637,27 @@
         <v>181982</v>
       </c>
       <c r="AA34" s="103">
-        <f t="shared" ref="AA34:AF38" si="85">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,AA$33)</f>
+        <f t="shared" ref="AA34:AF38" si="86">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_vendedor,AA$33)</f>
         <v>33623</v>
       </c>
       <c r="AB34" s="63">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>45235</v>
       </c>
       <c r="AC34" s="63">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>12423</v>
       </c>
       <c r="AD34" s="63">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>20990</v>
       </c>
       <c r="AE34" s="63">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>44558</v>
       </c>
       <c r="AF34" s="63">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>25153</v>
       </c>
       <c r="AG34" s="63">
@@ -10636,23 +10665,23 @@
         <v>181982</v>
       </c>
       <c r="AI34" s="81">
-        <f t="shared" ref="AI34:AM38" si="86">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_region,AI$33)</f>
+        <f t="shared" ref="AI34:AM38" si="87">SUMIFS(ventas_unidades,ventas_año,$A34,ventas_region,AI$33)</f>
         <v>33032</v>
       </c>
       <c r="AJ34" s="17">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>32696</v>
       </c>
       <c r="AK34" s="17">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>39124</v>
       </c>
       <c r="AL34" s="17">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>40573</v>
       </c>
       <c r="AM34" s="17">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>36557</v>
       </c>
       <c r="AN34" s="17">
@@ -10660,23 +10689,23 @@
         <v>181982</v>
       </c>
       <c r="AP34" s="110">
-        <f t="shared" ref="AP34:AT38" si="87">SUMIFS(ventas_total,ventas_año,$A34,ventas_region,AP$33)</f>
+        <f t="shared" ref="AP34:AT38" si="88">SUMIFS(ventas_total,ventas_año,$A34,ventas_region,AP$33)</f>
         <v>218669111</v>
       </c>
       <c r="AQ34" s="41">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>160364763</v>
       </c>
       <c r="AR34" s="41">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>220801841</v>
       </c>
       <c r="AS34" s="41">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>190929354</v>
       </c>
       <c r="AT34" s="41">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>216479082</v>
       </c>
       <c r="AU34" s="41">
@@ -10709,155 +10738,155 @@
         <v>1106846472</v>
       </c>
       <c r="E35" s="82">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>32671</v>
       </c>
       <c r="F35" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>31651</v>
       </c>
       <c r="G35" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>34000</v>
       </c>
       <c r="H35" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>39442</v>
       </c>
       <c r="I35" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>28900</v>
       </c>
       <c r="J35" s="18">
-        <f t="shared" ref="J35:J38" si="88">SUM(E35:I35)</f>
+        <f t="shared" ref="J35:J38" si="89">SUM(E35:I35)</f>
         <v>166664</v>
       </c>
       <c r="L35" s="97">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>203341463</v>
       </c>
       <c r="M35" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>201880917</v>
       </c>
       <c r="N35" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>239992813</v>
       </c>
       <c r="O35" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>221383553</v>
       </c>
       <c r="P35" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>240247726</v>
       </c>
       <c r="Q35" s="59">
-        <f t="shared" ref="Q35:Q38" si="89">SUM(L35:P35)</f>
+        <f t="shared" ref="Q35:Q38" si="90">SUM(L35:P35)</f>
         <v>1106846472</v>
       </c>
       <c r="S35" s="90">
-        <f t="shared" si="84"/>
-        <v>42339</v>
-      </c>
-      <c r="T35" s="30">
-        <f t="shared" si="84"/>
-        <v>39435</v>
-      </c>
-      <c r="U35" s="30">
-        <f t="shared" si="84"/>
-        <v>12194</v>
-      </c>
-      <c r="V35" s="30">
-        <f t="shared" si="84"/>
-        <v>11750</v>
-      </c>
-      <c r="W35" s="30">
-        <f t="shared" si="84"/>
-        <v>27319</v>
-      </c>
-      <c r="X35" s="30">
-        <f t="shared" si="84"/>
-        <v>33627</v>
-      </c>
-      <c r="Y35" s="30">
-        <f t="shared" ref="Y35:Y38" si="90">SUM(S35:X35)</f>
-        <v>166664</v>
-      </c>
-      <c r="AA35" s="104">
         <f t="shared" si="85"/>
         <v>42339</v>
       </c>
-      <c r="AB35" s="64">
+      <c r="T35" s="30">
         <f t="shared" si="85"/>
         <v>39435</v>
       </c>
-      <c r="AC35" s="64">
+      <c r="U35" s="30">
         <f t="shared" si="85"/>
         <v>12194</v>
       </c>
-      <c r="AD35" s="64">
+      <c r="V35" s="30">
         <f t="shared" si="85"/>
         <v>11750</v>
       </c>
-      <c r="AE35" s="64">
+      <c r="W35" s="30">
         <f t="shared" si="85"/>
         <v>27319</v>
       </c>
-      <c r="AF35" s="64">
+      <c r="X35" s="30">
         <f t="shared" si="85"/>
         <v>33627</v>
       </c>
+      <c r="Y35" s="30">
+        <f t="shared" ref="Y35:Y38" si="91">SUM(S35:X35)</f>
+        <v>166664</v>
+      </c>
+      <c r="AA35" s="104">
+        <f t="shared" si="86"/>
+        <v>42339</v>
+      </c>
+      <c r="AB35" s="64">
+        <f t="shared" si="86"/>
+        <v>39435</v>
+      </c>
+      <c r="AC35" s="64">
+        <f t="shared" si="86"/>
+        <v>12194</v>
+      </c>
+      <c r="AD35" s="64">
+        <f t="shared" si="86"/>
+        <v>11750</v>
+      </c>
+      <c r="AE35" s="64">
+        <f t="shared" si="86"/>
+        <v>27319</v>
+      </c>
+      <c r="AF35" s="64">
+        <f t="shared" si="86"/>
+        <v>33627</v>
+      </c>
       <c r="AG35" s="64">
-        <f t="shared" ref="AG35:AG38" si="91">SUM(AA35:AF35)</f>
+        <f t="shared" ref="AG35:AG38" si="92">SUM(AA35:AF35)</f>
         <v>166664</v>
       </c>
       <c r="AI35" s="82">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>32671</v>
       </c>
       <c r="AJ35" s="18">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>31651</v>
       </c>
       <c r="AK35" s="18">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>34000</v>
       </c>
       <c r="AL35" s="18">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>39442</v>
       </c>
       <c r="AM35" s="18">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>28900</v>
       </c>
       <c r="AN35" s="18">
-        <f t="shared" ref="AN35:AN38" si="92">SUM(AI35:AM35)</f>
+        <f t="shared" ref="AN35:AN38" si="93">SUM(AI35:AM35)</f>
         <v>166664</v>
       </c>
       <c r="AP35" s="111">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>203341463</v>
       </c>
       <c r="AQ35" s="44">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>201880917</v>
       </c>
       <c r="AR35" s="44">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>239992813</v>
       </c>
       <c r="AS35" s="44">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>221383553</v>
       </c>
       <c r="AT35" s="44">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>240247726</v>
       </c>
       <c r="AU35" s="44">
-        <f t="shared" ref="AU35:AU38" si="93">SUM(AP35:AT35)</f>
+        <f t="shared" ref="AU35:AU38" si="94">SUM(AP35:AT35)</f>
         <v>1106846472</v>
       </c>
       <c r="AW35" s="93"/>
@@ -10886,155 +10915,155 @@
         <v>1089310347</v>
       </c>
       <c r="E36" s="83">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>35334</v>
       </c>
       <c r="F36" s="19">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>40967</v>
       </c>
       <c r="G36" s="19">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>31330</v>
       </c>
       <c r="H36" s="19">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>33573</v>
       </c>
       <c r="I36" s="19">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>33451</v>
       </c>
       <c r="J36" s="19">
-        <f t="shared" si="88"/>
+        <f t="shared" si="89"/>
         <v>174655</v>
       </c>
       <c r="L36" s="98">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>218564244</v>
       </c>
       <c r="M36" s="60">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>214457221</v>
       </c>
       <c r="N36" s="60">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>216914467</v>
       </c>
       <c r="O36" s="60">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>240503116</v>
       </c>
       <c r="P36" s="60">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>198871299</v>
       </c>
       <c r="Q36" s="60">
-        <f t="shared" si="89"/>
+        <f t="shared" si="90"/>
         <v>1089310347</v>
       </c>
       <c r="S36" s="91">
-        <f t="shared" si="84"/>
-        <v>33889</v>
-      </c>
-      <c r="T36" s="31">
-        <f t="shared" si="84"/>
-        <v>40950</v>
-      </c>
-      <c r="U36" s="31">
-        <f t="shared" si="84"/>
-        <v>7739</v>
-      </c>
-      <c r="V36" s="31">
-        <f t="shared" si="84"/>
-        <v>24117</v>
-      </c>
-      <c r="W36" s="31">
-        <f t="shared" si="84"/>
-        <v>31540</v>
-      </c>
-      <c r="X36" s="31">
-        <f t="shared" si="84"/>
-        <v>36420</v>
-      </c>
-      <c r="Y36" s="31">
-        <f t="shared" si="90"/>
-        <v>174655</v>
-      </c>
-      <c r="AA36" s="105">
         <f t="shared" si="85"/>
         <v>33889</v>
       </c>
-      <c r="AB36" s="65">
+      <c r="T36" s="31">
         <f t="shared" si="85"/>
         <v>40950</v>
       </c>
-      <c r="AC36" s="65">
+      <c r="U36" s="31">
         <f t="shared" si="85"/>
         <v>7739</v>
       </c>
-      <c r="AD36" s="65">
+      <c r="V36" s="31">
         <f t="shared" si="85"/>
         <v>24117</v>
       </c>
-      <c r="AE36" s="65">
+      <c r="W36" s="31">
         <f t="shared" si="85"/>
         <v>31540</v>
       </c>
-      <c r="AF36" s="65">
+      <c r="X36" s="31">
         <f t="shared" si="85"/>
         <v>36420</v>
       </c>
-      <c r="AG36" s="65">
+      <c r="Y36" s="31">
         <f t="shared" si="91"/>
         <v>174655</v>
       </c>
-      <c r="AI36" s="83">
+      <c r="AA36" s="105">
         <f t="shared" si="86"/>
-        <v>35334</v>
-      </c>
-      <c r="AJ36" s="19">
+        <v>33889</v>
+      </c>
+      <c r="AB36" s="65">
         <f t="shared" si="86"/>
-        <v>40967</v>
-      </c>
-      <c r="AK36" s="19">
+        <v>40950</v>
+      </c>
+      <c r="AC36" s="65">
         <f t="shared" si="86"/>
-        <v>31330</v>
-      </c>
-      <c r="AL36" s="19">
+        <v>7739</v>
+      </c>
+      <c r="AD36" s="65">
         <f t="shared" si="86"/>
-        <v>33573</v>
-      </c>
-      <c r="AM36" s="19">
+        <v>24117</v>
+      </c>
+      <c r="AE36" s="65">
         <f t="shared" si="86"/>
-        <v>33451</v>
-      </c>
-      <c r="AN36" s="19">
+        <v>31540</v>
+      </c>
+      <c r="AF36" s="65">
+        <f t="shared" si="86"/>
+        <v>36420</v>
+      </c>
+      <c r="AG36" s="65">
         <f t="shared" si="92"/>
         <v>174655</v>
       </c>
+      <c r="AI36" s="83">
+        <f t="shared" si="87"/>
+        <v>35334</v>
+      </c>
+      <c r="AJ36" s="19">
+        <f t="shared" si="87"/>
+        <v>40967</v>
+      </c>
+      <c r="AK36" s="19">
+        <f t="shared" si="87"/>
+        <v>31330</v>
+      </c>
+      <c r="AL36" s="19">
+        <f t="shared" si="87"/>
+        <v>33573</v>
+      </c>
+      <c r="AM36" s="19">
+        <f t="shared" si="87"/>
+        <v>33451</v>
+      </c>
+      <c r="AN36" s="19">
+        <f t="shared" si="93"/>
+        <v>174655</v>
+      </c>
       <c r="AP36" s="112">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>218564244</v>
       </c>
       <c r="AQ36" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>214457221</v>
       </c>
       <c r="AR36" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>216914467</v>
       </c>
       <c r="AS36" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>240503116</v>
       </c>
       <c r="AT36" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>198871299</v>
       </c>
       <c r="AU36" s="45">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>1089310347</v>
       </c>
       <c r="AW36" s="93"/>
@@ -11063,155 +11092,155 @@
         <v>15082721</v>
       </c>
       <c r="E37" s="82">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>2738</v>
       </c>
       <c r="F37" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>4903</v>
       </c>
       <c r="G37" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>13926</v>
       </c>
       <c r="H37" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>129</v>
       </c>
       <c r="I37" s="18">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>107946</v>
       </c>
       <c r="J37" s="18">
-        <f t="shared" si="88"/>
+        <f t="shared" si="89"/>
         <v>129642</v>
       </c>
       <c r="L37" s="97">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>844832</v>
       </c>
       <c r="M37" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>483929</v>
       </c>
       <c r="N37" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>12448615</v>
       </c>
       <c r="O37" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>1203910</v>
       </c>
       <c r="P37" s="59">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>101435</v>
       </c>
       <c r="Q37" s="59">
-        <f t="shared" si="89"/>
+        <f t="shared" si="90"/>
         <v>15082721</v>
       </c>
       <c r="S37" s="90">
-        <f t="shared" si="84"/>
-        <v>9886</v>
-      </c>
-      <c r="T37" s="30">
-        <f t="shared" si="84"/>
-        <v>0</v>
-      </c>
-      <c r="U37" s="30">
-        <f t="shared" si="84"/>
-        <v>0</v>
-      </c>
-      <c r="V37" s="30">
-        <f t="shared" si="84"/>
-        <v>107066</v>
-      </c>
-      <c r="W37" s="30">
-        <f t="shared" si="84"/>
-        <v>9823</v>
-      </c>
-      <c r="X37" s="30">
-        <f t="shared" si="84"/>
-        <v>2867</v>
-      </c>
-      <c r="Y37" s="30">
-        <f t="shared" si="90"/>
-        <v>129642</v>
-      </c>
-      <c r="AA37" s="104">
         <f t="shared" si="85"/>
         <v>9886</v>
       </c>
-      <c r="AB37" s="64">
+      <c r="T37" s="30">
         <f t="shared" si="85"/>
         <v>0</v>
       </c>
-      <c r="AC37" s="64">
+      <c r="U37" s="30">
         <f t="shared" si="85"/>
         <v>0</v>
       </c>
-      <c r="AD37" s="64">
+      <c r="V37" s="30">
         <f t="shared" si="85"/>
         <v>107066</v>
       </c>
-      <c r="AE37" s="64">
+      <c r="W37" s="30">
         <f t="shared" si="85"/>
         <v>9823</v>
       </c>
-      <c r="AF37" s="64">
+      <c r="X37" s="30">
         <f t="shared" si="85"/>
         <v>2867</v>
       </c>
-      <c r="AG37" s="64">
+      <c r="Y37" s="30">
         <f t="shared" si="91"/>
         <v>129642</v>
       </c>
-      <c r="AI37" s="82">
+      <c r="AA37" s="104">
         <f t="shared" si="86"/>
-        <v>9072</v>
-      </c>
-      <c r="AJ37" s="18">
-        <f t="shared" si="86"/>
-        <v>107946</v>
-      </c>
-      <c r="AK37" s="18">
-        <f t="shared" si="86"/>
-        <v>7721</v>
-      </c>
-      <c r="AL37" s="18">
-        <f t="shared" si="86"/>
-        <v>4903</v>
-      </c>
-      <c r="AM37" s="18">
+        <v>9886</v>
+      </c>
+      <c r="AB37" s="64">
         <f t="shared" si="86"/>
         <v>0</v>
       </c>
-      <c r="AN37" s="18">
+      <c r="AC37" s="64">
+        <f t="shared" si="86"/>
+        <v>0</v>
+      </c>
+      <c r="AD37" s="64">
+        <f t="shared" si="86"/>
+        <v>107066</v>
+      </c>
+      <c r="AE37" s="64">
+        <f t="shared" si="86"/>
+        <v>9823</v>
+      </c>
+      <c r="AF37" s="64">
+        <f t="shared" si="86"/>
+        <v>2867</v>
+      </c>
+      <c r="AG37" s="64">
         <f t="shared" si="92"/>
         <v>129642</v>
       </c>
-      <c r="AP37" s="111">
+      <c r="AI37" s="82">
         <f t="shared" si="87"/>
-        <v>5532144</v>
-      </c>
-      <c r="AQ37" s="44">
+        <v>9072</v>
+      </c>
+      <c r="AJ37" s="18">
         <f t="shared" si="87"/>
-        <v>101435</v>
-      </c>
-      <c r="AR37" s="44">
+        <v>107946</v>
+      </c>
+      <c r="AK37" s="18">
         <f t="shared" si="87"/>
-        <v>8965213</v>
-      </c>
-      <c r="AS37" s="44">
+        <v>7721</v>
+      </c>
+      <c r="AL37" s="18">
         <f t="shared" si="87"/>
-        <v>483929</v>
-      </c>
-      <c r="AT37" s="44">
+        <v>4903</v>
+      </c>
+      <c r="AM37" s="18">
         <f t="shared" si="87"/>
         <v>0</v>
       </c>
+      <c r="AN37" s="18">
+        <f t="shared" si="93"/>
+        <v>129642</v>
+      </c>
+      <c r="AP37" s="111">
+        <f t="shared" si="88"/>
+        <v>5532144</v>
+      </c>
+      <c r="AQ37" s="44">
+        <f t="shared" si="88"/>
+        <v>101435</v>
+      </c>
+      <c r="AR37" s="44">
+        <f t="shared" si="88"/>
+        <v>8965213</v>
+      </c>
+      <c r="AS37" s="44">
+        <f t="shared" si="88"/>
+        <v>483929</v>
+      </c>
+      <c r="AT37" s="44">
+        <f t="shared" si="88"/>
+        <v>0</v>
+      </c>
       <c r="AU37" s="44">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>15082721</v>
       </c>
       <c r="AW37" s="93"/>
@@ -11240,155 +11269,155 @@
         <v>11533854</v>
       </c>
       <c r="E38" s="83">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>7128</v>
       </c>
       <c r="F38" s="19">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>194302</v>
       </c>
       <c r="G38" s="19">
-        <f t="shared" si="82"/>
-        <v>0</v>
-      </c>
-      <c r="H38" s="19">
-        <f t="shared" si="82"/>
-        <v>1927</v>
-      </c>
-      <c r="I38" s="19">
-        <f t="shared" si="82"/>
-        <v>1927</v>
-      </c>
-      <c r="J38" s="19">
-        <f t="shared" si="88"/>
-        <v>205284</v>
-      </c>
-      <c r="L38" s="98">
-        <f t="shared" si="83"/>
-        <v>9123918</v>
-      </c>
-      <c r="M38" s="60">
-        <f t="shared" si="83"/>
-        <v>937562</v>
-      </c>
-      <c r="N38" s="60">
         <f t="shared" si="83"/>
         <v>0</v>
       </c>
-      <c r="O38" s="60">
+      <c r="H38" s="19">
         <f t="shared" si="83"/>
-        <v>923982</v>
-      </c>
-      <c r="P38" s="60">
+        <v>1927</v>
+      </c>
+      <c r="I38" s="19">
         <f t="shared" si="83"/>
-        <v>548392</v>
-      </c>
-      <c r="Q38" s="60">
+        <v>1927</v>
+      </c>
+      <c r="J38" s="19">
         <f t="shared" si="89"/>
-        <v>11533854</v>
-      </c>
-      <c r="S38" s="91">
+        <v>205284</v>
+      </c>
+      <c r="L38" s="98">
         <f t="shared" si="84"/>
-        <v>1928</v>
-      </c>
-      <c r="T38" s="31">
+        <v>9123918</v>
+      </c>
+      <c r="M38" s="60">
+        <f t="shared" si="84"/>
+        <v>937562</v>
+      </c>
+      <c r="N38" s="60">
         <f t="shared" si="84"/>
         <v>0</v>
       </c>
-      <c r="U38" s="31">
+      <c r="O38" s="60">
         <f t="shared" si="84"/>
-        <v>0</v>
-      </c>
-      <c r="V38" s="31">
+        <v>923982</v>
+      </c>
+      <c r="P38" s="60">
         <f t="shared" si="84"/>
-        <v>192374</v>
-      </c>
-      <c r="W38" s="31">
-        <f t="shared" si="84"/>
-        <v>9055</v>
-      </c>
-      <c r="X38" s="31">
-        <f t="shared" si="84"/>
-        <v>1927</v>
-      </c>
-      <c r="Y38" s="31">
+        <v>548392</v>
+      </c>
+      <c r="Q38" s="60">
         <f t="shared" si="90"/>
-        <v>205284</v>
-      </c>
-      <c r="AA38" s="105">
+        <v>11533854</v>
+      </c>
+      <c r="S38" s="91">
         <f t="shared" si="85"/>
         <v>1928</v>
       </c>
-      <c r="AB38" s="65">
+      <c r="T38" s="31">
         <f t="shared" si="85"/>
         <v>0</v>
       </c>
-      <c r="AC38" s="65">
+      <c r="U38" s="31">
         <f t="shared" si="85"/>
         <v>0</v>
       </c>
-      <c r="AD38" s="65">
+      <c r="V38" s="31">
         <f t="shared" si="85"/>
         <v>192374</v>
       </c>
-      <c r="AE38" s="65">
+      <c r="W38" s="31">
         <f t="shared" si="85"/>
         <v>9055</v>
       </c>
-      <c r="AF38" s="65">
+      <c r="X38" s="31">
         <f t="shared" si="85"/>
         <v>1927</v>
       </c>
-      <c r="AG38" s="65">
+      <c r="Y38" s="31">
         <f t="shared" si="91"/>
         <v>205284</v>
       </c>
-      <c r="AI38" s="83">
+      <c r="AA38" s="105">
+        <f t="shared" si="86"/>
+        <v>1928</v>
+      </c>
+      <c r="AB38" s="65">
         <f t="shared" si="86"/>
         <v>0</v>
       </c>
-      <c r="AJ38" s="19">
+      <c r="AC38" s="65">
         <f t="shared" si="86"/>
         <v>0</v>
       </c>
-      <c r="AK38" s="19">
+      <c r="AD38" s="65">
         <f t="shared" si="86"/>
-        <v>3855</v>
-      </c>
-      <c r="AL38" s="19">
+        <v>192374</v>
+      </c>
+      <c r="AE38" s="65">
         <f t="shared" si="86"/>
-        <v>194301</v>
-      </c>
-      <c r="AM38" s="19">
+        <v>9055</v>
+      </c>
+      <c r="AF38" s="65">
         <f t="shared" si="86"/>
-        <v>7128</v>
-      </c>
-      <c r="AN38" s="19">
+        <v>1927</v>
+      </c>
+      <c r="AG38" s="65">
         <f t="shared" si="92"/>
         <v>205284</v>
       </c>
-      <c r="AP38" s="112">
+      <c r="AI38" s="83">
         <f t="shared" si="87"/>
         <v>0</v>
       </c>
-      <c r="AQ38" s="45">
+      <c r="AJ38" s="19">
         <f t="shared" si="87"/>
         <v>0</v>
       </c>
+      <c r="AK38" s="19">
+        <f t="shared" si="87"/>
+        <v>3855</v>
+      </c>
+      <c r="AL38" s="19">
+        <f t="shared" si="87"/>
+        <v>194301</v>
+      </c>
+      <c r="AM38" s="19">
+        <f t="shared" si="87"/>
+        <v>7128</v>
+      </c>
+      <c r="AN38" s="19">
+        <f t="shared" si="93"/>
+        <v>205284</v>
+      </c>
+      <c r="AP38" s="112">
+        <f t="shared" si="88"/>
+        <v>0</v>
+      </c>
+      <c r="AQ38" s="45">
+        <f t="shared" si="88"/>
+        <v>0</v>
+      </c>
       <c r="AR38" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>1032196</v>
       </c>
       <c r="AS38" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>1377740</v>
       </c>
       <c r="AT38" s="45">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>9123918</v>
       </c>
       <c r="AU38" s="45">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>11533854</v>
       </c>
       <c r="AW38" s="93"/>
@@ -11421,23 +11450,23 @@
         <v>110903</v>
       </c>
       <c r="F39" s="50">
-        <f t="shared" ref="F39" si="94">SUM(F34:F38)</f>
+        <f t="shared" ref="F39" si="95">SUM(F34:F38)</f>
         <v>304519</v>
       </c>
       <c r="G39" s="50">
-        <f t="shared" ref="G39" si="95">SUM(G34:G38)</f>
+        <f t="shared" ref="G39" si="96">SUM(G34:G38)</f>
         <v>118380</v>
       </c>
       <c r="H39" s="50">
-        <f t="shared" ref="H39" si="96">SUM(H34:H38)</f>
+        <f t="shared" ref="H39" si="97">SUM(H34:H38)</f>
         <v>115644</v>
       </c>
       <c r="I39" s="50">
-        <f t="shared" ref="I39" si="97">SUM(I34:I38)</f>
+        <f t="shared" ref="I39" si="98">SUM(I34:I38)</f>
         <v>208781</v>
       </c>
       <c r="J39" s="117">
-        <f t="shared" ref="J39" si="98">SUM(J34:J38)</f>
+        <f t="shared" ref="J39" si="99">SUM(J34:J38)</f>
         <v>858227</v>
       </c>
       <c r="L39" s="108">
@@ -11445,19 +11474,19 @@
         <v>650543568</v>
       </c>
       <c r="M39" s="68">
-        <f t="shared" ref="M39" si="99">SUM(M34:M38)</f>
+        <f t="shared" ref="M39" si="100">SUM(M34:M38)</f>
         <v>578124392</v>
       </c>
       <c r="N39" s="68">
-        <f t="shared" ref="N39" si="100">SUM(N34:N38)</f>
+        <f t="shared" ref="N39" si="101">SUM(N34:N38)</f>
         <v>690157736</v>
       </c>
       <c r="O39" s="68">
-        <f t="shared" ref="O39" si="101">SUM(O34:O38)</f>
+        <f t="shared" ref="O39" si="102">SUM(O34:O38)</f>
         <v>654943915</v>
       </c>
       <c r="P39" s="68">
-        <f t="shared" ref="P39" si="102">SUM(P34:P38)</f>
+        <f t="shared" ref="P39" si="103">SUM(P34:P38)</f>
         <v>656247934</v>
       </c>
       <c r="Q39" s="114">
@@ -11469,27 +11498,27 @@
         <v>121665</v>
       </c>
       <c r="T39" s="40">
-        <f t="shared" ref="T39:Y39" si="103">SUM(T34:T38)</f>
+        <f t="shared" ref="T39:Y39" si="104">SUM(T34:T38)</f>
         <v>125620</v>
       </c>
       <c r="U39" s="40">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>32356</v>
       </c>
       <c r="V39" s="40">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>356297</v>
       </c>
       <c r="W39" s="40">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>122295</v>
       </c>
       <c r="X39" s="40">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>99994</v>
       </c>
       <c r="Y39" s="40">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>858227</v>
       </c>
       <c r="AA39" s="106">
@@ -11497,27 +11526,27 @@
         <v>121665</v>
       </c>
       <c r="AB39" s="66">
-        <f t="shared" ref="AB39" si="104">SUM(AB34:AB38)</f>
+        <f t="shared" ref="AB39" si="105">SUM(AB34:AB38)</f>
         <v>125620</v>
       </c>
       <c r="AC39" s="66">
-        <f t="shared" ref="AC39" si="105">SUM(AC34:AC38)</f>
+        <f t="shared" ref="AC39" si="106">SUM(AC34:AC38)</f>
         <v>32356</v>
       </c>
       <c r="AD39" s="66">
-        <f t="shared" ref="AD39" si="106">SUM(AD34:AD38)</f>
+        <f t="shared" ref="AD39" si="107">SUM(AD34:AD38)</f>
         <v>356297</v>
       </c>
       <c r="AE39" s="66">
-        <f t="shared" ref="AE39" si="107">SUM(AE34:AE38)</f>
+        <f t="shared" ref="AE39" si="108">SUM(AE34:AE38)</f>
         <v>122295</v>
       </c>
       <c r="AF39" s="66">
-        <f t="shared" ref="AF39" si="108">SUM(AF34:AF38)</f>
+        <f t="shared" ref="AF39" si="109">SUM(AF34:AF38)</f>
         <v>99994</v>
       </c>
       <c r="AG39" s="114">
-        <f t="shared" ref="AG39" si="109">SUM(AG34:AG38)</f>
+        <f t="shared" ref="AG39" si="110">SUM(AG34:AG38)</f>
         <v>858227</v>
       </c>
       <c r="AI39" s="94">
@@ -11525,23 +11554,23 @@
         <v>110109</v>
       </c>
       <c r="AJ39" s="50">
-        <f t="shared" ref="AJ39:AN39" si="110">SUM(AJ34:AJ38)</f>
+        <f t="shared" ref="AJ39:AN39" si="111">SUM(AJ34:AJ38)</f>
         <v>213260</v>
       </c>
       <c r="AK39" s="50">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>116030</v>
       </c>
       <c r="AL39" s="50">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>312792</v>
       </c>
       <c r="AM39" s="50">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>106036</v>
       </c>
       <c r="AN39" s="117">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>858227</v>
       </c>
       <c r="AP39" s="113">
@@ -11549,23 +11578,23 @@
         <v>646106962</v>
       </c>
       <c r="AQ39" s="48">
-        <f t="shared" ref="AQ39" si="111">SUM(AQ34:AQ38)</f>
+        <f t="shared" ref="AQ39" si="112">SUM(AQ34:AQ38)</f>
         <v>576804336</v>
       </c>
       <c r="AR39" s="48">
-        <f t="shared" ref="AR39" si="112">SUM(AR34:AR38)</f>
+        <f t="shared" ref="AR39" si="113">SUM(AR34:AR38)</f>
         <v>687706530</v>
       </c>
       <c r="AS39" s="48">
-        <f t="shared" ref="AS39" si="113">SUM(AS34:AS38)</f>
+        <f t="shared" ref="AS39" si="114">SUM(AS34:AS38)</f>
         <v>654677692</v>
       </c>
       <c r="AT39" s="48">
-        <f t="shared" ref="AT39" si="114">SUM(AT34:AT38)</f>
+        <f t="shared" ref="AT39" si="115">SUM(AT34:AT38)</f>
         <v>664722025</v>
       </c>
       <c r="AU39" s="118">
-        <f t="shared" ref="AU39" si="115">SUM(AU34:AU38)</f>
+        <f t="shared" ref="AU39" si="116">SUM(AU34:AU38)</f>
         <v>3230017545</v>
       </c>
       <c r="AW39" s="93"/>
@@ -11584,4 +11613,124 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DAD1870-E097-4F50-A371-71EFC7F222CC}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="2" customWidth="1"/>
+    <col min="5" max="5" width="16.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="135" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="3">
+        <v>100000</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="51">
+        <f>IFERROR(VLOOKUP($E$1,vendedores,MATCH($D2,estadisticas!$A$16:$C$16,0),FALSE),"seleccione un vendedor")</f>
+        <v>99994</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="3">
+        <v>500000000</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="137">
+        <f>IFERROR(VLOOKUP($E$1,vendedores,MATCH($D3,estadisticas!$A$16:$C$16,0),FALSE),"seleccione un vendedor")</f>
+        <v>561953724</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4">
+        <f>IF(AND(E2&gt;=B2,E3&gt;=B3),2,IF(OR(E2&gt;=B2,E3&gt;=B3),1,0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="1">
+        <f>E3*VLOOKUP(E4,A5:B8,2,FALSE)</f>
+        <v>84293058.599999994</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0</v>
+      </c>
+      <c r="B6" s="136">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" s="136">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" s="136">
+        <v>0.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Vendedor No encontrado" error="Ingrese un nombre de vendedor que se encuentre registrado" xr:uid="{0AD58637-BCDD-4A9E-8D99-B372B763A97D}">
+          <x14:formula1>
+            <xm:f>listas!$B$2:$B$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>E1</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>